<commit_message>
Update berita 2026-08-07 06:08 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-07.xlsx
+++ b/data/berita_2026-08-07.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$370</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$462</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I370"/>
+  <dimension ref="A1:I462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -17823,8 +17823,4332 @@
         </is>
       </c>
     </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>PPAL aktif berikan rekomendasi untuk kepentingan TNI AL</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 13:03:57 +0700</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Ketua Umum Persatuan Purnawirawan Angkatan Laut (PPAL) Laksamana TNI (Purn) Yudo Margono mengatakan jajarannya selalu ...</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683853/ppal-aktif-berikan-rekomendasi-untuk-kepentingan-tni-al</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001562012.jpg</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Bandara Soetta layani 25,9 juta penumpang pada semester I 2026</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:59:44 +0700</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>PT Angkasa Pura Indonesia (Persero) atau InJourneyAirports melalui Kantor Cabang Bandara Soekarno-Hatta (Soetta), ...</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683849/bandara-soetta-layani-259-juta-penumpang-pada-semester-i-2026</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000290609.jpg</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Tumpukan sampah di Kedaung Kaliangke Jakbar kembali dikeluhkan warga</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:59:35 +0700</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Warga kembalimengeluhkan sampah yang menumpuk di kawasan RT 04/RW 03, Kelurahan Kedaung Kaliangke, Kecamatan ...</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683848/tumpukan-sampah-di-kedaung-kaliangke-jakbar-kembali-dikeluhkan-warga</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Sampah-Kedaung-Kaliangke-Jakbar.jpg</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Pembalap melakukan sesi latihan ARRC 2026 di Sirkuit Mandalika</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:58:22 +0700</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Pembalap JDT Racing Team Joshua Waters memacu motornya saat sesi free practice 1 balapan Asia Road Racing Championship ...</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5683844/pembalap-melakukan-sesi-latihan-arrc-2026-di-sirkuit-mandalika</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Arrc-2026-di-mandalika-070826-AS-7.jpg</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Ilmuwan AS ciptakan bakteriofag AI untuk pertama kali</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:58:08 +0700</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Sejumlah ilmuwan Amerika Serikat, untuk pertama kalinya, berhasil menggunakan model kecerdasan buatan (AI) untuk ...</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683840/ilmuwan-as-ciptakan-bakteriofag-ai-untuk-pertama-kali</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/12/16/Illustration_Gen-AI-by-Freepik.jpg</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>RSCM lakukan implantasi LVAD paling kecil di dunia</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:55:30 +0700</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Rumah Sakit Umum Pusat Nasional Dr. Cipto Mangunkusumo (RSCM) mengklaim telah sukses melakukan implantasi Left ...</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683837/rscm-lakukan-implantasi-lvad-paling-kecil-di-dunia</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-08.08.25.jpeg</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Bareskrim bongkar dugaan peredaran narkoba di THM Five Star, Bali</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:54:23 +0700</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Direktorat Tindak Pidana Narkoba (Dittipidnarkoba) Bareskrim Polri membongkar dugaan peredaran narkoba di tempat ...</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683835/bareskrim-bongkar-dugaan-peredaran-narkoba-di-thm-five-star-bali</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1000080547.jpg</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Trump perintahkan investigasi atas kebocoran informasi stok amunisi AS</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:53:14 +0700</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Presiden Amerika Serikat Donald Trump telah memerintahkan penyelidikan baru terkait pengungkapan informasi mengenai ...</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683832/trump-perintahkan-investigasi-atas-kebocoran-informasi-stok-amunisi-as</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/AA-20260802-42124703-42124695-TRUMPTARGETING_BANNER_DISPLAYED_IN_TEHRANS_AZADI_SQUARE.jpg</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Permohonan imigrasi AS "menumpuk" sampai 7,5 juta</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:52:38 +0700</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Lambatnya proses imigrasi Amerika Serikat telah menyebabkan penumpukan permohonan hingga mencapai rekor tertinggi, ...</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683829/permohonan-imigrasi-as-menumpuk-sampai-75-juta</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/07/CjkinzN000022_20251107_CBMFN0A001a.jpg</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>KPK terima permintaan Kejagung untuk periksa Febrie Adriansyah</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:52:37 +0700</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Komisi Pemberantasan Korupsi (KPK) menerima permintaan Kejaksaan Agung untuk memeriksa mantan Jaksa Agung Muda Bidang ...</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683828/kpk-terima-permintaan-kejagung-untuk-periksa-febrie-adriansyah</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1001013665.jpg</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Banyak Hipertensi, pelajar dilibatkan jadi agen penggerak hidup sehat</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:50:45 +0700</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota (Pemkot) Kediri, Jawa Timur, melibatkan pelajar Sekolah Menengah Atas (SMA) sebagai peer educator atau ...</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683825/banyak-hipertensi-pelajar-dilibatkan-jadi-agen-penggerak-hidup-sehat</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000897304.jpg</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Redmi Note 17 masuk ke pasar India, spesifikasinya mirip versi China</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:48:51 +0700</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Redmi telah meluncurkan Redmi Note 17 di pasar India, menawarkan ponsel yang spesifikasinya hampir ...</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683824/redmi-note-17-masuk-ke-pasar-india-spesifikasinya-mirip-versi-china</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/InShot_20260807_120221131.jpg</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>PPAL kenang jasa para pahlawan dengan berziarah ke TMP Kalibata</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:43:56 +0700</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Persatuan Purnawirawan Angkatan Laut (PPAL) mengenang jasa para pahlawan bangsa dengan menggelar ziarah di Taman Makam ...</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683823/ppal-kenang-jasa-para-pahlawan-dengan-berziarah-ke-tmp-kalibata</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001561814.jpg</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Kementerian PU gelar Gerakan Irigasi Bersih dukung ketahanan pangan</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:41:58 +0700</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Kementerian Pekerjaan Umum (PU) melalui Direktorat Jenderal Sumber Daya Air (SDA) menggelar Gerakan Irigasi ...</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683820/kementerian-pu-gelar-gerakan-irigasi-bersih-dukung-ketahanan-pangan</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000878502.jpg</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>DKI akui ada tumpang tindih jalur mikrolet 44 dan Mikrotrans JAK 48A</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:38:31 +0700</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi DKI Jakarta mengakui ada tumpang tindih jalur antara mikrolet 44 yang melayani trayek Kampung ...</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683817/dki-akui-ada-tumpang-tindih-jalur-mikrolet-44-dan-mikrotrans-jak-48a</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_2478.jpeg</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Bandara Soetta genjot peningkatan infrastruktur dan layanan digital</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:30:20 +0700</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>PT Angkasa Pura Indonesia (Persero) atau InJourney Airports melalui Kantor Cabang Bandara Internasional Soekarno-Hatta, ...</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683815/bandara-soetta-genjot-peningkatan-infrastruktur-dan-layanan-digital</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000453452.jpg</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Presiden Polandia tegaskan tak akan legalkan pernikahan sesama jenis</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:29:44 +0700</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Presiden Polandia Karol Nawrocki mengatakan dirinya terbuka untuk membahas peraturan yang memungkinkan untuk melegalkan ...</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683813/presiden-polandia-tegaskan-tak-akan-legalkan-pernikahan-sesama-jenis</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/09/21/ring-2407552_960_720.jpg</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>KemenPPPA gelar Kemudi Anak, sarana penyampaian aspirasi ke pemerintah</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:28:02 +0700</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>Kementerian Pemberdayaan Perempuan dan Perlindungan Anak (PPPA) menggelar kegiatan Kemudi Anak (Kepemimpinan Muda ...</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683811/kemenpppa-gelar-kemudi-anak-sarana-penyampaian-aspirasi-ke-pemerintah</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-05-at-15.30.43.jpg</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Polres Jakpus sita 132 kilogram ganja, dua DPO masih diburu</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:20:23 +0700</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Polres Metro Jakarta Pusat menyita sekitar 132 kilogram ganja dari pengungkapan tiga kasus peredaran narkotika ...</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683807/polres-jakpus-sita-132-kilogram-ganja-dua-dpo-masih-diburu</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/20260807_103050.jpg</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>DPP Perbasi gandeng Nico Widmer untuk kembangkan 3x3 di Indonesia</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:15:15 +0700</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>Badan 3x3 Dewan Pengurus Pusat Persatuan Bola Basket Seluruh Indonesia (DPP Perbasi) menggandeng Nico Widmer untuk ...</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683805/dpp-perbasi-gandeng-nico-widmer-untuk-kembangkan-3x3-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000475111.jpg</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Pramono angkat bicara soal temuan senjata di sekolah</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:12:42 +0700</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung mengatakan temuan berupa 995 pucuk senjata dan narkoba di salah satu sekolah ...</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683803/pramono-angkat-bicara-soal-temuan-senjata-di-sekolah</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_2465.jpeg</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Gubernur prioritaskan pembangunan jalan puluhan tahun dinanti di Nias</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:10:50 +0700</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Gubernur Sumatera Utara (Sumut) Bobby Nasution memprioritaskan pembangunan infrastruktur jalan yang telah dinantikan ...</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683799/gubernur-prioritaskan-pembangunan-jalan-puluhan-tahun-dinanti-di-nias</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001034262.jpg</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Daftar juara Piala Presiden 2015-2026, Persebaya juara terbaru</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:09:30 +0700</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Persebaya Surabaya berhasil mencatatkan sejarah baru dengan keluar sebagai juara Piala Presiden 2026. Gelar tersebut ...</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683796/daftar-juara-piala-presiden-2015-2026-persebaya-juara-terbaru</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/persebaya-juara-piala-presiden-2026-2836164.jpg</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Kalbar perkuat kesiapsiagaan hadapi puncak karhutla</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:07:30 +0700</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi Kalimantan Barat (Pemprov Kalbar) memperkuat kesiapsiagaan menghadapi puncak ancaman kebakaran ...</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683792/kalbar-perkuat-kesiapsiagaan-hadapi-puncak-karhutla</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-09.02.55.jpeg</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Kepala BNPB perkuat antisipasi karhutla di lahan gambut di Kubu Raya</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:06:38 +0700</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Kepala Badan Nasional Penanggulangan Bencana (BNPB) Suharyanto mengatakan kebakaran hutan dan lahan (karhutla) di ...</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683788/kepala-bnpb-perkuat-antisipasi-karhutla-di-lahan-gambut-di-kubu-raya</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/767101496_1372423328362643_3390602255780147155_n.jpeg</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Terkait 995 senjata, Yayasan sekolah tegaskan tak ada ekskul menembak</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:05:58 +0700</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Pengurus yayasan sekolah swasta di kawasan Pondok Pinang, Kebayoran Lama, Jakarta Selatan, menegaskan tidak ada ...</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683785/terkait-995-senjata-yayasan-sekolah-tegaskan-tak-ada-ekskul-menembak</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001016071.jpg</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Telkom pangkas 34 entitas dalam proses transformasi BUMN</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:05:29 +0700</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>PT Telkom Indonesia memangkas 34 entitas dari 67 entitas usaha dalam proses transformasi BUMN untuk membangun ...</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683781/telkom-pangkas-34-entitas-dalam-proses-transformasi-bumn</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-10.05.33.jpeg</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>KPPPA: Kepemimpinan ASN perempuan harus ditopang kemampuan komunikasi</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:04:45 +0700</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>Kementerian Pemberdayaan Perempuan dan Perlindungan Anak (KPPPA) menekankan pentingnya kemampuan komunikasi sebagai ...</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683779/kpppa-kepemimpinan-asn-perempuan-harus-ditopang-kemampuan-komunikasi</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-06-at-15.46.49.jpeg</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>CAF sampaikan dukungan penuh untuk Gianni Infantino</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:01:11 +0700</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Konfederasi Sepak Bola Afrika (CAF) menyampaikan dukungan penuh kepada Presiden FIFA Gianni Infantino dan ...</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683775/caf-sampaikan-dukungan-penuh-untuk-gianni-infantino</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_669e9774d8942ff9475105617b428127.jpg</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>BSKDN kembangkan SINTESIS hadirkan kebijakan tepat sasaran</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:58:33 +0700</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Badan Strategi Kebijakan Dalam Negeri (BSKDN) Kementerian Dalam Negeri terus memperkuat pengembangan platform SINTESIS ...</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683772/bskdn-kembangkan-sintesis-hadirkan-kebijakan-tepat-sasaran</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000581661.jpg</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Yayasan tegaskan belajar mengajar tetap normal usai temuan 995 senjata</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:56:18 +0700</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Pengurus yayasan sekolah swasta di Pondok Pinang, Kebayoran Lama, menegaskan kegiatan belajar mengajar tetap berjalan ...</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683769/yayasan-tegaskan-belajar-mengajar-tetap-normal-usai-temuan-995-senjata</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001016025.jpg</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Mantan PM Malaysia Ismail Sabri dirawat di RS di tengah kasus hukum</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:56:13 +0700</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Mantan perdana menteri Malaysia, Ismail Sabri Yaakob (66), dikabarkan dirawat di Rumah Sakit Institut Jantung ...</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683767/mantan-pm-malaysia-ismail-sabri-dirawat-di-rs-di-tengah-kasus-hukum</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/08/20/reuters_ismail_sabri2.jpg</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Pemerintah akan kirim tim untuk kaji langkah pemulihan Montara</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:52:04 +0700</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa menyatakan Pemerintah akan mengirim tim riset untuk mengkaji secara komprehensif ...</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683765/pemerintah-akan-kirim-tim-untuk-kaji-langkah-pemulihan-montara</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-08.12.49.jpeg</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Kemenkes: Pasien BPJS yang viral tunggu 8 jam karena HCU RSCM terbatas</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:51:26 +0700</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan (Kemenkes) mengatakan pasien BPJS Kesehatan yang viral di media sosial harus menunggu selama ...</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683764/kemenkes-pasien-bpjs-yang-viral-tunggu-8-jam-karena-hcu-rscm-terbatas</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/27/WhatsApp-Image-2025-11-27-at-17.49.15_831c9c5c.jpg</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>OpenAI akan rilis "speaker donat" pintar pada 2027</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:49:48 +0700</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Perusahaan kecerdasan buatan (AI) asal Amerika Serikat, OpenAI, sedang mengembangkan perangkat rumah tangga berbasis AI ...</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683760/openai-akan-rilis-speaker-donat-pintar-pada-2027</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/thumbs_b_c_c48eb58d9c1e7c83fd91f3633ecd20ec.jpg</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Iran kecam "diplomasi sandiwara" oleh AS</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:49:35 +0700</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Mohammad Bagher Ghalibaf, ketua parlemen Iran sekaligus ketua tim negosiator Iran dalam pembicaraan dengan ...</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683759/iran-kecam-diplomasi-sandiwara-oleh-as</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/AA-20260802-42124703-42124695-TRUMPTARGETING_BANNER_DISPLAYED_IN_TEHRANS_AZADI_SQUARE.jpg</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Kemenperin perkuat pengelolaan kemasan untuk pacu industri hijau</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:45:49 +0700</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Kementerian Perindustrian (Kemenperin) memperkuat pengelolaan kemasan pascakonsumsi sebagai bagian dari upaya ...</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683757/kemenperin-perkuat-pengelolaan-kemasan-untuk-pacu-industri-hijau</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/3-1.jpeg</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Penyanyi Ghea Indrawari hadirkan "Rasi Bintang" sebagai album kedua</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:44:06 +0700</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Penyanyi Ghea Indrawari merilis album studio keduanya bertajuk "Rasi Bintang" di seluruh platform musik ...</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683755/penyanyi-ghea-indrawari-hadirkan-rasi-bintang-sebagai-album-kedua</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Ghea-Indrawari-05.JPG.jpeg</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Presiden FA Yordania tegaskan tak akan dukung Gianni Infantino</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:32:53 +0700</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Presiden Asosiasi Sepak Bola (FA) Yordania Ali Al Hussein menegaskan tak akan memberikan dukungan kepada Gianni ...</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683753/presiden-fa-yordania-tegaskan-tak-akan-dukung-gianni-infantino</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/thumbs_b_c_4b35583a6a2b064678bf5739a06f4ada.jpg</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Warisan "fair play" dari stadion para pejuang</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:32:53 +0700</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Peluit panjang mengakhiri adu penalti di Stadion Kapten I Wayan Dipta, Gianyar, Kamis (6/8) malam. Para pemain ...</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683752/warisan-fair-play-dari-stadion-para-pejuang</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/279254.jpg</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Maroko siap bekerja sama pulangkan imigran anak</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:29:45 +0700</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>Pemerintah Maroko menyatakan siap bekerja sama dengan Spanyol dan Uni Eropa untuk memulangkan anak-anak di bawah umur ...</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683749/maroko-siap-bekerja-sama-pulangkan-imigran-anak</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/thumbs_b_c_163e90d67c855177fcf9553fd9012181.jpg</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>AFA berikan dukungan untuk Gianni Infantino</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:27:34 +0700</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Federasi Sepak Bola Argentina (AFA) memberikan dukungan untuk Presiden FIFA Gianni Infantino yang pada beberapa waktu ...</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683747/afa-berikan-dukungan-untuk-gianni-infantino</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/20/timnas-spanyol-juara-piala-dunia-2026-2824232.jpg</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>BBTNKS luncurkan program penghijauan di kaki Gunung Kerinci</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:27:19 +0700</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Balai Besar Taman Nasional Kerinci Seblat (BBTNKS) meluncurkan program penghijauan (greenline) di kaki Gunung Kerinci ...</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683743/bbtnks-luncurkan-program-penghijauan-di-kaki-gunung-kerinci</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/566130.jpg</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Arab Saudi yakini kelompok bersenjata asing siapkan serangan</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:26:13 +0700</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Arab Saudi memperoleh informasi intelijen yang mengindikasikan adanya persiapan serangan terhadap kerajaan ...</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683740/arab-saudi-yakini-kelompok-bersenjata-asing-siapkan-serangan</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/01/23/CjkinzN007037_20220123_CBPFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Pramono Sindir ASN 'Curi-curi' Tak Naik Transportasi Umum Saat Rabu: Saya Tahu</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:44:52 +0700</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Pramono menyoroti ASN yang masih menggunakan mobil pribadi meski diwajibkan menggunakan transportasi umum setiap Rabu. Dia tahu ada ASN yang tak patuh.</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608326/pramono-sindir-asn-curi-curi-tak-naik-transportasi-umum-saat-rabu-saya-tahu</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/gubernur-dki-jakarta-pramono-anung-brigittadetik-1786081467940_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Kera yang Menyerang di Inhil Sudah Ditangkap, Warga Diminta Tetap Waspada</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:31:34 +0700</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Kera ekor panjang yang menyerang 17 warga di Tembilahan, Riau, telah ditangkap. Polisi imbau warga tetap waspada meski serangan sudah berhenti.</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608316/kera-yang-menyerang-di-inhil-sudah-ditangkap-warga-diminta-tetap-waspada</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/kera-ekor-panjang-yang-menyerang-warga-sudah-diamankan-pada-kamis-682026-1786080546645_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Melihat Lebih Dekat Stasiun Gunung Putri di Bogor yang Terbengkalai</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:31:14 +0700</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Rizky Adha Mahendra</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Kereta melintas setiap hari, tapi tak satu pun penumpang naik atau turun di Stasiun Gunung Putri. Bangunan stasiun itu kini terbengkalai dipenuhi ilalang.</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608315/melihat-lebih-dekat-stasiun-gunung-putri-di-bogor-yang-terbengkalai</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/kondisi-stasiun-gunung-putri-bogor-yang-kini-terbengkalai-1786080454648_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>2 Pelaku Demo Anarkis Minta Jatah Limbah Perusahaan di Tangerang Ditangkap</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:28:20 +0700</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Polda Banten menangkap dua pria yang diduga menjadi otak demonstrasi anarkis di PT EDS. Mereka dituduh merusak fasilitas dan menuntut pengelolaan limbah.</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608304/2-pelaku-demo-anarkis-minta-jatah-limbah-perusahaan-di-tangerang-ditangkap</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/07/25/ilustrasi-penangkapan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Pramono Pastikan Gaji ASN DKI Aman Meski DBH Dipangkas: Semuanya Terpenuhi</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:25:13 +0700</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Pramono menegaskan kewajiban Pemprov DKI kepada ASN tetap dapat dipenuhi. Pembayaran gaji maupun hak-hak pegawai tidak terdampak oleh kebijakan pemangkasan DBH.</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608303/pramono-pastikan-gaji-asn-dki-aman-meski-dbh-dipangkas-semuanya-terpenuhi</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/gubernur-dki-jakarta-pramono-anung-beliadetikcom-1786080281071_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Balap Liar di Taman Mini Dibubarkan, Pelaku Kocar-kacir Dikejar Polisi</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:19:38 +0700</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Tim Patroli Brimob membubarkan aksi balap liar di Jakarta Timur, mengamankan 11 pemuda dan sepeda motor. Patroli rutin untuk mencegah gangguan keamanan.</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608298/balap-liar-di-taman-mini-dibubarkan-pelaku-kocar-kacir-dikejar-polisi</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/patroli-gabungan-brimob-polda-metro-jaya-dan-tim-perintis-polres-jakarta-timur-membubarkan-balap-liar-di-kawasan-taman-mini-ja-1786079956709_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Pramono Perintahkan DLH Bersihkan Gunungan Sampah Dekat SD Kedaung Kali Angke</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:17:36 +0700</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Pramono Anung memerintahkan Dinas Lingkungan Hidup (DLH) DKI Jakarta segera membersihkan gunungan sampah di dekat SDN Kedaung Kali Angke 12, Jakarta Barat.</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608290/pramono-perintahkan-dlh-bersihkan-gunungan-sampah-dekat-sd-kedaung-kali-angke</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/gubernur-dki-jakarta-pramono-anung-beliadetikcom-1786079771132_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Bareskrim Bongkar Peredaran Narkoba di Five Stars Bali, 53 Orang Diamankan</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:13:00 +0700</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Dittipidnarkoba Bareskrim Polri mengungkap peredaran narkoba di kelab malam Five Stars Bali, mengamankan 53 orang sebagai tersangka dan saksi.</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608288/bareskrim-bongkar-peredaran-narkoba-di-five-stars-bali-53-orang-diamankan</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/bareskrim-polri-mengungkap-peredaran-di-five-stars-denpasar-bali-dan-mengamankan-53-orang-1786079431797_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Legislator Soroti Nakes Hina Pasien BPJS, Minta Evaluasi Total Manajemen RS</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:06:25 +0700</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Matius Alfons Hutajulu</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Ia memandang harus ada evaluasi total terkait durasi masa tunggu bagi pasien rawat inap untuk mendapatkan perawatan.</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608270/legislator-soroti-nakes-hina-pasien-bpjs-minta-evaluasi-total-manajemen-rs</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/04/16/ilustrasi-dokter-dengan-pasien-1744783009967_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Ada Konflik Internal di Balik Temuan Ratusan Senjata di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:58:43 +0700</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Taufiq Syarifudin, Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Pihak sekolah mengungkap temuan ratusan senjata di ruang mantan ketua yayasan, terkait sengketa internal. Polisi selidiki kasus ini lebih lanjut.</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608255/ada-konflik-internal-di-balik-temuan-ratusan-senjata-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/temuan-ratusan-pucuk-senjata-di-sekolah-swasta-di-pondok-pinang-jakarta-selatan-1786014363648_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Ketua DPD Sambangi Kediaman Boediono, Sampaikan Undangan Sidang Bersama</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:57:56 +0700</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Ketua DPD RI Sultan Najamudin mengunjungi kediaman Boediono. Kunjungan itu dalam rangka menyampaikan undangan Sidang Bersama DPR-DPD RI 2026.</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608253/ketua-dpd-sambangi-kediaman-boediono-sampaikan-undangan-sidang-bersama</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/ketua-dpd-ri-sultan-baktiar-najamudin-menyambangi-kediaman-wakil-presiden-ke-11-ri-boediono-1786078635188_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Dinkes Pastikan Nakes Viral Cibir Pasien BPJS Bukan Pegawai Pemprov DKI</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:53:23 +0700</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Dinkes DKI Jakarta menegaskan nakes yang mencibir pasien BPJS bukan pegawai Pemprov. Nakes tersebut tidak bekerja di RSUD milik Pemprov Jakarta.</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608241/dinkes-pastikan-nakes-viral-cibir-pasien-bpjs-bukan-pegawai-pemprov-dki</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/kepala-dinas-kesehatan-dki-jakarta-ani-ruspitawati-brigittadetik-1786078386930_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Pemprov DKI Kaji Rute Angkot JakLingko dan M44 Agar Tak Tumpang Tindih</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:30:07 +0700</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Dinas Perhubungan (Dishub) DKI Jakarta akan mengkaji ulang rute Mikrotrans atau angkot JakLingko 48 dengan angkot M44 jurusan Karet-Kampung Melayu.</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608209/pemprov-dki-kaji-rute-angkot-jaklingko-dan-m44-agar-tak-tumpang-tindih</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/angkot-kosong-ditinggal-oleh-sopirnya-yang-sedang-berdemo-di-balai-kota-adhfar-aulia-syuhadadetikcom-1785990400876_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Anggota DPR Minta Usut Tuntas Temuan Ratusan Senjata di Sekolah Swasta Jaksel</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:27:00 +0700</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Matius Alfons Hutajulu</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Sejumlah anggota DPR RI turut menanggapi perihal temuan ratusan senjata di salah satu sekolah swasta di Kebayoran Lama. Mereka meminta temuan itu diusut tuntas.</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608205/anggota-dpr-minta-usut-tuntas-temuan-ratusan-senjata-di-sekolah-swasta-jaksel</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/temuan-ratusan-pucuk-senjata-di-sekolah-swasta-di-pondok-pinang-jakarta-selatan-1786014363566_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Pramono Dukung Polisi Usut Temuan Senjata-Narkoba di Sekolah Swasta Jaksel</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:25:11 +0700</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Gubernur Jakarta Pramono Anung mendukung aparat mengusut tuntas temuan ratusan senjata, narkoba, hingga film dewasa di sebuah sekolah swasta di Jaksel.</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608201/pramono-dukung-polisi-usut-temuan-senjata-narkoba-di-sekolah-swasta-jaksel</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/temuan-ratusan-pucuk-senjata-di-sekolah-swasta-di-pondok-pinang-jakarta-selatan-1786014363566_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Kera Ekor Panjang Serang Warga Inhil, 18 Orang Jadi Korban</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 10:34:18 +0700</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Kera ekor panjang menyerang permukiman di Tembilahan, Riau, melukai 18 warga. Pemerintah setempat meningkatkan kewaspadaan dan penanganan.</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608101/kera-ekor-panjang-serang-warga-inhil-18-orang-jadi-korban</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/10/05/kera-ekor-panjang-di-kabupaten-gunungkidul-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Mail Syahputra, Asisten Nikita Mirzani Ajukan PK Dugaan TTPU dan Pemerasan</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:24:54 +0700</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Ismail Marzuki, asisten Nikita Mirzani, ajukan PK atas dugaan pemerasan dan TPPU. Kuasa hukum kritik kekhilafan hakim dalam penerapan UU ITE.</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8608269/mail-syahputra-asisten-nikita-mirzani-ajukan-pk-dugaan-ttpu-dan-pemerasan</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/07/24/nikita-mirzani-jalani-sidang-ttpu-1753328999013_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Fakta Lain soal Anak Vicky Prasetyo dengan Fangfang</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:03:13 +0700</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Fangfang mengungkap ketidakterbukaan Vicky Prasetyo tentang jumlah anaknya. Dia terkejut mengetahui anak yang dikandungnya adalah anak kesembilan.</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8608140/fakta-lain-soal-anak-vicky-prasetyo-dengan-fangfang</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/17/fangfang-1784271583661_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Pawzia Bikin Heboh Lewat Selain Donatur Dilarang Ngatur</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:37:41 +0700</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Pawzia merilis lagu terbaru Selain Donatur Dilarang Ngatur yang viral. Meski bahagia, ia menghadapi perbandingan dengan Veni Nur yang menyakitkan.</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/music/d-8608098/pawzia-bikin-heboh-lewat-selain-donatur-dilarang-ngatur</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/pawzia-1786073508427_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Tantang Titi Kamal hingga Sarah Tumiwa Bintangi Perumahan Laddaland</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:25:58 +0700</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Titi Kamal bintangi film horor psikologis Perumahan Laddaland. Titi Kamal hingga Sarah Tumiw amenceritakan tantangan membintangi film tersebut.</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/movie/d-8607954/tantang-titi-kamal-hingga-sarah-tumiwa-bintangi-perumahan-laddaland</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/film-perumahan-laddaland-1786066142597_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Simulasi Ranking FIFA Indonesia vs Singapura di Piala AFF 2026, Menang Jadi Harga Mati</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:49:28 +0700</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Simulasi hitungan ranking FIFA Timnas Indonesia vs Singapura di Piala AFF 2026, Garuda wajib menang jika tak ingin lengser.</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865194/simulasi-ranking-fifa-indonesia-vs-singapura-di-piala-aff-2026-menang-jadi-harga-mati</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/yNQRBwgJz2YPPsUobmy3fY0wL6Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Piala-AFF-2026-Timnas-Indonesia-Tekuk-Timor-Leste-3-0_20260731_231927.jpg</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Penemuan 995 Senpi di Sekolah Jaksel, Ketua Komisi X DPR RI: 'Ini Persoalan Serius'</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:49:23 +0700</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>Ketua Komisi X DPR meminta polisi mengusut temuan 995 senjata di sekolah Jaksel. Perbakin menyebutnya airsoft gun untuk olahraga</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865193/penemuan-995-senpi-di-sekolah-jaksel-ketua-komisi-x-dpr-ri-ini-persoalan-serius</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/c23bmk4PHY76ZCmOECtNP5j3wK4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ratusan-senjata-api-di-sekolah-swasta-Pondok-Pinang-Kebayoran-Lama-Jakarta-Selatan.jpg</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Kode Redeem FF Terbaru Hari Ini, Jumat 7 Agustus 2026: Klaim Hadiahnya Secara Gratis</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:48:10 +0700</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>Kumpulan kode redeem Free Fire terbaru pada hari ini, Jumat (7/8/2026) di laman reward.ff.garena.com, klaim kodenya dan dapat hadiah gratisnya.</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/techno/7865192/kode-redeem-ff-terbaru-hari-ini-jumat-7-agustus-2026-klaim-hadiahnya-secara-gratis</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8I9GRYZwCbjGkKc3Ukw81342xcw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/bermain-gim-Garena-Free-Fire-FF-baru-saja.jpg</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Kementerian Luar Negeri Himpun Masukan Multipihak, Perkuat Diplomasi Dekarbonisasi</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:42:24 +0700</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>Masukan peserta akan menjadi bahan pendalaman dalam pertemuan dengan tenant dan kunjungan lapangan ke KEK Batang.</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865191/kementerian-luar-negeri-himpun-masukan-multipihak-perkuat-diplomasi-dekarbonisasi</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/3-KA1NYO2DeLd13wC1FvminrfdU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/iplomasi-dekarbonisasi-qw.jpg</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Timnas Voli Putra Indonesia Genjot Fisik Jelang Asian Games 2026, Dony Haryono: Latihan Semi Militer</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:42:11 +0700</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Timnas voli putra Indonesia menggenjot fisik jelang Asian Games 2026, Dony Haryono ikutan nimbrung dan sampai menyebutnya "latihan semi militer".</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865190/timnas-voli-putra-indonesia-genjot-fisik-jelang-asian-games-2026-dony-haryono-latihan-semi-militer</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8n95cKP3vY7IbrPEMcOvww5MSpU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/GAGAL-KE-FINAL-Asa-Timnas-voli-putra-Indonesia.jpg</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Mahfud MD Setuju Kabinet Bayangan Dibentuk: Pemerintahan Prabowo Menteri-menterinya Agak Lemah</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:42:09 +0700</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Eks Menkopolhukam RI Mahfud MD menilai, dibentuknya Kabinet Bayangan oleh Koalisi Masyarakat Sipil pada 27 Juli 2026 tidak jadi masalah.</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865189/mahfud-md-setuju-kabinet-bayangan-dibentuk-pemerintahan-prabowo-menteri-menterinya-agak-lemah</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/m1cHCktOUEc2P8dLa7Hi6MrNrcc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Mahfud-MD-Bicara-soal-Kasus-Saiful-Mujani_1.jpg</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Sosok Pelaku Pembunuhan Marbot Masjid di Purwakarta, Sakit Hati dengan Ucapan Korban</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:40:40 +0700</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Marbut masjid di Purwakarta tewas dibacok tetangganya akibat sakit hati sering dihina pengangguran. Pelaku ditangkap dengan ancaman 15 tahun penjara.</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865188/sosok-pelaku-pembunuhan-marbot-masjid-di-purwakarta-sakit-hati-dengan-ucapan-korban</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iVQoFd00f4I54X3zKDiHAJJIyGM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Marbot-Masjid-Tewas.jpg</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Harga Emas Antam Hari Ini, Jumat 7 Agustus 2026: Terjun di Level Rp2.650.000 per Gram</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:38:19 +0700</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Harga emas pada hari ini, Jumat (7/8/2026), terjun drastis di level Rp 2.650.000, simak rincian harga emas terbarunya.</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865187/harga-emas-antam-hari-ini-jumat-7-agustus-2026-terjun-di-level-rp2650000-per-gram</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/J5yz2H6KghKOYYUDkxXa0zEptx0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Harga-Emas-Antam-Naik_20251007_212034.jpg</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Persiapan India sebagai Tuan Rumah Kejuaraan Dunia BWF 2026, Cegah Burung dan Monyet Masuk Arena</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:37:29 +0700</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>India selaku tuan rumah menyiapkan langkah antisipasi guna mencegah burung dan monyet masuk arena jelang Kejuaraan Dunia BWF 2026.</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865186/persiapan-india-sebagai-tuan-rumah-kejuaraan-dunia-bwf-2026-cegah-burung-dan-monyet-masuk-arena</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/SKgoLpkjtyOCGf319vgkqeLC20M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/India-Open-kotoran-Burung-Loh-Kean-Yae.jpg</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban IPAS Kelas 6 SD Kurikulum Merdeka Hal 161 Edisi Revisi: Ayo, Simpulkan</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:37:02 +0700</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>Simak berikut merupakan kunci jawaban buku pelajaran IPAS kelas 6 SD/MI Kurikulum Merdeka (Edisi Revisi) halaman 161 bab 6: Ayo, Simpulkan</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865185/kunci-jawaban-ipas-kelas-6-sd-kurikulum-merdeka-hal-161-edisi-revisi-ayo-simpulkan</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/O6GemeIcgrqlBjxOSV1OQuh-qRw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Siswa-Tetap-Semangat-Masuk-Sekolah-Setelah-Libur-Lebaran-2026_20260330_123016.jpg</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Banyak Ibu Kejar Stok ASI sampai Freezer Penuh, Dokter Ingatkan Risiko Mastitis karena Oversupply</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:34:49 +0700</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Banyak ibu berlomba memperlihatkan freezer penuh Tren menyimpan stok ASI dalam jumlah besar semakin sering terlihat di media sosial.</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865184/banyak-ibu-kejar-stok-asi-sampai-freezer-penuh-dokter-ingatkan-risiko-mastitis-karena-oversupply</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/deqyqX9iXfkTNmFZ7ai7E69o1T8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/asi-eksklusif-2-0313.jpg</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Bareskrim Bongkar Sarang Narkoba di Kelab Malam Bali, Dikendalikan Manajemen, 53 Orang Diamankan</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:33:31 +0700</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>Bareskrim bongkar sarang narkoba yang beroperasi di kelab malam bernama Five Star di Kota Denpasar, Bali pada Jumat (7/8/2026) dini hari</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865183/bareskrim-bongkar-sarang-narkoba-di-kelab-malam-bali-dikendalikan-manajemen-53-orang-diamankan</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/c3WhMmS7ZqVfAXc7O59KV7fKwsI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/peredaran-narkoba-di-Five-Star-di-Denpasar-Bali.jpg</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>RB Leipzig Sindir Fabrizio Romano saat Resmikan Transfer Yan Diomande ke Real Madrid</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:28:07 +0700</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>RB Leipzig sindir Fabrizio Romano saat umumkan transfer Yann Diomande ke Real Madrid dengan kalimat "HERE WE ACTUALLY GO".</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865182/rb-leipzig-sindir-fabrizio-romano-saat-resmikan-transfer-yan-diomande-ke-real-madrid</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/E54RA_I8M15KG7G9nmg6eXOU94s=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-klub-Real-Madrid.jpg</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Terungkap Lokasi Rumah Sakit dan Alasan Yurizal Pasien BPJS yang Menunggu 8 Jam Sebelum Meninggal</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:27:50 +0700</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Kasus komentar niremapti nakes dan dokter pada pasien BPJS viral.Hebohnya kasus ini mengungkap fakta lokasi rumah sakit yang dimaksud.</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865181/terungkap-lokasi-rumah-sakit-dan-alasan-yurizal-pasien-bpjs-yang-menunggu-8-jam-sebelum-meninggal</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/JpmCUL7yNHEkxI9Hn17BoXEHfGw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ramli-di-rscm.jpg</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Ketua KPU Kotawaringin Timur Beserta 4 Komisioner Tersangka Dugaan Korupsi Dana Hibah Pilkada 2024</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:27:39 +0700</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Lima Komisioner KPU Kotawaringin Timur ditetapkan sebagai tersangka dugaan korupsi dana hibah Pilkada 2024.</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865180/ketua-kpu-kotawaringin-timur-beserta-4-komisioner-tersangka-dugaan-korupsi-dana-hibah-pilkada-2024</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/_CftJ4Pu8xm_7GEGubhbQ5d30Xs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Komisioner-KPU-Kotim-Tersangka_1.jpg</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Mantan Manajer Sarwendah Ungkap Kondisi Kesehatan Ruben Onsu di Tengah Isu Penyakit Kronis</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:20:14 +0700</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Mantan manajer Sarwendah, Nanda Persada mengungkap kondisi kesehatan Ruben Onsu setelah muncul isu penyakit kronis.</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865179/mantan-manajer-sarwendah-ungkap-kondisi-kesehatan-ruben-onsu-di-tengah-isu-penyakit-kronis</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZG3_PDED1CjlCCKn-J5WB8tswOA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ruben-Onsu-KPAI.jpg</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Bahasa Indonesia Kelas 9 Halaman 56, 57, 58 Edisi Revisi Latihan 1</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:20:09 +0700</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Kunci jawaban Bahasa Indonesia kelas 9 halaman 56, 57, 58 Kurikulum Merdeka Edisi Revisi, Latihan 1 Bab 2 Belajar Berpantun.</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865178/kunci-jawaban-bahasa-indonesia-kelas-9-halaman-56-57-58-edisi-revisi-latihan-1</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/FBmkDqYmlx5UM0pD7_3NuyX3Hwc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SMP-BELAJAR-10.jpg</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Tim 9 Kejagung Jemput Eks Jampidsus Febrie Adriansyah di KPK Siang Ini</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:19:56 +0700</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>Tim 9 Kejagung bersiap melakukan pemeriksaan lanjutan terhadap mantan Jampidsus Febrie Adriansyah terkait kasus dugaan TPPU.</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865177/tim-9-kejagung-jemput-eks-jampidsus-febrie-adriansyah-di-kpk-siang-ini</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/gNaM9P5dS5GBE26SM6ozbYNMZJE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/mobil-siap-jemput-febrie-adriansyah-diperiksa-tim-9.jpg</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban IPAS 6 SD Kurikulum Merdeka Hal 167 Edisi Revisi: Satelit dan Teknologi Antariksa</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:19:31 +0700</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Berikut merupakan kunci jawaban buku pelajaran IPAS kelas 6 SD/MI Kurikulum Merdeka (Edisi Revisi) halaman 167 bab 6: Satelit dan Teknologi Antariksa</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865176/kunci-jawaban-ipas-6-sd-kurikulum-merdeka-hal-167-edisi-revisi-satelit-dan-teknologi-antariksa</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Q5yW0uMJfi6M5C8kylsmRdOWTcs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Siswa-Tetap-Semangat-Masuk-Sekolah-Setelah-Libur-Lebaran-2026_20260330_123000.jpg</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>SPK: Pernyataan Kampus soal Gaji Dosen Rp20-50 Juta Malah Timbulkan Polemik Baru</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:15:16 +0700</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>SPK menilai klaim gaji dosen Rp20 juta-Rp50 juta memicu polemik. Mereka menegaskan angka itu bukan gaji pokok, melainkan termasuk tunjangan</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865175/spk-pernyataan-kampus-soal-gaji-dosen-rp20-50-juta-malah-timbulkan-polemik-baru</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0GLE2g4P6afy-H0qs5aPIaR9ZVQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sidang-gaji-dosen-di-MK.jpg</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Pupuk Kaltim Kembangkan Agrowisata Berbasis Pertanian di Gowa</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 13:05:26 +0700</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – PT Pupuk Kalimantan Timur (Pupuk Kaltim) meresmikan Kampung Sawah Abadi (KSA) Bulutana di Kabupaten Gowa, Sulawesi Selatan, sebagai kawasan yang mengintegrasikan pertanian berkelanjutan dengan agrowisata. Program tersebut...</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjdxzl416/pupuk-kaltim-kembangkan-agrowisata-berbasis-pertanian-di-gowa</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260807130500-912.png</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Braze Perkuat Customer Engagement Berbasis AI di Indonesia</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:42:11 +0700</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Friska Yolandha</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA — Braze, platform customer engagement global terkemuka, mengumumkan bahwa PT Pertamina Patra Niaga, unit usaha ritel dan distribusi dari perusahaan energi milik negara Indonesia, serta PT Telkomsel,...</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjdx6b370/braze-perkuat-customer-engagement-berbasis-ai-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260807124137-824.png</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Amran Perintahkan Bulog Segera Kirim Beras SPHP ke Alor Untuk Netralisir Harga</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:44:01 +0700</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Friska Yolandha</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Kepala Badan Pangan Nasional (Bapanas) Andi Amran Sulaiman memerintahkan Perum Bulog segera mengirimkan beras program Stabilisasi Pasokan dan Harga Pangan (SPHP) ke Kabupaten Alor, Nusa Tenggara...</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjduhd370/amran-perintahkan-bulog-segera-kirim-beras-sphp-ke-alor-untuk-netralisir-harga</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/057218600-1771936201-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Kejagung Jemput Febrie Adriansyah di Rutan KPK</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:57:59 +0700</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>Febrie akan menjalani pemeriksaan lanjutan terkait kasus TPPU.</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264134/kejagung-jemput-febrie-adriansyah-di-rutan-kpk</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/KHyKZj-hqnufk-4rOxO_1qVv9P8=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317957/original/009574100_1786082243-IMG_20260807_113438_2.jpg</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Profil Muhammad Soleh Pengacara No Viral No Justice, Warisannya Mengubah Sistem Pemilu</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:14:38 +0700</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>Gugatan yang diajukan pada 2008 bukan sekadar memenangkan sengketa, melainkan mengubah cara rakyat memilih wakilnya di parlemen.</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264111/profil-muhammad-soleh-pengacara-no-viral-no-justice-warisannya-mengubah-sistem-pemilu</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/_n4mLUYf1d8_RgZK65k5kyBXjT4=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317874/original/090240100_1786076097-079028200_1786075648-IMG-20260807-WA0005.webp</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Hype</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Oasis Dikabarkan Reuni Akhir Tahun 2026</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 13:08:29 +0700</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>Oasis dikabarkan akan gelar reuni akhir tahun 2026, berniat kumpulkan semua anggota</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/hype/read/2026/08/07/130702166/oasis-dikabarkan-reuni-akhir-tahun-2026</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/yDZlmZp-eGtEdBECat7fnJnH2ns=/0x0:660x440/1200x675/filters:watermark(data/photo/2026/01/30/697c8191ee571.png,0,-0,1)/data/photo/2022/03/19/62358c5f714ec.jpg</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Dinkes DKI Pastikan Nakes yang Diduga Cibir Pasien BPJS Tak Bekerja di Faskes Pemprov</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 13:08:29 +0700</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Kadinkes DKI Ani Ruspitawati mengatakan, salah satu dari nakes yang diduga mencibir pasien BPJS Kesehatan memang bekerja di salah satu RS di Jakarta.</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/07/12401801/dinkes-dki-pastikan-nakes-yang-diduga-cibir-pasien-bpjs-tak-bekerja-di</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/_9yh_0xHF8tK9nA7GDO3b_Ou0Sc=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/05/11/6a01c0d6bef91.jpg</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Jelang Pemeriksaan Febrie, Mobil Tahanan Kejagung Parkir di Rutan KPK</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 13:08:29 +0700</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>Eks Jampidsus Febrie Adriansyah diperiksa KPK terkait dugaan TPPU. Mobil tahanan Jaksa Agung Muda Bidang Pidana Khusus tiba di Rutan KPK hari ini.</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/07/12132031/jelang-pemeriksaan-febrie-mobil-tahanan-kejagung-parkir-di-rutan-kpk</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/teM9JptxduI7Gzwj_RBDnH-LtyY=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/07/6a75652fe9a0b.jpeg</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I370"/>
+  <autoFilter ref="A1:I462"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 12:42 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-07.xlsx
+++ b/data/berita_2026-08-07.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$987</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1067</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I987"/>
+  <dimension ref="A1:I1067"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -46822,8 +46822,3768 @@
         </is>
       </c>
     </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Polri pastikan pemeriksaan anggota Polresta Banda Aceh transparan</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:35:08 +0700</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>Polri memastikan pemeriksaan dua anggota Polresta Banda Aceh oleh Divisi Profesi dan Pengamanan (Divpropam) Polri ...</t>
+        </is>
+      </c>
+      <c r="F988" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G988" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684707/polri-pastikan-pemeriksaan-anggota-polresta-banda-aceh-transparan</t>
+        </is>
+      </c>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000086556.jpg</t>
+        </is>
+      </c>
+      <c r="I988" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Bahlil tegaskan ekspor bauksit dan tembaga dilarang demi hilirisasi</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:34:54 +0700</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menegaskan pemerintah akan mempertahankan larangan ...</t>
+        </is>
+      </c>
+      <c r="F989" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G989" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684703/bahlil-tegaskan-ekspor-bauksit-dan-tembaga-dilarang-demi-hilirisasi</t>
+        </is>
+      </c>
+      <c r="H989" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_7687.jpg</t>
+        </is>
+      </c>
+      <c r="I989" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>BPOM: Apoteker perlu kuasai ATMP &amp; living therapy, dukung ketahanan RI</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:30:20 +0700</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>Badan Pengawas Obat dan Makanan (BPOM) mengatakan seiring perkembangan teknologi peran apoteker juga semakin ...</t>
+        </is>
+      </c>
+      <c r="F990" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G990" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684700/bpom-apoteker-perlu-kuasai-atmp-living-therapy-dukung-ketahanan-ri</t>
+        </is>
+      </c>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1786099467196.jpg</t>
+        </is>
+      </c>
+      <c r="I990" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Analis BEI lihat peluang kinerja LQ45 tumbuh pada semester II 2026</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:30:09 +0700</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>Analis Senior Divisi Riset Bursa Efek Indonesia (BEI) Fikrian Naufal Hardiatmojo melihat peluang kinerja 45 saham ...</t>
+        </is>
+      </c>
+      <c r="F991" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G991" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684696/analis-bei-lihat-peluang-kinerja-lq45-tumbuh-pada-semester-ii-2026</t>
+        </is>
+      </c>
+      <c r="H991" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000178311.jpg</t>
+        </is>
+      </c>
+      <c r="I991" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Danantara dan JBS Group kolaborasi pengembangan ekosistem protein RI</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:23:55 +0700</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>Danantara Indonesia melalui Danantara Investment Management (DIM) menjalin kemitraan strategis jangka panjang ...</t>
+        </is>
+      </c>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684692/danantara-dan-jbs-group-kolaborasi-pengembangan-ekosistem-protein-ri</t>
+        </is>
+      </c>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/19/WhatsApp-Image-2025-11-19-at-14.11.00_83e2c60d_1.jpg</t>
+        </is>
+      </c>
+      <c r="I992" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>ESDM: Implementasi B50 hasil pengembangan yang panjang</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:23:49 +0700</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>Kementerian Energi dan Sumber Daya Mineral (ESDM) mengatakan bahwa implementasi biodiesel B50 merupakan hasil ...</t>
+        </is>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G993" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5684688/esdm-implementasi-b50-hasil-pengembangan-yang-panjang</t>
+        </is>
+      </c>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/10/penggunaan-b50-mobil-industri-semarang-100726-aaa-116.jpg</t>
+        </is>
+      </c>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Pemkot Bandung: Pembelajaran siswa SDN 026 Bojongloa tetap berjalan</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:23:12 +0700</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Bandung memastikan proses kegiatan belajar sekitar 900 siswa SDN 026 Bojongloa harus tetap berjalan ...</t>
+        </is>
+      </c>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684684/pemkot-bandung-pembelajaran-siswa-sdn-026-bojongloa-tetap-berjalan</t>
+        </is>
+      </c>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_9198.jpeg</t>
+        </is>
+      </c>
+      <c r="I994" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>Temuan senjata api, Yayasan minta polisi lakukan sterilisasi sekolah</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:20:51 +0700</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>Kuasa hukum yayasan sekolah swasta di kawasan Pondok Pinang, Kebayoran Lama, Jakarta Selatan meminta kepolisian ...</t>
+        </is>
+      </c>
+      <c r="F995" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G995" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684675/temuan-senjata-api-yayasan-minta-polisi-lakukan-sterilisasi-sekolah</t>
+        </is>
+      </c>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001016766.jpg</t>
+        </is>
+      </c>
+      <c r="I995" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>FAA perintahkan inspeksi pesawat Boeing 737 MAX terkait retakan</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:15:31 +0700</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>Administrasi Penerbangan Federal (Federal Aviation Administration/FAA) Amerika Serikat (AS) telah memerintahkan ...</t>
+        </is>
+      </c>
+      <c r="F996" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G996" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684672/faa-perintahkan-inspeksi-pesawat-boeing-737-max-terkait-retakan</t>
+        </is>
+      </c>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/12/19/Xinhua-News-Agency.jpg</t>
+        </is>
+      </c>
+      <c r="I996" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Amartha komitmen dukung gaya hidup sehat lewat Amartha 10X Run 2026</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:13:45 +0700</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E997" t="inlineStr">
+        <is>
+          <t>Senior Vice President (SVP) Growth &amp; Marketing Amartha Financial Sheldon Chuan mengatakan perusahaan tersebut ...</t>
+        </is>
+      </c>
+      <c r="F997" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G997" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684668/amartha-komitmen-dukung-gaya-hidup-sehat-lewat-amartha-10x-run-2026</t>
+        </is>
+      </c>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000475673.jpg</t>
+        </is>
+      </c>
+      <c r="I997" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Legislator DKI dukung deklarasi perangi peredaran tramadol ilegal</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:12:20 +0700</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E998" t="inlineStr">
+        <is>
+          <t>Anggota Komisi B DPRD DKI Jakarta, Wa Ode Herlina mendukung deklarasi yang dilakukan Forum Koordinasi Pimpinan Kota ...</t>
+        </is>
+      </c>
+      <c r="F998" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G998" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684664/legislator-dki-dukung-deklarasi-perangi-peredaran-tramadol-ilegal</t>
+        </is>
+      </c>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000833694.jpg</t>
+        </is>
+      </c>
+      <c r="I998" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Isuzu mu-X terbaru dipamerkan di GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:11:33 +0700</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr">
+        <is>
+          <t>PT Isuzu Astra Motor Indonesia memamerkan Isuzu mu-X terbaru di ajang Gaikindo Indonesia International Auto Show ...</t>
+        </is>
+      </c>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G999" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5684663/isuzu-mu-x-terbaru-dipamerkan-di-giias-2026</t>
+        </is>
+      </c>
+      <c r="H999" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Photo-2-New-Isuzu-mu-X.jpg</t>
+        </is>
+      </c>
+      <c r="I999" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Sedikitnya tujuh tewas dalam penembakan di sekolah Thailand</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:11:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1000" t="inlineStr">
+        <is>
+          <t>ANTARA - Sedikitnya tujuh orang tewas dalam insiden penembakan di Sekolah Debsirin, Provinsi Nonthaburi, Thailand, ...</t>
+        </is>
+      </c>
+      <c r="F1000" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1000" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5684575/sedikitnya-tujuh-tewas-dalam-penembakan-di-sekolah-thailand</t>
+        </is>
+      </c>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SEDIKITNYA-TUJUH-TEWAS-DALAM-PENEMBAKAN-DI-SEKOLAH-THAILAND.jpg</t>
+        </is>
+      </c>
+      <c r="I1000" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Perdagangan luar negeri China tumbuh 19,2 persen pada Juli 2026</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:10:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1001" t="inlineStr">
+        <is>
+          <t>Data Administrasi Umum Kepabeanan (General Administration of Customs/GAC) China yang dirilis pada Jumat (7/8) ...</t>
+        </is>
+      </c>
+      <c r="F1001" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1001" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684659/perdagangan-luar-negeri-china-tumbuh-192-persen-pada-juli-2026</t>
+        </is>
+      </c>
+      <c r="H1001" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/CjkinzN000016_20260807_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1001" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Apakah gula aren lebih baik dari gula putih? Ini faktanya</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:09:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1002" t="inlineStr">
+        <is>
+          <t>Belakangan ini, gula aren semakin populer sebagai pemanis alami untuk berbagai makanan dan minuman. Mulai dari kopi ...</t>
+        </is>
+      </c>
+      <c r="F1002" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1002" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684656/apakah-gula-aren-lebih-baik-dari-gula-putih-ini-faktanya</t>
+        </is>
+      </c>
+      <c r="H1002" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/04/gula-merah-ppu.jpeg</t>
+        </is>
+      </c>
+      <c r="I1002" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Ideatax sebut penundaan PPh lokapasar beri ruang penyempurnaan</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:07:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1003" t="inlineStr">
+        <is>
+          <t>Praktisi perpajakan yang juga Managing Partner Ideatax Jonathan Nainggolan mengatakan keputusan pemerintah menunda ...</t>
+        </is>
+      </c>
+      <c r="F1003" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1003" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684653/ideatax-sebut-penundaan-pph-lokapasar-beri-ruang-penyempurnaan</t>
+        </is>
+      </c>
+      <c r="H1003" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Pemerintah-Tunda-Penerapan-Pajak-Lokapasar-060826-DAN-03.jpg</t>
+        </is>
+      </c>
+      <c r="I1003" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Bupati Bogor-KSAD tanda tangani pengolahan sampah jadi BBM</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:07:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1004" t="inlineStr">
+        <is>
+          <t>Bupati Bogor Rudy Susmanto dan Kepala Staf Angkatan Darat (KSAD) Jenderal TNI Maruli Simanjuntak menandatangani kerja ...</t>
+        </is>
+      </c>
+      <c r="F1004" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1004" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684651/bupati-bogor-ksad-tanda-tangani-pengolahan-sampah-jadi-bbm</t>
+        </is>
+      </c>
+      <c r="H1004" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1003321321.jpg</t>
+        </is>
+      </c>
+      <c r="I1004" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Bank BSN Catat Tingkat Keterhunian Rumah Subsidi Capai 92,58 Persen</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:05:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1005" t="inlineStr">
+        <is>
+          <t>Jakarta (ANTARA) – PT Bank Syariah Nasional (Bank BSN) mencatat tingkat validasi elektronik monitoring dan ...</t>
+        </is>
+      </c>
+      <c r="F1005" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1005" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684645/bank-bsn-catat-tingkat-keterhunian-rumah-subsidi-capai-9258-persen</t>
+        </is>
+      </c>
+      <c r="H1005" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-18.48.57-1.jpeg</t>
+        </is>
+      </c>
+      <c r="I1005" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Angkutan Retail KAI Capai 146.617 Ton, Naik 19,59 Persen dalam Dua Tahun</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:00:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1006" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) mencatat volume angkutan retail sebesar 146.617 ton sepanjang Januari–Juli ...</t>
+        </is>
+      </c>
+      <c r="F1006" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1006" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684641/angkutan-retail-kai-capai-146617-ton-naik-1959-persen-dalam-dua-tahun</t>
+        </is>
+      </c>
+      <c r="H1006" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-18.07.58.jpeg</t>
+        </is>
+      </c>
+      <c r="I1006" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>DPR minta usut tuntas kasus temuan senjata demi keamanan pendidikan</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:59:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Komisi X DPR RI Lalu Hadrian Irfani meminta kepada aparat untuk mengusut tuntas kasus temuan ratusan ...</t>
+        </is>
+      </c>
+      <c r="F1007" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1007" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684639/dpr-minta-usut-tuntas-kasus-temuan-senjata-demi-keamanan-pendidikan</t>
+        </is>
+      </c>
+      <c r="H1007" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/656463b7-bd6c-46b6-9ad6-409fe8b6dcb2.jpg</t>
+        </is>
+      </c>
+      <c r="I1007" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Pelanggan KA Lokal Bandung Raya Tembus 11,87 Juta, KAI Dorong Infrastruktur Berbasis Kebutuhan</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:57:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1008" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) mencatat kebutuhan masyarakat terhadap layanan kereta api di kawasan Bandung Raya ...</t>
+        </is>
+      </c>
+      <c r="F1008" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1008" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684637/pelanggan-ka-lokal-bandung-raya-tembus-1187-juta-kai-dorong-infrastruktur-berbasis-kebutuhan</t>
+        </is>
+      </c>
+      <c r="H1008" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/KA-LOKAL-BANDUNG-RAYA.jpg</t>
+        </is>
+      </c>
+      <c r="I1008" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>PLN perluas infrastruktur pengisian daya kendaraan listrik</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:56:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>PT Perusahaan Listrik Negara (Persero) atau PLN memperluas infrastruktur pengisian daya kendaraan listrik sebagai upaya ...</t>
+        </is>
+      </c>
+      <c r="F1009" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1009" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684635/pln-perluas-infrastruktur-pengisian-daya-kendaraan-listrik</t>
+        </is>
+      </c>
+      <c r="H1009" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/SPKLUGIIAS.jpg</t>
+        </is>
+      </c>
+      <c r="I1009" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Prabowo minta Bahlil Lahadalia teruskan pengabdian terbaik bagi negara</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:52:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto meminta Ketua Umum Partai Golkar sekaligus Menteri ESDM Bahlil Lahadalia untuk terus ...</t>
+        </is>
+      </c>
+      <c r="F1010" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1010" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684632/prabowo-minta-bahlil-lahadalia-teruskan-pengabdian-terbaik-bagi-negara</t>
+        </is>
+      </c>
+      <c r="H1010" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Peluncuran-10-buku-karya-nyata-untuk-negeri-Bahlil-Lahadalia-070826-Ada-1.jpg</t>
+        </is>
+      </c>
+      <c r="I1010" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Airlangga: Indonesia miliki KEK siap dimanfaatkan sektor industri</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:52:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr">
+        <is>
+          <t>Menteri Kordinator Bidang Perekonomian Airlangga Hartarto menegaskan bahwa pemerintah Indonesia memiliki Kawasan ...</t>
+        </is>
+      </c>
+      <c r="F1011" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1011" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5684629/airlangga-indonesia-miliki-kek-siap-dimanfaatkan-sektor-industri</t>
+        </is>
+      </c>
+      <c r="H1011" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_1374.jpeg</t>
+        </is>
+      </c>
+      <c r="I1011" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Otto tekankan pentingnya kewenangan dan harmonisasi dalam regulasi</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:51:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Koordinator Bidang Hukum, HAM, Imigrasi, dan Pemasyarakatan Otto Hasibuan menekankan pentingnya ...</t>
+        </is>
+      </c>
+      <c r="F1012" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1012" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684627/otto-tekankan-pentingnya-kewenangan-dan-harmonisasi-dalam-regulasi</t>
+        </is>
+      </c>
+      <c r="H1012" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000474664.jpg</t>
+        </is>
+      </c>
+      <c r="I1012" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Pemkot Cirebon lanjutkan GPM hingga akhir 2026 jaga daya beli warga</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:50:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Cirebon, Jawa Barat, memastikan program Gerakan Pangan Murah (GPM) terus dilaksanakan hingga akhir 2026 ...</t>
+        </is>
+      </c>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1013" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684624/pemkot-cirebon-lanjutkan-gpm-hingga-akhir-2026-jaga-daya-beli-warga</t>
+        </is>
+      </c>
+      <c r="H1013" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001522792.jpg</t>
+        </is>
+      </c>
+      <c r="I1013" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>12.957 Pelamar Ikuti Rekrutmen PJL KAI, Perkuat Keselamatan sekaligus Buka Kesempatan Kerja</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:49:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) melanjutkan penguatan keselamatan perlintasan sebidang melalui pemenuhan kebutuhan ...</t>
+        </is>
+      </c>
+      <c r="F1014" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1014" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684620/12957-pelamar-ikuti-rekrutmen-pjl-kai-perkuat-keselamatan-sekaligus-buka-kesempatan-kerja</t>
+        </is>
+      </c>
+      <c r="H1014" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-18.07.56.jpeg</t>
+        </is>
+      </c>
+      <c r="I1014" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>SP Palu dampingi pekerja migran Sigi terkait pelanggaran hak</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:49:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>Solidaritas Perempuan (SP) Palu mendampingi seorang pekerja migran perempuan asal Kabupaten Sigi, Sulawesi Tengah, ...</t>
+        </is>
+      </c>
+      <c r="F1015" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1015" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684619/sp-palu-dampingi-pekerja-migran-sigi-terkait-pelanggaran-hak</t>
+        </is>
+      </c>
+      <c r="H1015" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/ec28b584-1895-4c8c-a977-f88d6f01abfd.jpeg</t>
+        </is>
+      </c>
+      <c r="I1015" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Prabowo ungkap rumus bernegara dari mantan Gubernur NTT Ben Mboi</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:45:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto membagikan dua rumus penting bernegara yang diperoleh dari tokoh senior Ben Mboi untuk ...</t>
+        </is>
+      </c>
+      <c r="F1016" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1016" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684617/prabowo-ungkap-rumus-bernegara-dari-mantan-gubernur-ntt-ben-mboi</t>
+        </is>
+      </c>
+      <c r="H1016" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Peluncuran-10-buku-karya-nyata-untuk-negeri-Bahlil-Lahadalia-070826-Ada-6_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1016" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Berkas tersangka anak kasus santri terbakar dilimpahkan ke jaksa</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:45:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>Penyidik Direktorat Reserse Perlindungan Perempuan dan Anak serta Pemberantasan Perdagangan Orang Polda Nusa Tenggara ...</t>
+        </is>
+      </c>
+      <c r="F1017" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1017" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684616/berkas-tersangka-anak-kasus-santri-terbakar-dilimpahkan-ke-jaksa</t>
+        </is>
+      </c>
+      <c r="H1017" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/MG_3083.jpg</t>
+        </is>
+      </c>
+      <c r="I1017" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Bupati Manokwari: Festival Kopi Manokwari akselerasi pengembangan UMKM</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:45:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>Bupati Manokwari Hermus Indou mengatakan penyelenggaraan Festival Kopi Manokwari 2026 merupakan salah satu strategi ...</t>
+        </is>
+      </c>
+      <c r="F1018" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1018" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684615/bupati-manokwari-festival-kopi-manokwari-akselerasi-pengembangan-umkm</t>
+        </is>
+      </c>
+      <c r="H1018" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/FotoJet-2.jpg</t>
+        </is>
+      </c>
+      <c r="I1018" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Kenapa bantal tidur cepat menguning? Ini penyebabnya</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:44:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>Bantal tidur yang awalnya berwarna putih sering berubah menjadi kuning setelah digunakan dalam waktu tertentu. ...</t>
+        </is>
+      </c>
+      <c r="F1019" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1019" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684611/kenapa-bantal-tidur-cepat-menguning-ini-penyebabnya</t>
+        </is>
+      </c>
+      <c r="H1019" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/03/16/tidur_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1019" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Operasi gabungan Polda Jabar ungkap ratusan kejahatan jalanan, kendaraan dan senjata disita dari para pelaku</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:41:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>Sejumlah pelaku kejahatan jalanan dihadirkan saat rilis pengungkapan kasus kejahatan jalanan di Mapolda Jabar, Bandung, ...</t>
+        </is>
+      </c>
+      <c r="F1020" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1020" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5684607/operasi-gabungan-polda-jabar-ungkap-ratusan-kejahatan-jalanan-kendaraan-dan-senjata-disita-dari-para-pelaku</t>
+        </is>
+      </c>
+      <c r="H1020" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Rilis-pengungkapan-kasus-kejahatan-jalanan-di-Polda-Jabar-070826-NA-4.jpg</t>
+        </is>
+      </c>
+      <c r="I1020" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>BGN berhentikan 66 kepala dapur MBG atas tindakan tidak disiplin</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:40:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>Kepala Badan Gizi Nasional (BGN) Sudaryono menyatakan pihaknya telah memberhentikan 66 Sarjana Penggerak Pembangunan ...</t>
+        </is>
+      </c>
+      <c r="F1021" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1021" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684604/bgn-berhentikan-66-kepala-dapur-mbg-atas-tindakan-tidak-disiplin</t>
+        </is>
+      </c>
+      <c r="H1021" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/20260807_161317.jpg</t>
+        </is>
+      </c>
+      <c r="I1021" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Bappenas dukung Papeda Summit 2026 di Sorong</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:40:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>Kementerian Perencanaan Pembangunan Nasional/Badan Perencanaan Pembangunan Nasional (PPN/Bappenas) menyatakan dukungan ...</t>
+        </is>
+      </c>
+      <c r="F1022" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1022" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684601/bappenas-dukung-papeda-summit-2026-di-sorong</t>
+        </is>
+      </c>
+      <c r="H1022" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-3.54.43-PM.jpeg</t>
+        </is>
+      </c>
+      <c r="I1022" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>IHSG ditutup menguat ke level tertinggi tiga bulan, sinyal positif pasar saham kian menguat</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:38:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr">
+        <is>
+          <t>Pengunjung memotret layar pergerakan Indeks Harga Saham Gabungan (IHSG) di Bursa Efek Indonesia (BEI), Jakarta, ...</t>
+        </is>
+      </c>
+      <c r="F1023" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1023" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5684599/ihsg-ditutup-menguat-ke-level-tertinggi-tiga-bulan-sinyal-positif-pasar-saham-kian-menguat</t>
+        </is>
+      </c>
+      <c r="H1023" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IHSG-ditutup-menguat-65-94-poin-070826-Fah-1.jpg</t>
+        </is>
+      </c>
+      <c r="I1023" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Menpora dukung promotor hadirkan laga pramusim di Indonesia</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:38:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>Menteri Pemuda dan Olahraga Erick Thohir mendukung pihak perusahaan-perusahaan promotor swasta untuk menghadirkan laga ...</t>
+        </is>
+      </c>
+      <c r="F1024" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1024" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684596/menpora-dukung-promotor-hadirkan-laga-pramusim-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H1024" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/aston-villa-menang-atas-indonesia-all-stars-2832201.jpg</t>
+        </is>
+      </c>
+      <c r="I1024" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>Pemprov dorong SBI optimalkan produksi semen penuhi kebutuhan Aceh</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:37:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1025" t="inlineStr">
+        <is>
+          <t>Pemerintah Aceh mendorong PT Solusi Bangun Indonesia (SBI) melalui anak perusahaannya PT Solusi Bangun Andalas (SBA) ...</t>
+        </is>
+      </c>
+      <c r="F1025" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1025" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684593/pemprov-dorong-sbi-optimalkan-produksi-semen-penuhi-kebutuhan-aceh</t>
+        </is>
+      </c>
+      <c r="H1025" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG-20260807-WA0022.jpg</t>
+        </is>
+      </c>
+      <c r="I1025" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>114 Dapur MBG di Papua hingga NTT Akan Beroperasi Pekan Depan</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:27:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E1026" t="inlineStr">
+        <is>
+          <t>BGN akan mengaktifkan 114 dapur MBG pekan depan. Dapur tersebut tersebar di sejumlah wilayah, termasuk Papua, Nusa Tenggara Timur (NTT), dan Maluku.</t>
+        </is>
+      </c>
+      <c r="F1026" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1026" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609046/114-dapur-mbg-di-papua-hingga-ntt-akan-beroperasi-pekan-depan</t>
+        </is>
+      </c>
+      <c r="H1026" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/kepala-bgn-sudaryono-brigittadetikcom-1786101809094_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1026" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Bima Arya Dorong Penghijauan Jadi Gerakan Berkelanjutan di Daerah</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:09:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E1027" t="inlineStr">
+        <is>
+          <t>Wamendagri Bima Arya dorong Pemda untuk penghijauan berkelanjutan. Kolaborasi lintas sektor penting untuk keberhasilan rehabilitasi hutan dan lahan.</t>
+        </is>
+      </c>
+      <c r="F1027" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1027" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609032/bima-arya-dorong-penghijauan-jadi-gerakan-berkelanjutan-di-daerah</t>
+        </is>
+      </c>
+      <c r="H1027" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/wakil-menteri-dalam-negeri-wamendagri-bima-arya-sugiarto-1786104463489.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1027" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Menilik Ruangan Ditemukan Senjata di Sekolah Swasta Jaksel, Kini Digaris Polisi</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:09:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>Taufiq Syarifudin</t>
+        </is>
+      </c>
+      <c r="E1028" t="inlineStr">
+        <is>
+          <t>Sekolah swasta di Pondok Pinang, Jakarta Selatan dihebohkan karena ditemukan 995 senjata. Kini ruangan tersebut digaris polisi.</t>
+        </is>
+      </c>
+      <c r="F1028" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1028" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609029/menilik-ruangan-ditemukan-senjata-di-sekolah-swasta-jaksel-kini-digaris-polisi</t>
+        </is>
+      </c>
+      <c r="H1028" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/ruangan-mantan-kepala-yayasan-ditemukannya-senjata-di-sekolah-swasta-jaksel-taufiqdetikcom-1786104460641_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1028" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Solusi 4C Lintasarta Bantu Bank Daerah Kebut Transformasi Digital</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:07:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>Annisa Sekar Melati</t>
+        </is>
+      </c>
+      <c r="E1029" t="inlineStr">
+        <is>
+          <t>Bank Pembangunan Daerah didorong untuk percepat transformasi digital guna tingkatkan layanan dan peran ekonomi.</t>
+        </is>
+      </c>
+      <c r="F1029" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1029" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609026/solusi-4c-lintasarta-bantu-bank-daerah-kebut-transformasi-digital</t>
+        </is>
+      </c>
+      <c r="H1029" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/lintasarta-cxo-bpd-summit-2026-1786016739700_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1029" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>Kebakaran di Suryakencana Gunung Gede Capai 1 Hektar, 5 Meter dari Taman Edelweiss</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:57:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>Muchamad Sholihin</t>
+        </is>
+      </c>
+      <c r="E1030" t="inlineStr">
+        <is>
+          <t>Kebakaran di alun-alun Suryakencana Gunung Gede melanda area seluas 1 hektar. Lokasi kebakaran hanya berjarak 5 meter dari Taman Edelweiss.</t>
+        </is>
+      </c>
+      <c r="F1030" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1030" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609008/kebakaran-di-suryakencana-gunung-gede-capai-1-hektar-5-meter-dari-taman-edelweiss</t>
+        </is>
+      </c>
+      <c r="H1030" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/gunung-gede-pangrango-kebakaran-1786025219821_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1030" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Lintasarta Dorong Bank Daerah Tingkatkan Ketahanan Siber dan AI</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:57:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E1031" t="inlineStr">
+        <is>
+          <t>Lintasarta dan ASBANDA tandatangani MoU di CxO BPD Summit 2026 untuk transformasi digital BPD, fokus pada ketahanan siber dan pemanfaatan AI.</t>
+        </is>
+      </c>
+      <c r="F1031" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1031" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609007/lintasarta-dorong-bank-daerah-tingkatkan-ketahanan-siber-dan-ai</t>
+        </is>
+      </c>
+      <c r="H1031" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/lintasarta-cxo-bpd-summit-2026-1786016739700.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1031" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>Polisi Sebut Ada Pihak Sengaja Pesan Konten Hoax: Berpotensi Gaduh!</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:53:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E1032" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya ungkap kasus penyebaran konten hoax di medsos. 28 orang diamankan, 10 diproses hukum. Polisi imbau masyarakat bijak menggunakan medsos.</t>
+        </is>
+      </c>
+      <c r="F1032" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1032" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609004/polisi-sebut-ada-pihak-sengaja-pesan-konten-hoax-berpotensi-gaduh</t>
+        </is>
+      </c>
+      <c r="H1032" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/dirkrimum-polda-metro-jaya-kombes-iman-imanuddin-1786096322096_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1032" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>BGN Pecat 66 Kepala Dapur MBG, Terlibat Judol hingga 'Hengki Pengki'</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:49:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E1033" t="inlineStr">
+        <is>
+          <t>BGN memproses pemecatan 66 kepala dapur MBG yang melakukan pelanggaran. Pelanggarannya ada yang terlibat judi online hingga 'hengki pengki'.</t>
+        </is>
+      </c>
+      <c r="F1033" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1033" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609001/bgn-pecat-66-kepala-dapur-mbg-terlibat-judol-hingga-hengki-pengki</t>
+        </is>
+      </c>
+      <c r="H1033" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/27/tancap-gas-kepala-bgn-sudaryono-pecat-261-pegawai-bermasalah-1785138053252_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1033" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Prabowo Ultimatum Kepala Daerah: Tak Bisa Penuhi Teriakan Rakyat, Presiden Turun Tangan</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:42:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>Eva Safitri</t>
+        </is>
+      </c>
+      <c r="E1034" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo memberi ultimatum kepada kepala daerah untuk memenuhi kebutuhan rakyat. Jika tidak, pemerintah pusat akan turun tangan membangun infrastruktur.</t>
+        </is>
+      </c>
+      <c r="F1034" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1034" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8608989/prabowo-ultimatum-kepala-daerah-tak-bisa-penuhi-teriakan-rakyat-presiden-turun-tangan</t>
+        </is>
+      </c>
+      <c r="H1034" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/prabowo-subianto-evadetikcom-1786092746269_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1034" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Luhut Cerita Dulu RI Ditertawakan soal Nikel, Kini Dunia Datang Investasi</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:30:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E1035" t="inlineStr">
+        <is>
+          <t>Luhut Binsar Pandjaitan membahas larangan ekspor biji nikel yang menuai kritik.</t>
+        </is>
+      </c>
+      <c r="F1035" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1035" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8608990/luhut-cerita-dulu-ri-ditertawakan-soal-nikel-kini-dunia-datang-investasi</t>
+        </is>
+      </c>
+      <c r="H1035" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/24/ketua-dewan-ekonomi-nasional-den-luhut-binsar-pandjaitan-1782274037708_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1035" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>Freeport Mundurkan Produksi Tambang Kucing Liar ke 2029</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:00:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>PT Freeport Indonesia memastikan produksi tambang Kucing Liar di Grasberg mundur ke 2029. Perpanjangan izin usaha juga diajukan untuk kelangsungan operasional.</t>
+        </is>
+      </c>
+      <c r="F1036" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1036" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8608967/freeport-mundurkan-produksi-tambang-kucing-liar-ke-2029</t>
+        </is>
+      </c>
+      <c r="H1036" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/presiden-direktur-pt-freeport-indonesia-ptfi-tony-wenas-1786101675207_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1036" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>Kekecewaan Pihak Asisten Nikita Mirzani, Sidang PK TPPU Ditunda</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:08:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>Ismail Marzuki, asisten Nikita Mirzani, ajukan Peninjauan Kembali atas dugaan pemerasan dan TPPU. Sidang perdana digelar di Jakarta Selatan.</t>
+        </is>
+      </c>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1037" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8608627/kekecewaan-pihak-asisten-nikita-mirzani-sidang-pk-tppu-ditunda</t>
+        </is>
+      </c>
+      <c r="H1037" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/07/24/nikita-mirzani-jalani-sidang-ttpu-1753328999013_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1037" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Pihak Sekolah di Jaksel Klarifikasi, Bunker Sudah Diperiksa Polisi</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:33:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>Pihak sekolah swasta di Jakarta memastikan bunker yang diduga menyimpan senjata telah diperiksa polisi. Ratusan senjata dan narkoba ditemukan di lokasi.</t>
+        </is>
+      </c>
+      <c r="F1038" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1038" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807182957-12-1389874/pihak-sekolah-di-jaksel-klarifikasi-bunker-sudah-diperiksa-polisi</t>
+        </is>
+      </c>
+      <c r="H1038" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/ratusan-senjata-di-yayasan-sekolah-jaksel-1786100090384_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1038" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>Kapolresta dan Kasat Narkoba Banda Aceh Masih Diperiksa di Mabes Polri</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:29:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>Kapolresta Banda Aceh dan Kasat Resnarkoba diperiksa Propam Mabes Polri. Proses dilakukan transparan dan profesional, menunggu hasil resmi untuk publik.</t>
+        </is>
+      </c>
+      <c r="F1039" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1039" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807191947-12-1389914/kapolresta-dan-kasat-narkoba-banda-aceh-masih-diperiksa-di-mabes-polri</t>
+        </is>
+      </c>
+      <c r="H1039" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/09/03/pengamanan-sidang-etik-penabrak-sopir-ojek-daring-di-tncc-polri-1756878770745_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1039" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Polda Metro Tindak 28 Pegiat Medsos Sebar Provokasi-Hoaks, 9 Tersangka</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:08:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya menindak 28 pegiat medsos terkait penyebaran hoaks. Sembilan orang ditetapkan sebagai tersangka, sementara 30 konten telah diturunkan.</t>
+        </is>
+      </c>
+      <c r="F1040" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1040" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807185640-12-1389889/polda-metro-tindak-28-pegiat-medsos-sebar-provokasi-hoaks-9-tersangka</t>
+        </is>
+      </c>
+      <c r="H1040" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/09/12/ilustrasi-hacker-ilustrasi-serangan-siber-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1040" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Penampakan Ruang Penyimpanan Ratusan Senjata di Yayasan Sekolah</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:56:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>Penampakan dua ruangan yang ditemukan ratusan senjata dan narkoba di salah satu sekolah swasta di Pondok Pinang, Jaksel, Jumat (7/8).</t>
+        </is>
+      </c>
+      <c r="F1041" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1041" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807182953-16-1389873/penampakan-ruang-penyimpanan-ratusan-senjata-di-yayasan-sekolah</t>
+        </is>
+      </c>
+      <c r="H1041" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/penampakan-ruangan-penyimpanan-ratusan-senjata-di-sekolah-jaksel-1786102460839_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1041" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Kebakaran di Alun-alun Suryakencana Gunung Gede Sudah Padam</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:45:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>Kebakaran lahan di Alun-Alun Suryakencana, Taman Nasional Gunung Gede Pangrango, berhasil dikendalikan. Penyebab kebakaran masih dalam penyelidikan.</t>
+        </is>
+      </c>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1042" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807173650-20-1389877/kebakaran-di-alun-alun-suryakencana-gunung-gede-sudah-padam</t>
+        </is>
+      </c>
+      <c r="H1042" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/bb-tnggp-tutup-jalur-pendakian-karena-kebakaran-alun-alun-suryakancana-1786099073263_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1042" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>30 Puisi Cinta Romantis yang Menyentuh Hati, Penuh Makna tentang Rindu dan Kesetiaan</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:33:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>Puisi cinta menjadi salah satu cara indah untuk mengungkapkan perasaan yang sulit disampaikan melalui kata-kata biasa, inilah 30 puisi cinta romantis.</t>
+        </is>
+      </c>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1043" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865458/30-puisi-cinta-romantis-yang-menyentuh-hati-penuh-makna-tentang-rindu-dan-kesetiaan</t>
+        </is>
+      </c>
+      <c r="H1043" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/oex3nTadQ4mlr7fG6Zffxm4z76U=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Promo-Valentine-Day-di-Georgia-Florist-Semarang_20250131_152414.jpg</t>
+        </is>
+      </c>
+      <c r="I1043" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>Susy Susanti Perluas Pembinaan Olahraga, Bisbol Jadi Program Baru ASNA Academy</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:29:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1044" t="inlineStr">
+        <is>
+          <t>Susy mengatakan Jepang dipilih karena memiliki sistem pembinaan bisbol yang matang dan pengalaman panjang dalam mencetak atlet berprestasi.</t>
+        </is>
+      </c>
+      <c r="F1044" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1044" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865457/susy-susanti-perluas-pembinaan-olahraga-bisbol-jadi-program-baru-asna-academy</t>
+        </is>
+      </c>
+      <c r="H1044" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tnYIWXvBd7AMdDkD6BtsjG5l6lI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Legenda-pebulutangkis-Indonesia-Susy-Susanti-dan-Alan-Budikusuma-2121.jpg</t>
+        </is>
+      </c>
+      <c r="I1044" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>Wujud Kolaborasi JKN dan Pemda dari 0 KM Indonesia: Peresmian Taman Budaya Gotong Royong di Sabang</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:28:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1045" t="inlineStr">
+        <is>
+          <t>Taman Budaya Gotong Royong mencerminkan falsafah luhur Indonesia yang menjadi fondasi penyelenggaraan Program JKN.</t>
+        </is>
+      </c>
+      <c r="F1045" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1045" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865456/wujud-kolaborasi-jkn-dan-pemda-dari-0-km-indonesia-peresmian-taman-budaya-gotong-royong-di-sabang</t>
+        </is>
+      </c>
+      <c r="H1045" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/7TC5Iu6tiadTOpohRO-WVzndXEE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/eresmikan-Taman-Budaya-Gotong-Royong-dan-Prasasti-INISIATIF-BPJS-Kesehatan.jpg</t>
+        </is>
+      </c>
+      <c r="I1045" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>SUV 7-Seater yang Wajib Anda Test Drive di GIIAS 2026, dari New XL7 Hybrid Sampai Eksion PHEV</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:28:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1046" t="inlineStr">
+        <is>
+          <t>Pameran otomotif GIIAS 2026 menawarkan puluhan kendaraan model terbaru dari berbagai kategori dan powertrain untuk di-test drive pengunjung</t>
+        </is>
+      </c>
+      <c r="F1046" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1046" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865455/suv-7-seater-yang-wajib-anda-test-drive-di-giias-2026-dari-new-xl7-hybrid-sampai-eksion-phev</t>
+        </is>
+      </c>
+      <c r="H1046" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/oHHLc5CsdCHeaXW6QiTw-8hNplM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/XL7-Hybrid-di-pameran-GIIAS-2026-BSD-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I1046" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>Susunan Pemain Timnas Indonesia vs Singapura: Cahya Gantikan Nadeo, Jordi Amat Diistirahatkan</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:28:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1047" t="inlineStr">
+        <is>
+          <t>Starting XI Timnas Indonesia vs Singapura resmi dirilis. John Herdman merotasi kiper dan lini belakang demi Garuda lolos ke semifinal Piala AFF 2026.</t>
+        </is>
+      </c>
+      <c r="F1047" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1047" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865454/susunan-pemain-timnas-indonesia-vs-singapura-cahya-gantikan-nadeo-jordi-amat-diistirahatkan</t>
+        </is>
+      </c>
+      <c r="H1047" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/yNQRBwgJz2YPPsUobmy3fY0wL6Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Piala-AFF-2026-Timnas-Indonesia-Tekuk-Timor-Leste-3-0_20260731_231927.jpg</t>
+        </is>
+      </c>
+      <c r="I1047" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>Misi Ussy Sulistiawaty di Event Lari 10K Bareng Suami: Harus Bisa Sejajar dan Happy</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:27:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1048" t="inlineStr">
+        <is>
+          <t>Sebagai pelari yang lebih terbiasa, Ussy harus menahan kecepatan larinya agar Andhika bisa berlari sejajar dengannya dan tidak ngos-ngosan.</t>
+        </is>
+      </c>
+      <c r="F1048" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1048" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865453/misi-ussy-sulistiawaty-di-event-lari-10k-bareng-suami-harus-bisa-sejajar-dan-happy</t>
+        </is>
+      </c>
+      <c r="H1048" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5VzrzJf_FTWayAtjNEkYAwmZK70=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ussy-Sulistiawaty-1-07082026.jpg</t>
+        </is>
+      </c>
+      <c r="I1048" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>Persaingan Memanas, 18 Atlet Berebut Super Tiket Audisi PB Djarum di Makassar</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:26:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1049" t="inlineStr">
+        <is>
+          <t>Hingga Jumat (7/8/2026), sebanyak 18 atlet tersisa dan akan memperebutkan tiket menuju tahap berikutnya di GOR Dafest Makassar</t>
+        </is>
+      </c>
+      <c r="F1049" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1049" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865452/persaingan-memanas-18-atlet-berebut-super-tiket-audisi-pb-djarum-di-makassar</t>
+        </is>
+      </c>
+      <c r="H1049" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/QvZlTzRm1f76ec7JobnUNgsVr2s=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Super-Tiket-pada-Audisi-Umum-PB-Djarum-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I1049" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>Istana Tak Mau Komentari Soal Nobel MBG: Pemerintah Fokus Jalankan Program</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:21:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1050" t="inlineStr">
+        <is>
+          <t>Pras enggan mengomentari dugaan adanya pencatutan nama presiden dalam makalah MBG yang disebut untuk dinominasikan dalam Nobel Perdamaian 2026.</t>
+        </is>
+      </c>
+      <c r="F1050" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1050" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865451/istana-tak-mau-komentari-soal-nobel-mbg-pemerintah-fokus-jalankan-program</t>
+        </is>
+      </c>
+      <c r="H1050" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hH7V60ix95CcR0SInm1prH87c_M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Prasetyo-Hadi-di-Wisma-Negara-Komplek-Istana-07082026.jpg</t>
+        </is>
+      </c>
+      <c r="I1050" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>Kepala BGN Sampaikan Permintaan Maaf Terbuka ke Keluarga Korban Keracunan MBG di Papua Hingga Jogja</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:21:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1051" t="inlineStr">
+        <is>
+          <t>Sudaryono menyampaikan permohonan maaf secara terbuka kepada seluruh korban dan pihak keluarga atas insiden keracunan Program MBG.</t>
+        </is>
+      </c>
+      <c r="F1051" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1051" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865450/kepala-bgn-sampaikan-permintaan-maaf-terbuka-ke-keluarga-korban-keracunan-mbg-di-papua-hingga-jogja</t>
+        </is>
+      </c>
+      <c r="H1051" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Y5lgDd3Odghq_xVmdEJ68vikNT0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Konferensi-Pers-Kepala-BGN-Sudaryono_20260727_165349.jpg</t>
+        </is>
+      </c>
+      <c r="I1051" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>Menpora Erick: Indonesia Makin Diminati sebagai Lokasi  Pramusim Internasional, Ini Sinyal Positif</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:20:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1052" t="inlineStr">
+        <is>
+          <t>Tren tersebut menjadi tanda bahwa atmosfer sepak bola dan industri olahraga Indonesia makin mendapat pengakuan dunia.</t>
+        </is>
+      </c>
+      <c r="F1052" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1052" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865449/menpora-erick-indonesia-makin-diminati-sebagai-lokasi-pramusim-internasional-ini-sinyal-positif</t>
+        </is>
+      </c>
+      <c r="H1052" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/gtfZaVm82NqrBbI30YP2j6YmRJk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Menpora-Erick-Thohir-087082026.jpg</t>
+        </is>
+      </c>
+      <c r="I1052" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>Bertemu KBPBI, Kapolri Minta Pengawalan RUU Ketenagakerjaan Utamakan Dialog</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:19:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1053" t="inlineStr">
+        <is>
+          <t>Kapolri siap menjembatani komunikasi, sementara KBPBI menegaskan aksi tetap dapat digelar jika aspirasi buruh tidak diakomodasi.</t>
+        </is>
+      </c>
+      <c r="F1053" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1053" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865448/bertemu-kbpbi-kapolri-minta-pengawalan-ruu-ketenagakerjaan-utamakan-dialog</t>
+        </is>
+      </c>
+      <c r="H1053" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GtD3aVR0q9O9I-gdav41_WOa_jg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/BURUH-KBPBI-kapolri-ruu-ketenagakerjaan.jpg</t>
+        </is>
+      </c>
+      <c r="I1053" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>Hubungan Maverick Vinales dan KTM Memanas, Bos Tech3 Sebut Semua Berawal dari Cedera Bahu</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:17:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1054" t="inlineStr">
+        <is>
+          <t>Masa depan Maverick Vinales di MotoGP 2027 semakin tidak menentu setelah cedera bahunya belum pulih serta bos Tech3 belum ada kepastian.</t>
+        </is>
+      </c>
+      <c r="F1054" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1054" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865447/hubungan-maverick-vinales-dan-ktm-memanas-bos-tech3-sebut-semua-berawal-dari-cedera-bahu</t>
+        </is>
+      </c>
+      <c r="H1054" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/M0XoOEGeMji8fIWColfmIdcSwHw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Vinales-vs-Marquez-di-Qatar.jpg</t>
+        </is>
+      </c>
+      <c r="I1054" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>Pakar Dorong Pembenahan Tata Kelola agar Program MBG Lebih Efektif</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:14:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1055" t="inlineStr">
+        <is>
+          <t>Tata kelola transparan hingga pengawasan yang efektif dinilai akan menjadi faktor penentu agar manfaat program dapat dirasakan secara lebih luas</t>
+        </is>
+      </c>
+      <c r="F1055" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1055" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865446/pakar-dorong-pembenahan-tata-kelola-agar-program-mbg-lebih-efektif</t>
+        </is>
+      </c>
+      <c r="H1055" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Kxy0Y85qxTHxMbNcepFDroLjqqk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/food-tray-mbg-2kf.jpg</t>
+        </is>
+      </c>
+      <c r="I1055" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>Denda Parkir Ribuan Kendaraan Diplomatik di Jepang Kedaluwarsa, RI Catat 17 Pelanggaran</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:13:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1056" t="inlineStr">
+        <is>
+          <t>Ribuan denda parkir kendaraan diplomatik di Jepang kedaluwarsa dan tak tertagih. Pada 2025, kendaraan Kedubes RI tercatat 17 pelanggaran</t>
+        </is>
+      </c>
+      <c r="F1056" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1056" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865445/denda-parkir-ribuan-kendaraan-diplomatik-di-jepang-kedaluwarsa-ri-catat-17-pelanggaran</t>
+        </is>
+      </c>
+      <c r="H1056" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hTSTaO0V0mpADmjQriiCCQZuRMw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kedubesindonesidijepang1.jpg</t>
+        </is>
+      </c>
+      <c r="I1056" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>30 Ucapan Hari Singa Sedunia 2026 Inspiratif, Penuh Makna tentang Konservasi dan Cinta Satwa Liar</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:13:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1057" t="inlineStr">
+        <is>
+          <t>Hari Singa Sedunia atau World Lion Day diperingati setiap tanggal 10 Agustus, inilah 30 ucapan Hari Singa Sedunia 2026 yang inspiratif, penuh makna.</t>
+        </is>
+      </c>
+      <c r="F1057" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1057" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865444/30-ucapan-hari-singa-sedunia-2026-inspiratif-penuh-makna-tentang-konservasi-dan-cinta-satwa-liar</t>
+        </is>
+      </c>
+      <c r="H1057" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/BAmz7J7p3S7BTrCYYvpJ6GyzyVQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/singa-mati-kepanasan-di-jepang.jpg</t>
+        </is>
+      </c>
+      <c r="I1057" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>Kepala BGN Siapkan Sanksi Suspend Permanen Bagi Dapur MBG Penyebab Siswa Keracunan</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:12:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1058" t="inlineStr">
+        <is>
+          <t>BGN menerapkan kebijakan sanksi hingga penutupan permanen bagi fasilitas dapur penyedia MBG yang terbukti menjadi penyebab siswa keracunan.</t>
+        </is>
+      </c>
+      <c r="F1058" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1058" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865443/kepala-bgn-siapkan-sanksi-suspend-permanen-bagi-dapur-mbg-penyebab-siswa-keracunan</t>
+        </is>
+      </c>
+      <c r="H1058" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/4f0-zgr4hrnVHPQgVmsf_X-PPFM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Konferensi-Pers-Kepala-BGN-Sudaryono_20260727_163650.jpg</t>
+        </is>
+      </c>
+      <c r="I1058" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>BGN Bakal Aktivasi 114 Dapur MBG di Papua dan Wilayah 3T Pekan Depan</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:03:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1059" t="inlineStr">
+        <is>
+          <t>BGN bersiap mengaktivasi 114 fasilitas dapur penyedia Makan Bergizi Gratis (MBG) di wilayah Papua, Maluku, NTT, dan kawasan 3T pekan depan</t>
+        </is>
+      </c>
+      <c r="F1059" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1059" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865442/bgn-bakal-aktivasi-114-dapur-mbg-di-papua-dan-wilayah-3t-pekan-depan</t>
+        </is>
+      </c>
+      <c r="H1059" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/lTxA0XNqqRXLEstPwFl6NIDq18E=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/dapur-mbg2.jpg</t>
+        </is>
+      </c>
+      <c r="I1059" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>Trofi Piala AFF 2026 Sudah di Indonesia, Mampukah Skuad Garuda Membawanya Pulang?</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:02:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1060" t="inlineStr">
+        <is>
+          <t>Di area pameran, trofi ASEAN Hyundai Cup 2026 ditempatkan bersama sejumlah atribut turnamen.</t>
+        </is>
+      </c>
+      <c r="F1060" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1060" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865441/trofi-piala-aff-2026-sudah-di-indonesia-mampukah-skuad-garuda-membawanya-pulang</t>
+        </is>
+      </c>
+      <c r="H1060" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/htpzVdF_nAm8PPuQyKT3HfjGvgA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Trofi-ASEAN-Hyundai-Cup-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I1060" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>Perang AS-Iran Diyakini Akan Berakhir, Trump Klaim Teheran Tak Mampu Bertahan karena Pasokan Senjata</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1061" t="inlineStr">
+        <is>
+          <t>Menurut Trump, Iran tidak akan mampu bertahan lebih lama lagi atas perangnya melawan AS.</t>
+        </is>
+      </c>
+      <c r="F1061" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1061" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865440/perang-as-iran-diyakini-akan-berakhir-trump-klaim-teheran-tak-mampu-bertahan-karena-pasokan-senjata</t>
+        </is>
+      </c>
+      <c r="H1061" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zAJrXAtbprOaJvloF4HTWYbFg8I=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/DONALD-TRUMP-SAAT-BERPIDATO-DI-MICHIGAN-27072026.jpg</t>
+        </is>
+      </c>
+      <c r="I1061" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>Wamendagri Bima Arya Ajak Pemda jadikan Penghijauan sebagai Gerakan Berkelanjutan</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:59:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1062" t="inlineStr">
+        <is>
+          <t>Upaya rehabilitasi hutan dan lahan tidak berhenti pada penanaman pohon, tetapi perlu disertai perawatan serta kolaborasi berbagai pihak.</t>
+        </is>
+      </c>
+      <c r="F1062" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1062" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865439/wamendagri-bima-arya-ajak-pemda-jadikan-penghijauan-sebagai-gerakan-berkelanjutan</t>
+        </is>
+      </c>
+      <c r="H1062" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/7rBNuGGRJqMvbBXFZcThMh-3C10=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/peresmian-Pusat-Persemaian-Sriwijaya-Kemampo.jpg</t>
+        </is>
+      </c>
+      <c r="I1062" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>BGN Pecat 66 Kepala Dapur MBG, Ada yang Terjerat Judi Online</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:23:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1063" t="inlineStr">
+        <is>
+          <t>BGN memproses pemecatan tidak hormat 66 kepala dapur MBG akibat berbagai pelanggaran disiplin.</t>
+        </is>
+      </c>
+      <c r="F1063" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1063" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264599/bgn-pecat-66-kepala-dapur-mbg-ada-yang-terjerat-judi-online</t>
+        </is>
+      </c>
+      <c r="H1063" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/ugc3f_O3CnjjEQV-fkElBMb_n8k=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318578/original/016581600_1786105434-IMG_20260807_163305_363.jpg</t>
+        </is>
+      </c>
+      <c r="I1063" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>Akun X TMC Polda Metro Jaya Diretas</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:51:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1064" t="inlineStr">
+        <is>
+          <t>Upaya pemulihan masih terus dilakukan.</t>
+        </is>
+      </c>
+      <c r="F1064" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1064" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264565/akun-x-tmc-polda-metro-jaya-diretas</t>
+        </is>
+      </c>
+      <c r="H1064" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/KW2ZVGQIcI9JdIS1ziu4gBEJQnI=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318551/original/094695300_1786103501-Screenshot_2026-08-07_184037.jpg</t>
+        </is>
+      </c>
+      <c r="I1064" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>John Herdman: Piala AFF 2026 Bagian dari Misi Menuju Piala Dunia 2030</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:42:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1065" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia punya dahaga gelar di Piala AFF 2026, mampukan tim asuhan John Herdman yang mematahkan kutukan tak pernah juara?</t>
+        </is>
+      </c>
+      <c r="F1065" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1065" t="inlineStr">
+        <is>
+          <t>https://bola.kompas.com/read/2026/08/07/19420528/john-herdman-piala-aff-2026-bagian-dari-misi-menuju-piala-dunia-2030</t>
+        </is>
+      </c>
+      <c r="H1065" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/DicUUyMV1n5ZSZ_B0wj7jj2KNk4=/0x0:2265x1510/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/07/18/6a5b175b0ade3.jpg</t>
+        </is>
+      </c>
+      <c r="I1065" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>Susunan Pemain Timnas Indonesia Vs Singapura: Herdman Mainkan Cahya dan Wahyu Prasetyo</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:42:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1066" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia wajib menang di laga ini jika ingin melangkahkan kakinya ke fase gugur Piala AFF 2026.</t>
+        </is>
+      </c>
+      <c r="F1066" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1066" t="inlineStr">
+        <is>
+          <t>https://bola.kompas.com/read/2026/08/07/19264738/susunan-pemain-timnas-indonesia-vs-singapura-herdman-mainkan-cahya-dan-wahyu</t>
+        </is>
+      </c>
+      <c r="H1066" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/BaeTjmZDOImSvWBkCx8pX6BsXB0=/2x65:1473x1046/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/07/31/6a6c926a79508.png</t>
+        </is>
+      </c>
+      <c r="I1066" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>Di Balik Gang Sempit Cakung Jaktim, Ada Sawah dan Kebun Menghidupi Warga</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:42:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>Di tengah hiruk pikuk Jakarta, hamparan sawah hijau masih lestari di Cakung. Kisah sukses Kelompok Tani Baliku Lestari menjaga ruang hijau dan pangan kota.</t>
+        </is>
+      </c>
+      <c r="F1067" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1067" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/07/19082041/di-balik-gang-sempit-cakung-jaktim-ada-sawah-dan-kebun-menghidupi-warga</t>
+        </is>
+      </c>
+      <c r="H1067" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/wB7kW-1ZixJn0p5npsP0jfXwk7o=/266x513:4032x3024/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/07/6a75c9cda024b.jpeg</t>
+        </is>
+      </c>
+      <c r="I1067" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I987"/>
+  <autoFilter ref="A1:I1067"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 15:47 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-07.xlsx
+++ b/data/berita_2026-08-07.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1295</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1191"/>
+  <dimension ref="A1:I1295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -56410,8 +56410,4896 @@
         </is>
       </c>
     </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>Suzuki ramaikan persaingan mobil irit BBM di segmen LSUV</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:37:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E1192" t="inlineStr">
+        <is>
+          <t>Persaingan di industri otomotif segmen Low Sport Utility Vehicle (LSUV) di Indonesia, semakin menunjukkan keseriusannya ...</t>
+        </is>
+      </c>
+      <c r="F1192" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1192" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5685115/suzuki-ramaikan-persaingan-mobil-irit-bbm-di-segmen-lsuv</t>
+        </is>
+      </c>
+      <c r="H1192" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-07-31-at-09.15.48.jpeg</t>
+        </is>
+      </c>
+      <c r="I1192" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>Kongres MGBKGI di Unhas fokus perkuat riset berdampak</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:35:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1193" t="inlineStr">
+        <is>
+          <t>Universitas Hasanuddin (Unhas) menggelar kongres perdana Majelis Guru Besar Kedokteran Gigi Indonesia (MGBKGI) yang ...</t>
+        </is>
+      </c>
+      <c r="F1193" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1193" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685109/kongres-mgbkgi-di-unhas-fokus-perkuat-riset-berdampak</t>
+        </is>
+      </c>
+      <c r="H1193" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG-20260807-WA0064.jpg</t>
+        </is>
+      </c>
+      <c r="I1193" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>Pemprov beri 20 hektare, minta Mensos tambah Sekolah Rakyat di Sulsel</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:35:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1194" t="inlineStr">
+        <is>
+          <t>Gubernur Sulawesi Selatan (Sulsel) Andi Sudirman Sulaiman meminta kepada Menteri Sosial Saifullah Yusuf (Gus Ipul) ...</t>
+        </is>
+      </c>
+      <c r="F1194" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1194" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685108/pemprov-beri-20-hektare-minta-mensos-tambah-sekolah-rakyat-di-sulsel</t>
+        </is>
+      </c>
+      <c r="H1194" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/download.jpg</t>
+        </is>
+      </c>
+      <c r="I1194" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>RealCo: Hilirisasi sarang walet buka peluang nilai tambah ekspor RI</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:34:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1195" t="inlineStr">
+        <is>
+          <t>CEO PT Abadi Lestari Indonesia Tbk (RealCo) Edwin Pranata menilai hilirisasi sarang burung walet (SBW) dapat ...</t>
+        </is>
+      </c>
+      <c r="F1195" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1195" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685104/realco-hilirisasi-sarang-walet-buka-peluang-nilai-tambah-ekspor-ri</t>
+        </is>
+      </c>
+      <c r="H1195" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000178490.jpg</t>
+        </is>
+      </c>
+      <c r="I1195" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>Muktamar XI Himi Persis tegaskan transformasi gerakan bangun peradaban</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:27:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1196" t="inlineStr">
+        <is>
+          <t>Himpunan Mahasiswi Persatuan Islam (Himi Persis) menggelar Muktamar XI di Gedung PPSDM Kemendikdasmen, Depok, pada 7-9 ...</t>
+        </is>
+      </c>
+      <c r="F1196" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1196" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685100/muktamar-xi-himi-persis-tegaskan-transformasi-gerakan-bangun-peradaban</t>
+        </is>
+      </c>
+      <c r="H1196" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000177104.jpg</t>
+        </is>
+      </c>
+      <c r="I1196" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>Marco Palestra yakin Chelsea jalani musim hebat bersama Alonso</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:25:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1197" t="inlineStr">
+        <is>
+          <t>Pemain rekrutan baru Chelsea Marco Palestra meyakini Chelsea akan menjalani musim kompetisi yang hebat di bawah asuhan ...</t>
+        </is>
+      </c>
+      <c r="F1197" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1197" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685099/marco-palestra-yakin-chelsea-jalani-musim-hebat-bersama-alonso</t>
+        </is>
+      </c>
+      <c r="H1197" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_20260807_220403.jpg</t>
+        </is>
+      </c>
+      <c r="I1197" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>Berkat bantuan kewirausahaan Kemensos, Oneng stop mengemis</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:25:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1198" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1198" t="inlineStr">
+        <is>
+          <t>Eks pengemis di Kota Bandung, Oneng, kini berhasil alih profesi menjadi penjual kopi dan aneka minuman di warung berkat ...</t>
+        </is>
+      </c>
+      <c r="F1198" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1198" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685096/berkat-bantuan-kewirausahaan-kemensos-oneng-stop-mengemis</t>
+        </is>
+      </c>
+      <c r="H1198" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-20.41.19.jpeg</t>
+        </is>
+      </c>
+      <c r="I1198" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>LPSK: Pembayaran restitusi korban TPKS baru Rp87,69 juta</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:24:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1199" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1199" t="inlineStr">
+        <is>
+          <t>Lembaga Pelindungan Saksi dan Korban (LPSK) mencatat realisasi pembayaran restitusi oleh pelaku tindak pidana kekerasan ...</t>
+        </is>
+      </c>
+      <c r="F1199" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1199" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685092/lpsk-pembayaran-restitusi-korban-tpks-baru-rp8769-juta</t>
+        </is>
+      </c>
+      <c r="H1199" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001224422.jpg</t>
+        </is>
+      </c>
+      <c r="I1199" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>Indonesia bermain imbang 1-1 kontra Singapura</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:24:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1200" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1200" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia bermain imbang dengan skor 1-1 kontra Timnas Singapura pada pertandingan Grup A Piala AFF 2026 di ...</t>
+        </is>
+      </c>
+      <c r="F1200" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1200" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685091/indonesia-bermain-imbang-1-1-kontra-singapura</t>
+        </is>
+      </c>
+      <c r="H1200" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833516.jpg</t>
+        </is>
+      </c>
+      <c r="I1200" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>LPM bentuk jaringan pengaman guna lawan 4 penyakit sosial di desa</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:22:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1201" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1201" t="inlineStr">
+        <is>
+          <t>DPP Lembaga Pemberdayaan Masyarakat (LPM) menyatakan bakal membentuk jaringan posko sebagai katup pengaman di seluruh ...</t>
+        </is>
+      </c>
+      <c r="F1201" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1201" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685087/lpm-bentuk-jaringan-pengaman-guna-lawan-4-penyakit-sosial-di-desa</t>
+        </is>
+      </c>
+      <c r="H1201" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000036267.jpg</t>
+        </is>
+      </c>
+      <c r="I1201" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>Komisi VI DPR dan BRI Situbondo edukasi pencegahan kejahatan digital</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:19:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1202" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1202" t="inlineStr">
+        <is>
+          <t>Komisi VI Dewan Perwakilan Rakyat Republik Indonesia bersama PT Bank Rakyat Indonesia (Persero) Tbk Cabang Situbondo, ...</t>
+        </is>
+      </c>
+      <c r="F1202" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1202" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685083/komisi-vi-dpr-dan-bri-situbondo-edukasi-pencegahan-kejahatan-digital</t>
+        </is>
+      </c>
+      <c r="H1202" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG-20260807-WA0154.jpg</t>
+        </is>
+      </c>
+      <c r="I1202" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>PM Spanyol perketat keamanan saat liburan di tengah krisis migrasi</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:18:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1203" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1203" t="inlineStr">
+        <is>
+          <t>Perdana Menteri Spanyol Pedro Sanchez memperketat penjagaan keamanan selama melakukan liburan di Kepulauan Canary dan ...</t>
+        </is>
+      </c>
+      <c r="F1203" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1203" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685079/pm-spanyol-perketat-keamanan-saat-liburan-di-tengah-krisis-migrasi</t>
+        </is>
+      </c>
+      <c r="H1203" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/timnas-spanyol-juara-piala-dunia-2026-2824285.jpg</t>
+        </is>
+      </c>
+      <c r="I1203" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>Ratusan siswa Sekolah Rakyat Makassar sambut Mensos dengan "paper mob"</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:17:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1204" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1204" t="inlineStr">
+        <is>
+          <t>Ratusan siswa menyambut kedatangan Menteri Sosial Saifullah Yusuf (Gus Ipul) dengan penampilan paper mob di Sekolah ...</t>
+        </is>
+      </c>
+      <c r="F1204" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1204" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685075/ratusan-siswa-sekolah-rakyat-makassar-sambut-mensos-dengan-paper-mob</t>
+        </is>
+      </c>
+      <c r="H1204" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-20.24.11.jpeg</t>
+        </is>
+      </c>
+      <c r="I1204" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>Gempa magnitudo 5,0 guncang barat laut Jepara pada Jumat malam</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:16:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1205" t="inlineStr">
+        <is>
+          <t>Gempa bumi magnitudo 5,0 mengguncang wilayah perairan Laut Jawa, tepatnya di 102 kilometer ke arah barat laut dari ...</t>
+        </is>
+      </c>
+      <c r="F1205" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1205" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685071/gempa-magnitudo-50-guncang-barat-laut-jepara-pada-jumat-malam</t>
+        </is>
+      </c>
+      <c r="H1205" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/ilustrasi-gempa-3_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1205" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>Pemerintah siapkan aturan PT Timah serap produksi tambang rakyat</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:15:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1206" t="inlineStr">
+        <is>
+          <t>Kementerian Energi dan Sumber Daya Mineral (ESDM) menyampaikan pemerintah sedang mempersiapkan peraturan presiden ...</t>
+        </is>
+      </c>
+      <c r="F1206" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1206" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685068/pemerintah-siapkan-aturan-pt-timah-serap-produksi-tambang-rakyat</t>
+        </is>
+      </c>
+      <c r="H1206" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/10/16/target-produksi-pt-timah-hingga-akhir-2025-2647369.jpg</t>
+        </is>
+      </c>
+      <c r="I1206" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>Satya Wacana lepas Hengky Lakay usai kebersamaan selama sembilan tahun</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:13:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1207" t="inlineStr">
+        <is>
+          <t>Satya Wacana Salatiga memutuskan untuk melepas kapten tim Henry Cornelis Lakay atau kerap disapa Hengky Lakay, setelah ...</t>
+        </is>
+      </c>
+      <c r="F1207" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1207" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685065/satya-wacana-lepas-hengky-lakay-usai-kebersamaan-selama-sembilan-tahun</t>
+        </is>
+      </c>
+      <c r="H1207" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/09/02/IBla.jpeg</t>
+        </is>
+      </c>
+      <c r="I1207" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>Kubu Febrie Adriansyah siapkan saksi dan ahli meringankan</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:10:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1208" t="inlineStr">
+        <is>
+          <t>Kubu mantan Jaksa Agung Muda Bidang Tindak Pidana Khusus (Jampidsus) Febrie Adriansyah akan menghadirkan saksi dan ahli ...</t>
+        </is>
+      </c>
+      <c r="F1208" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1208" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685063/kubu-febrie-adriansyah-siapkan-saksi-dan-ahli-meringankan</t>
+        </is>
+      </c>
+      <c r="H1208" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000087486.jpg</t>
+        </is>
+      </c>
+      <c r="I1208" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>Siap guncang GBK besok! Intip aksi memukau skuad AC Milan di Senayan sebelum jamu Chelsea</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:10:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1209" t="inlineStr">
+        <is>
+          <t>Pesepak bola AC Milan mengikuti sesi latihan di Stadion Madya, Senayan, Jakarta, Jumat (7/8/2026). AC Milan melakukan ...</t>
+        </is>
+      </c>
+      <c r="F1209" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1209" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685061/siap-guncang-gbk-besok-intip-aksi-memukau-skuad-ac-milan-di-senayan-sebelum-jamu-chelsea</t>
+        </is>
+      </c>
+      <c r="H1209" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Latihan-AC-Milan-jelang-melawan-Chelsea-070826-fzn-4.jpg</t>
+        </is>
+      </c>
+      <c r="I1209" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>Ekonom dorong pemisahan fungsi pengaturan BEI dalam demutualisasi</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:07:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1210" t="inlineStr">
+        <is>
+          <t>Kepala Ekonom PermataBank Josua Pardede mendorong pemisahan fungsi pengaturan Bursa Efek Indonesia (BEI) dalam proses ...</t>
+        </is>
+      </c>
+      <c r="F1210" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1210" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685057/ekonom-dorong-pemisahan-fungsi-pengaturan-bei-dalam-demutualisasi</t>
+        </is>
+      </c>
+      <c r="H1210" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IHSG-ditutup-menguat-65-94-poin-070826-Fah-1.jpg</t>
+        </is>
+      </c>
+      <c r="I1210" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>LPSK luncurkan dana bantuan untuk penuhi restitusi korban TPKS</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:07:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1211" t="inlineStr">
+        <is>
+          <t>Lembaga Pelindungan Saksi dan Korban (LPSK) meluncurkan Dana Bantuan Korban (DBK) untuk membantu memenuhi restitusi ...</t>
+        </is>
+      </c>
+      <c r="F1211" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1211" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685056/lpsk-luncurkan-dana-bantuan-untuk-penuhi-restitusi-korban-tpks</t>
+        </is>
+      </c>
+      <c r="H1211" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001224363.jpg</t>
+        </is>
+      </c>
+      <c r="I1211" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>Dedi Mulyadi sebut utang hajatan picu TKI ilegal dan TPPO di Jabar</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:06:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1212" t="inlineStr">
+        <is>
+          <t>Gubernur Jawa Barat Dedi Mulyadi menyebut tradisi berutang untuk biaya hajatan dan pernikahan menjadi salah satu faktor ...</t>
+        </is>
+      </c>
+      <c r="F1212" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1212" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685055/dedi-mulyadi-sebut-utang-hajatan-picu-tki-ilegal-dan-tppo-di-jabar</t>
+        </is>
+      </c>
+      <c r="H1212" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000036265.jpg</t>
+        </is>
+      </c>
+      <c r="I1212" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>BGN sisir 13 ribu SPPG, prioritaskan operasional di 3T-rawan stunting</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:06:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1213" t="inlineStr">
+        <is>
+          <t>Badan Gizi Nasional (BGN) menyisir pembangunan 13 ribu Satuan Pelayanan Pemenuhan Gizi (SPPG) dan memprioritaskan ...</t>
+        </is>
+      </c>
+      <c r="F1213" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1213" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685051/bgn-sisir-13-ribu-sppg-prioritaskan-operasional-di-3t-rawan-stunting</t>
+        </is>
+      </c>
+      <c r="H1213" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/BGN-berhentikan-66-kepala-dapur-MBG-070826-rn-01.jpg</t>
+        </is>
+      </c>
+      <c r="I1213" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>BGN pecat 66 kepala dapur MBG karena tindakan indisipliner</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:03:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1214" t="inlineStr">
+        <is>
+          <t>ANTARA - Kepala Badan Gizi Nasional (BGN) Sudaryono mengatakan hingga Jumat (7/8), pihaknya telah memberhentikan 66 ...</t>
+        </is>
+      </c>
+      <c r="F1214" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1214" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5684984/bgn-pecat-66-kepala-dapur-mbg-karena-tindakan-indisipliner</t>
+        </is>
+      </c>
+      <c r="H1214" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/BGN-PECAT-66-KEPALA-DAPUR-MBG-KARENA-TINDAKAN-INDISIPLINER.jpg</t>
+        </is>
+      </c>
+      <c r="I1214" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>Bappenas: Pembangunan Papua jadi ikhtiar untuk kemajuan kawasan</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:01:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1215" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Perencanaan Pembangunan Nasional (PPN)/Wakil Kepala Badan Perencanaan Pembangunan Nasional (Bappenas) ...</t>
+        </is>
+      </c>
+      <c r="F1215" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1215" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685043/bappenas-pembangunan-papua-jadi-ikhtiar-untuk-kemajuan-kawasan</t>
+        </is>
+      </c>
+      <c r="H1215" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Bappenas-Papua.jpg</t>
+        </is>
+      </c>
+      <c r="I1215" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>Tumpukan sampah Kedaung Kaliangke akibat transisi sistem pengelolaan</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:59:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1216" t="inlineStr">
+        <is>
+          <t>Kepala Suku Dinas Lingkungan Hidup (Kasudin LH) Jakarta Barat, Aldi Jansen menyampaikan bahwa tumpukan sampah di RW 03 ...</t>
+        </is>
+      </c>
+      <c r="F1216" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1216" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685041/tumpukan-sampah-kedaung-kaliangke-akibat-transisi-sistem-pengelolaan</t>
+        </is>
+      </c>
+      <c r="H1216" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG-20260807-WA0013_3.jpg</t>
+        </is>
+      </c>
+      <c r="I1216" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>Prabowo terima laporan pendapatan Danantara naik 400 persen</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:59:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1217" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto mengungkapkan menerima laporan bahwa pendapatan Danantara meningkat sekitar 400 persen dalam ...</t>
+        </is>
+      </c>
+      <c r="F1217" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1217" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685039/prabowo-terima-laporan-pendapatan-danantara-naik-400-persen</t>
+        </is>
+      </c>
+      <c r="H1217" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/19308ac9-e06c-4451-9835-757ab1cfb7d3.jpeg</t>
+        </is>
+      </c>
+      <c r="I1217" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>OpenAI dikabarkan pasarkan pengeras suara mulai dari Rp5,3 jutaan</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:58:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1218" t="inlineStr">
+        <is>
+          <t>OpenAI dikabarkan memasarkan produk teknologi berupa perangkat keras speaker atau pengeras suara pintar mulai ...</t>
+        </is>
+      </c>
+      <c r="F1218" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1218" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685036/openai-dikabarkan-pasarkan-pengeras-suara-mulai-dari-rp53-jutaan</t>
+        </is>
+      </c>
+      <c r="H1218" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/10/09/Clipboard_10-09-2024_04.jpg</t>
+        </is>
+      </c>
+      <c r="I1218" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>KPK geledah rumah Sekretaris DPRD Kota Bengkulu</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:57:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1219" t="inlineStr">
+        <is>
+          <t>Penyidik Komisi Pemberantasan Korupsi (KPK) menggeledah rumah Sekretaris DPRD Kota Bengkulu Syofyan Tosoni di Kelurahan ...</t>
+        </is>
+      </c>
+      <c r="F1219" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1219" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685032/kpk-geledah-rumah-sekretaris-dprd-kota-bengkulu</t>
+        </is>
+      </c>
+      <c r="H1219" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_20260807_210151.jpg</t>
+        </is>
+      </c>
+      <c r="I1219" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>Sultra perkuat akses ekspor UMKM melalui program GETRA</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:57:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1220" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Provinsi Sulawesi Tenggara bersama Bank Indonesia memperkuat akses ekspor bagi pelaku usaha mikro, ...</t>
+        </is>
+      </c>
+      <c r="F1220" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1220" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685000/sultra-perkuat-akses-ekspor-umkm-melalui-program-getra</t>
+        </is>
+      </c>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SANS_SULTRA-PERKUAT-AKSES-EKSPOR-UMKM-MELALUI-PROGRAM-GATRA_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1220" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>Wagub Papua: Feskop 2026 lahirkan petani muda kopi</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:56:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1221" t="inlineStr">
+        <is>
+          <t>Wakil Gubernur Papua Aryoko Rumaropen mengatakan penyelenggaraan Festival Kopi Papua (Feskop) 2026 mampu melahirkan ...</t>
+        </is>
+      </c>
+      <c r="F1221" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1221" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685031/wagub-papua-feskop-2026-lahirkan-petani-muda-kopi</t>
+        </is>
+      </c>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1002075495.jpg</t>
+        </is>
+      </c>
+      <c r="I1221" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>Kapolri siap jembatani dialog buruh-DPR soal RUU Ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:55:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1222" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Pol. Listyo Sigit Prabowo menyatakan pihaknya siap menjembatani kalangan buruh dengan DPR RI dalam ...</t>
+        </is>
+      </c>
+      <c r="F1222" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1222" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685025/kapolri-siap-jembatani-dialog-buruh-dpr-soal-ruu-ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000087467.jpg</t>
+        </is>
+      </c>
+      <c r="I1222" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>Ekonom: Penundaan pajak marketplace beri ruang UMKM jaga arus kas</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:53:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1223" t="inlineStr">
+        <is>
+          <t>Ekonom Center of Reform on Economics (CORE) Yusuf Rendy Manilet menilai ditundanya pungutan Pajak Penghasilan (PPh) ...</t>
+        </is>
+      </c>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1223" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685021/ekonom-penundaan-pajak-marketplace-beri-ruang-umkm-jaga-arus-kas</t>
+        </is>
+      </c>
+      <c r="H1223" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/11/13/InShot_20200910_104834146.jpg</t>
+        </is>
+      </c>
+      <c r="I1223" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>RANS Simba Bogor dan Juan Laurent sepakat akhiri kerja sama</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:47:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1224" t="inlineStr">
+        <is>
+          <t>RANS Simba Bogor mengumumkan telah mengakhiri kerja sama dengan pebasket Juan Laurent Kokodiputra berdasarkan ...</t>
+        </is>
+      </c>
+      <c r="F1224" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1224" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685015/rans-simba-bogor-dan-juan-laurent-sepakat-akhiri-kerja-sama</t>
+        </is>
+      </c>
+      <c r="H1224" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/01/11/Tangerang-Hawks-dikalahkan-Satria-Muda-Pertamina-Bandung-11012026-gp-18.jpg</t>
+        </is>
+      </c>
+      <c r="I1224" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>Penguatan pendidikan melalui pembaruan buku ajar nasional</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:45:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1225" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah terus mematangkan pembaruan buku ajar nasional sebagai bagian dari upaya memperkuat kualitas ...</t>
+        </is>
+      </c>
+      <c r="F1225" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1225" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5684957/penguatan-pendidikan-melalui-pembaruan-buku-ajar-nasional</t>
+        </is>
+      </c>
+      <c r="H1225" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PENGUATAN-PENDIDIKAN-MELALUI-PEMBARUAN-BUKU-AJAR-NASIONAL.jpg</t>
+        </is>
+      </c>
+      <c r="I1225" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>KY umumkan 14 calon lolos seleksi hakim agung dan ad hoc</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:42:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1226" t="inlineStr">
+        <is>
+          <t>Komisi Yudisial (KY) mengumumkan 14 calon hakim agung dan hakim ad hoc yang dinyatakan lolos seleksi calon hakim agung, ...</t>
+        </is>
+      </c>
+      <c r="F1226" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1226" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685013/ky-umumkan-14-calon-lolos-seleksi-hakim-agung-dan-ad-hoc</t>
+        </is>
+      </c>
+      <c r="H1226" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001849541.jpg</t>
+        </is>
+      </c>
+      <c r="I1226" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>Polsek Tambora kembalikan enam motor curian kepada pemilik</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:40:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1227" t="inlineStr">
+        <is>
+          <t>Kepolisian mengembalikan enam unit sepeda motor hasil curian kepada pemilknya di Polsek Tambora, Jakarta Barat, ...</t>
+        </is>
+      </c>
+      <c r="F1227" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1227" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685005/polsek-tambora-kembalikan-enam-motor-curian-kepada-pemilik</t>
+        </is>
+      </c>
+      <c r="H1227" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG-20260807-WA0040.jpg</t>
+        </is>
+      </c>
+      <c r="I1227" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>Bappenas: Kopi dan kakao sumber penghidupan jutaan keluarga Indonesia</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:40:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1228" t="inlineStr">
+        <is>
+          <t>Deputi Bidang Pangan, Sumber Daya Alam, dan Lingkungan Hidup Kementerian Perencanaan Pembangunan Nasional/Badan ...</t>
+        </is>
+      </c>
+      <c r="F1228" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1228" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685001/bappenas-kopi-dan-kakao-sumber-penghidupan-jutaan-keluarga-indonesia</t>
+        </is>
+      </c>
+      <c r="H1228" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Teguh-Pettani.jpg</t>
+        </is>
+      </c>
+      <c r="I1228" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>BGN buka PO box pengaduan MBG perkuat transparansi dan pengawasan</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:36:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1229" t="inlineStr">
+        <is>
+          <t>Badan Gizi Nasional (BGN) membuka jalur pengaduan melalui mekanisme PO box untuk memperkuat transparansi dan sistem ...</t>
+        </is>
+      </c>
+      <c r="F1229" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1229" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684992/bgn-buka-po-box-pengaduan-mbg-perkuat-transparansi-dan-pengawasan</t>
+        </is>
+      </c>
+      <c r="H1229" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG-20260806-WA0015_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1229" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>Akun X TMC Polda Metro Jaya diretas pihak tak dikenal</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:35:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1230" t="inlineStr">
+        <is>
+          <t>Akun X TMC Polda Metro Jaya diretas pihak tak dikenal, sehingga mengganggu publikasi informasi lalu lintas di wilayah ...</t>
+        </is>
+      </c>
+      <c r="F1230" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1230" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684988/akun-x-tmc-polda-metro-jaya-diretas-pihak-tak-dikenal</t>
+        </is>
+      </c>
+      <c r="H1230" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/IMG_20260630_094425.jpg</t>
+        </is>
+      </c>
+      <c r="I1230" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>Kekurangan staf picu penundaan dan pembatalan penerbangan di Sydney</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:35:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1231" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1231" t="inlineStr">
+        <is>
+          <t>Kekurangan staf layanan penerbangan dilaporkan menyebabkan penundaan penerbangan secara luas dan sejumlah pembatalan ...</t>
+        </is>
+      </c>
+      <c r="F1231" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1231" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684985/kekurangan-staf-picu-penundaan-dan-pembatalan-penerbangan-di-sydney</t>
+        </is>
+      </c>
+      <c r="H1231" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/CjkinzN000023_20260807_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1231" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>Prabowo: "Kita bekerja beri harapan rakyat yang paling tak berdaya"</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:34:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1232" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1232" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto saat memberikan sambutan dalam acara peluncuran 10 buku karya Menteri ESDM Bahlil Lahadalia ...</t>
+        </is>
+      </c>
+      <c r="F1232" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1232" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684980/prabowo-kita-bekerja-beri-harapan-rakyat-yang-paling-tak-berdaya</t>
+        </is>
+      </c>
+      <c r="H1232" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Peluncuran-10-buku-karya-nyata-untuk-negeri-Bahlil-Lahadalia-070826-Ada-4.jpg</t>
+        </is>
+      </c>
+      <c r="I1232" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>BGN tetapkan pembagian jajaran pejabat di daerah untuk awasi MBG</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:32:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1233" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1233" t="inlineStr">
+        <is>
+          <t>Badan Gizi Nasional (BGN) menetapkan pembagian wilayah tanggung jawab bagi jajaran pejabat eselon I dan II untuk ...</t>
+        </is>
+      </c>
+      <c r="F1233" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1233" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684979/bgn-tetapkan-pembagian-jajaran-pejabat-di-daerah-untuk-awasi-mbg</t>
+        </is>
+      </c>
+      <c r="H1233" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/BGN-berhentikan-66-kepala-dapur-MBG-070826-rn-01.jpg</t>
+        </is>
+      </c>
+      <c r="I1233" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>Grup musik D'MASIV agendakan Hong Kong dalam tur Asia Home Run 2026</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:31:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1234" t="inlineStr">
+        <is>
+          <t>Grup band D'MASIV mengagendakan lawatan ke Hong Kong dalam tur Asia pada 2026 bertajuk "D'MASIV Asia Home ...</t>
+        </is>
+      </c>
+      <c r="F1234" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1234" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684976/grup-musik-dmasiv-agendakan-hong-kong-dalam-tur-asia-home-run-2026</t>
+        </is>
+      </c>
+      <c r="H1234" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG-20260807-WA0013-3.jpg</t>
+        </is>
+      </c>
+      <c r="I1234" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>Presiden Meksiko umumkan rencana keamanan untuk ekspor alpukat ke AS</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:31:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1235" t="inlineStr">
+        <is>
+          <t>Presiden Meksiko Claudia Sheinbaum pada Kamis (6/8) mengatakan pemerintahannya sedang menyusun rencana aksi untuk ...</t>
+        </is>
+      </c>
+      <c r="F1235" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1235" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684973/presiden-meksiko-umumkan-rencana-keamanan-untuk-ekspor-alpukat-ke-as</t>
+        </is>
+      </c>
+      <c r="H1235" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/CjkinzN000025_20260807_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1235" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>Wizards dan Davis tunda negosiasi kontrak hingga awal musim reguler</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:31:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1236" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1236" t="inlineStr">
+        <is>
+          <t>Washington Wizards dan Anthony Davis bersepakat untuk menunda pembahasan perpanjangan kontrak hingga awal musim reguler ...</t>
+        </is>
+      </c>
+      <c r="F1236" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1236" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684972/wizards-dan-davis-tunda-negosiasi-kontrak-hingga-awal-musim-reguler</t>
+        </is>
+      </c>
+      <c r="H1236" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/04/20/2023-04-20T000958Z_741082554_MT1USATODAY20498153_RTRMADP_3_NBA-PLAYOFFS-LOS-ANGELES-LAKERS-AT-MEMPHIS-GRIZZLIES.jpg</t>
+        </is>
+      </c>
+      <c r="I1236" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>Polda Jabar ungkap 352 kasus kejahatan jalanan dan siapkan pencegahan</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:30:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1237" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1237" t="inlineStr">
+        <is>
+          <t>ANTARA - Polda Jawa Barat mengungkap 352 kasus kejahatan jalanan dengan 413 pelaku sepanjang Juni hingga Agustus 2026. ...</t>
+        </is>
+      </c>
+      <c r="F1237" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1237" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5684943/polda-jabar-ungkap-352-kasus-kejahatan-jalanan-dan-siapkan-pencegahan</t>
+        </is>
+      </c>
+      <c r="H1237" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/POLDA-JABAR-UNGKAP-352-KASUS-KEJAHATAN-JALANAN-DAN-SIAPKAN-PENCEGAHAN.jpg</t>
+        </is>
+      </c>
+      <c r="I1237" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>Bursa saham Singapura catat rekor pendapatan dan laba bersih pada 2026</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:27:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1238" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1238" t="inlineStr">
+        <is>
+          <t>Bursa Saham Singapura (Singapore Exchange/SGX Group) mencatatkan rekor pendapatan dan laba bersih untuk tahun keuangan ...</t>
+        </is>
+      </c>
+      <c r="F1238" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1238" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684969/bursa-saham-singapura-catat-rekor-pendapatan-dan-laba-bersih-pada-2026</t>
+        </is>
+      </c>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/CjkinzN000027_20260807_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1238" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>Chelsea jadikan laga pramusim di Jakarta bangun mentalitas pemenang</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:27:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1239" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1239" t="inlineStr">
+        <is>
+          <t>Manajer Chelsea Xabi Alonso menjadikan laga tur pramusim di Jakarta menjadi bagian dari momentum membangun mentalitas ...</t>
+        </is>
+      </c>
+      <c r="F1239" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1239" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684968/chelsea-jadikan-laga-pramusim-di-jakarta-bangun-mentalitas-pemenang</t>
+        </is>
+      </c>
+      <c r="H1239" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_20260807_211305.jpg</t>
+        </is>
+      </c>
+      <c r="I1239" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>Menkum ungkap alasan pemerintah perketat naturalisasi WNA</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:27:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1240" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1240" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Hukum Supratman Andi Agtas di Jakarta, Jumat (7/8), mengatakan pemerintah telah memperketat ...</t>
+        </is>
+      </c>
+      <c r="F1240" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1240" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5684923/menkum-ungkap-alasan-pemerintah-perketat-naturalisasi-wna</t>
+        </is>
+      </c>
+      <c r="H1240" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MENKUM-UNGKAP-ALASAN-PEMERINTAH-PERKETAT-NATURALISASI-WNA.jpg</t>
+        </is>
+      </c>
+      <c r="I1240" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>China rilis peta bulan yang disempurnakan</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:25:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1241" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1241" t="inlineStr">
+        <is>
+          <t>Sebuah tim peneliti China telah merampungkan peta geologis terbaru dari seluruh permukaan Bulan dengan skala ...</t>
+        </is>
+      </c>
+      <c r="F1241" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1241" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5684965/china-rilis-peta-bulan-yang-disempurnakan</t>
+        </is>
+      </c>
+      <c r="H1241" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/CjkinzN000021_20260807_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1241" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>Polri Pastikan Periksa Personel Polresta Banda Aceh Transparan</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:08:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1242" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1242" t="inlineStr">
+        <is>
+          <t>Polri memastikan pemeriksaan Kapolresta Banda Aceh dan Kasat Narkoba dilakukan secara profesional dan transparan.</t>
+        </is>
+      </c>
+      <c r="F1242" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1242" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609267/polri-pastikan-periksa-personel-polresta-banda-aceh-transparan</t>
+        </is>
+      </c>
+      <c r="H1242" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/02/25/kadiv-humas-polri-johnny-eddizon-isir-1771994950407_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1242" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>Gaduh di Jakut Saat Ada Pencuri Kabel Tersengat Listik hingga Melepuh</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:01:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1243" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E1243" t="inlineStr">
+        <is>
+          <t>Suasana di Sunter Agung, Jakarta Utara (Jakut), mendadak gaduh. Seorang pria ditarik paksa dari gardu PLN karena diduga hendak mencuri kabel listrik.</t>
+        </is>
+      </c>
+      <c r="F1243" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1243" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609235/gaduh-di-jakut-saat-ada-pencuri-kabel-tersengat-listik-hingga-melepuh</t>
+        </is>
+      </c>
+      <c r="H1243" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/maling-kabel-listrik-di-gardu-pln-sunter-agung-jakut-kesetrum-hingga-badan-melepuh-1786074935209_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1243" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>Kapolres Malang Gandeng Driver Ojol Jaga Keamanan Warga</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:52:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>Firda Cynthia Anggrainy</t>
+        </is>
+      </c>
+      <c r="E1244" t="inlineStr">
+        <is>
+          <t>Kapolres Malang, AKBP Rulian Syauri, ajak pengemudi ojol jaga kamtibmas. Pertemuan ini bertujuan mempererat komunikasi dan sinergi dengan komunitas ojol.</t>
+        </is>
+      </c>
+      <c r="F1244" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1244" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609228/kapolres-malang-gandeng-driver-ojol-jaga-keamanan-warga</t>
+        </is>
+      </c>
+      <c r="H1244" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/kapolres-malang-akbp-rulian-syauri-berdialog-dengan-perhimpunan-driver-ojek-indonesia-pdoi-malang-raya-1786114289613_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1244" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>Guyon Bahlil ke Cak Imin: Ketum Lama Belum Tentu Punya Buku Diteken Presiden</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:51:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1245" t="inlineStr">
+        <is>
+          <t>Eva Safitri</t>
+        </is>
+      </c>
+      <c r="E1245" t="inlineStr">
+        <is>
+          <t>Ketum Golkar Bahlil Lahadalia bercanda tentang bukunya yang ditandatangani Prabowo, menyindir Cak Imin. Candaan ini mengundang tawa audiens di Jakarta.</t>
+        </is>
+      </c>
+      <c r="F1245" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1245" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609227/guyon-bahlil-ke-cak-imin-ketum-lama-belum-tentu-punya-buku-diteken-presiden</t>
+        </is>
+      </c>
+      <c r="H1245" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/bahlil-lahadalia-1786111824719_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1245" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>Pansus DPRD DKI Bakal Sidak 200 Vendor Pengelola Sampah, Cek Dibuang ke Mana</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:36:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1246" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E1246" t="inlineStr">
+        <is>
+          <t>DPRD DKI Jakarta akan sidak 200 vendor pengelola sampah untuk memastikan kepatuhan dalam pengolahan dan pembuangan sampah sesuai dengan aturan.</t>
+        </is>
+      </c>
+      <c r="F1246" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1246" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609216/pansus-dprd-dki-bakal-sidak-200-vendor-pengelola-sampah-cek-dibuang-ke-mana</t>
+        </is>
+      </c>
+      <c r="H1246" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/judistira-1786113237333_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1246" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>Terduga Pembunuh Bos Konter HP Ambarawa Ditangkap, Ternyata Teman Korban</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:24:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1247" t="inlineStr">
+        <is>
+          <t>Ardian Dwi Kurnia</t>
+        </is>
+      </c>
+      <c r="E1247" t="inlineStr">
+        <is>
+          <t>Polres Semarang dan Polda Jateng menangkap terduga pelaku pencurian dengan kekerasan yang mengakibatkan kematian pemilik konter ponsel Royal Phone Ambarawa.</t>
+        </is>
+      </c>
+      <c r="F1247" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1247" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609199/terduga-pembunuh-bos-konter-hp-ambarawa-ditangkap-ternyata-teman-korban</t>
+        </is>
+      </c>
+      <c r="H1247" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/konter-hp-royal-phone-di-ambarawa-tkp-pencurian-dengan-kekerasan-kamis-682026-1786034565792_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1247" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>7 Jam Diperiksa Kejagung, Febrie Adriansyah Dibawa Lagi ke Rutan KPK</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:22:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1248" t="inlineStr">
+        <is>
+          <t>Mulia Budi, Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1248" t="inlineStr">
+        <is>
+          <t>Febrie Adriansyah selesai diperiksa sebagai tersangka di kasus tindak pidana pencucian uang (TPPU). Usai 7 jam diperiksa, Febrie dikembalikan ke Rutan KPK.</t>
+        </is>
+      </c>
+      <c r="F1248" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1248" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609198/7-jam-diperiksa-kejagung-febrie-adriansyah-dibawa-lagi-ke-rutan-kpk</t>
+        </is>
+      </c>
+      <c r="H1248" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/febrie-adriansyah-selesai-diperiksa-kejagung-langsung-dibawa-lagi-ke-rutan-kpk-muliadetikcom-1786112429835_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1248" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>Bahlil Puji Luhut Mentornya: Ada Saat Dia Menekan, Ada Saat Dia Sayang-sayang Saya</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:12:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1249" t="inlineStr">
+        <is>
+          <t>Eva Safitri</t>
+        </is>
+      </c>
+      <c r="E1249" t="inlineStr">
+        <is>
+          <t>Ketua Umum Golkar Bahlil Lahadalia menyebut Luhut sebagai mentornya. Ia mengaku dimentori Luhut tentang negosiasi investasi saat menjabat Menteri Investasi.</t>
+        </is>
+      </c>
+      <c r="F1249" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1249" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609192/bahlil-puji-luhut-mentornya-ada-saat-dia-menekan-ada-saat-dia-sayang-sayang-saya</t>
+        </is>
+      </c>
+      <c r="H1249" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/bahlil-lahadalia-1786111824719_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1249" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>Polisi Ungkap Kendala Pencarian Kaki Korban Mutilasi di Kali Licin Depok</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:10:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1250" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E1250" t="inlineStr">
+        <is>
+          <t>Polisi masih mencari potongan kaki korban mutilasi K (51) di Kali Licin, Depok. Kendala pencarian akibat aliran sungai yang membawa potongan tersebut.</t>
+        </is>
+      </c>
+      <c r="F1250" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1250" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609186/polisi-ungkap-kendala-pencarian-kaki-korban-mutilasi-di-kali-licin-depok</t>
+        </is>
+      </c>
+      <c r="H1250" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/polisi-lanjut-cari-potongan-kaki-korban-mutilasi-di-kali-licin-depok-devidetikcom-1786074971703_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1250" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>Herman Deru Dorong Penguatan Sinergi untuk Jaga Kelestarian Hutan Sumsel</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:00:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1251" t="inlineStr">
+        <is>
+          <t>Hana Nushratu Uzma</t>
+        </is>
+      </c>
+      <c r="E1251" t="inlineStr">
+        <is>
+          <t>Gubernur Sumsel Herman Deru dorong sinergi masyarakat dan pemerintah untuk jaga kelestarian hutan. Pentingnya kearifan lokal dan penambahan Polhut juga disorot.</t>
+        </is>
+      </c>
+      <c r="F1251" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1251" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609166/herman-deru-dorong-penguatan-sinergi-untuk-jaga-kelestarian-hutan-sumsel</t>
+        </is>
+      </c>
+      <c r="H1251" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/pemprov-sumsel-1786111204596_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1251" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>Api Cemburu Bikin Remaja Sayat Leher Warga Depok Pakai Cutter</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:00:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E1252" t="inlineStr">
+        <is>
+          <t>Remaja RAN (19) ditangkap setelah menyerang MAN (16) di Depok karena cemburu. Pelaku menyayat leher korban dengan cutter.</t>
+        </is>
+      </c>
+      <c r="F1252" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1252" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609165/api-cemburu-bikin-remaja-sayat-leher-warga-depok-pakai-cutter</t>
+        </is>
+      </c>
+      <c r="H1252" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/polisi-tangkap-pelaku-penyerangan-terhadap-warga-di-depok-dokistimewa-1786087228399_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1252" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>Aturan Logam Tanah Jarang Lagi Disusun, Bakal Diolah di Dalam Negeri</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:25:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E1253" t="inlineStr">
+        <is>
+          <t>Menteri ESDM Bahlil Lahadalia mengatakan pemerintah sedang menyusun aturan teknis terkait larangan ekspor rare earth atau Logam Tanah Jarang (LTJ).</t>
+        </is>
+      </c>
+      <c r="F1253" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1253" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8609275/aturan-logam-tanah-jarang-lagi-disusun-bakal-diolah-di-dalam-negeri</t>
+        </is>
+      </c>
+      <c r="H1253" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/10/09/logam-tanah-jarang-jadi-harta-karun-yang-diincar-dunia-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1253" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>Jawaban Bahlil Usai Dapat Rapor Memuaskan dari Prabowo</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:03:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E1254" t="inlineStr">
+        <is>
+          <t>Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia merespons penilaian Presiden Prabowo Subianto yang menyebut kinerjanya memuaskan.</t>
+        </is>
+      </c>
+      <c r="F1254" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1254" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8609236/jawaban-bahlil-usai-dapat-rapor-memuaskan-dari-prabowo</t>
+        </is>
+      </c>
+      <c r="H1254" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1254" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>Pasar Murah Ringankan Beban Belanja Warga</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:40:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>Agung Pambudhy</t>
+        </is>
+      </c>
+      <c r="E1255" t="inlineStr">
+        <is>
+          <t>Pemprov Jatim bersama Perum Bulog menggelar pasar murah di Sidoarjo untuk menjaga stabilitas harga pangan, mengendalikan inflasi, dan membantu daya beli warga.</t>
+        </is>
+      </c>
+      <c r="F1255" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1255" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8609097/pasar-murah-ringankan-beban-belanja-warga</t>
+        </is>
+      </c>
+      <c r="H1255" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/pasar-murah-di-sidoarjo-1786108342125_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1255" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>BGN Sisir Sekolah Swasta Elite Tak Butuh MBG</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:25:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>Retno Ayuningrum</t>
+        </is>
+      </c>
+      <c r="E1256" t="inlineStr">
+        <is>
+          <t>Kepala Badan Gizi Nasional (BGN) Sudaryono menyampaikan sekolah swasta elit tidak membutuhkan program makan bergizi gratis (MBG).</t>
+        </is>
+      </c>
+      <c r="F1256" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1256" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609200/bgn-sisir-sekolah-swasta-elite-tak-butuh-mbg</t>
+        </is>
+      </c>
+      <c r="H1256" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/kepala-badan-gizi-nasional-bgn-sudaryono-1786101835426_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1256" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>Prabowo Pastikan Harga BBM Subsidi Tidak Naik</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:07:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E1257" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto menyebut Indonesia berhasil menjaga harga Bahan Bakar Minyak (BBM) bersubsidi tidak naik</t>
+        </is>
+      </c>
+      <c r="F1257" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1257" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8609174/prabowo-pastikan-harga-bbm-subsidi-tidak-naik</t>
+        </is>
+      </c>
+      <c r="H1257" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/31/presiden-prabowo-subianto-saat-memberikan-taklimat-di-depan-para-pimpinan-kamar-dagang-dan-industri-indonesia-kadin-di-istana--1785493704749_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1257" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>Larangan Ekspor Tembaga &amp;amp; Bauksit Mentah Tetap Berlaku!</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 20:45:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E1258" t="inlineStr">
+        <is>
+          <t>Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia buka suara soal ekspor mineral. Bahlil memastikan pemerintah melarang ekspor mineral mentah.</t>
+        </is>
+      </c>
+      <c r="F1258" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1258" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8609135/larangan-ekspor-tembaga-bauksit-mentah-tetap-berlaku</t>
+        </is>
+      </c>
+      <c r="H1258" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1258" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>Dari Lereng Arjuno Menembus Pasar Ekspor</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 20:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>Agung Pambudhy</t>
+        </is>
+      </c>
+      <c r="E1259" t="inlineStr">
+        <is>
+          <t>Industri kopi rumahan di Malang mengolah hasil panen 207 petani mitra menjadi produk bernilai tambah yang dipasarkan ke dalam negeri hingga ekspor.</t>
+        </is>
+      </c>
+      <c r="F1259" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1259" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8609121/dari-lereng-arjuno-menembus-pasar-ekspor</t>
+        </is>
+      </c>
+      <c r="H1259" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/industri-pengolahan-dan-pusat-studi-kopi-nusantara-di-malang-1786109312747_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1259" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung di Jalan Abdul Muis Jakpus, 20 Unit Damkar Dikerahkan</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:29:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1260" t="inlineStr">
+        <is>
+          <t>Kebakaran terjadi di bangunan bertingkat yang berada di Jalan Abdul Muis, Jakarta Pusat. 20 unit damkar, 100 personel dikerahkan.</t>
+        </is>
+      </c>
+      <c r="F1260" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1260" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807221850-20-1389979/kebakaran-gedung-di-jalan-abdul-muis-jakpus-20-unit-damkar-dikerahkan</t>
+        </is>
+      </c>
+      <c r="H1260" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/03/30/ilustrasi-ledakan-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1260" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>Gempa M5,0 di Jepara Jateng, Tak Berpotensi Tsunami</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:11:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1261" t="inlineStr">
+        <is>
+          <t>Gempa bumi tektonik M5.0 mengguncang Jepara, Jawa Tengah, Jumat (7/8). Tidak berpotensi tsunami.</t>
+        </is>
+      </c>
+      <c r="F1261" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1261" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807220347-20-1389976/gempa-m50-di-jepara-jateng-tak-berpotensi-tsunami</t>
+        </is>
+      </c>
+      <c r="H1261" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2016/11/21/f26faae5-d7b3-4ba6-b508-e53f4ff585e4_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1261" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>Kebakaran Bromo Meluas 176 Hektare, Heli Dikerahkan Water Bombing</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:59:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1262" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan di Bromo meluas hingga 176,20 hektare. Upaya pemadaman melibatkan helikopter dan tim gabungan. Belum ada laporan korban jiwa.</t>
+        </is>
+      </c>
+      <c r="F1262" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1262" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807201108-12-1389942/kebakaran-bromo-meluas-176-hektare-heli-dikerahkan-water-bombing</t>
+        </is>
+      </c>
+      <c r="H1262" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/kebakaran-bromo-meluas-jadi-176-hektare-1786108419489_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1262" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>KBPBI Apresiasi Komitmen Kapolri Kawal Pembahasan RUU Ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:42:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1263" t="inlineStr">
+        <is>
+          <t>Kapolri Listyo menilai, dialog diperlukan dalam berbagai persoalan ketenagakerjaan, sehingga dapat menghasilkan regulasi yang berimbang.</t>
+        </is>
+      </c>
+      <c r="F1263" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1263" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807210753-25-1389970/kbpbi-apresiasi-komitmen-kapolri-kawal-pembahasan-ruu-ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="H1263" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/polri-1786111823262_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1263" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>Pemprov DKI Sanksi Semua Pelaku Pembuangan Sampah Ilegal di Dukuh</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:21:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1264" t="inlineStr">
+        <is>
+          <t>Pemprov DKI menindak tegas pelaku pembuangan sampah ilegal di Kramat Jati. Tiga pelaku dijatuhi sanksi administratif untuk mencegah pencemaran lingkungan.</t>
+        </is>
+      </c>
+      <c r="F1264" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1264" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807205344-25-1389958/pemprov-dki-sanksi-semua-pelaku-pembuangan-sampah-ilegal-di-dukuh</t>
+        </is>
+      </c>
+      <c r="H1264" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/pemprov-dki-1786110503521_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1264" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>Pihak Sekolah Minta Polisi Bongkar Bunker Usai Temuan Ratusan Senjata</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:20:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1265" t="inlineStr">
+        <is>
+          <t>Sekolah swasta di Jakarta Selatan minta polisi bongkar bunker setelah ratusan senjata ditemukan. Kuasa hukum khawatir ada senjata lain di dalamnya.</t>
+        </is>
+      </c>
+      <c r="F1265" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1265" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807125001-12-1389679/pihak-sekolah-minta-polisi-bongkar-bunker-usai-temuan-ratusan-senjata</t>
+        </is>
+      </c>
+      <c r="H1265" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/995-senjata-yang-ditemukan-di-ruang-mantan-ketua-yayasan-sekolah-jaksel-1786011308099_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1265" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>Dokter PPDS UGM yang Cibir Pasien BPJS Dinonaktifkan 3 Bulan</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 20:37:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1266" t="inlineStr">
+        <is>
+          <t>FK-KMK UGM menonaktifkan Elda Putri Rahardini selama 3 bulan akibat komentar nirempati terhadap pasien BPJS. Investigasi pelanggaran etik sedang berlangsung.</t>
+        </is>
+      </c>
+      <c r="F1266" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1266" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807201756-12-1389945/dokter-ppds-ugm-yang-cibir-pasien-bpjs-dinonaktifkan-3-bulan</t>
+        </is>
+      </c>
+      <c r="H1266" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/05/15/universitas-gadjah-mada-1747298810323_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1266" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>Polisi Tangkap 15 Pria Terduga Pemerkosa Anak di Mamuju Sulbar</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 20:10:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1267" t="inlineStr">
+        <is>
+          <t>Polisi Mamuju tangkap 15 pria terkait kasus pemerkosaan anak 15 tahun yang hamil 3 bulan. Kasus terungkap setelah laporan keluarga.</t>
+        </is>
+      </c>
+      <c r="F1267" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1267" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807192400-12-1389915/polisi-tangkap-15-pria-terduga-pemerkosa-anak-di-mamuju-sulbar</t>
+        </is>
+      </c>
+      <c r="H1267" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/11/25/ilustrasi-penjara_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1267" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>Wamendagri Bima Arya Dorong Penghijauan Jadi Gerakan Berkelanjutan</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:47:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1268" t="inlineStr">
+        <is>
+          <t>Wamendagri Bima Arya mendorong Pemda untuk menjadikan penghijauan sebagai gerakan berkelanjutan, menekankan kolaborasi dan perawatan untuk dampak nyata.</t>
+        </is>
+      </c>
+      <c r="F1268" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1268" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807193943-20-1389924/wamendagri-bima-arya-dorong-penghijauan-jadi-gerakan-berkelanjutan</t>
+        </is>
+      </c>
+      <c r="H1268" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/wakil-menteri-dalam-negeri-wamendagri-bima-arya-sugiarto-1786106207706_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1268" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>FOTO: Jalintim Palembang Jambi Lumpuh Dua Pekan</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:45:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1269" t="inlineStr">
+        <is>
+          <t>Sejumlah kendaraan terjebak kemacetan di Jalan Lintas Timur Palembang-Jambi di Air Batu, Kabupaten Banyuasin, Sumatera Selatan, Jumat (7/8).</t>
+        </is>
+      </c>
+      <c r="F1269" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1269" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807185911-22-1389890/foto-jalintim-palembang-jambi-lumpuh-dua-pekan</t>
+        </is>
+      </c>
+      <c r="H1269" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/jalintim-palembang-jambi-lumpuh-dua-pekan-1786102821694_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1269" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>Cegah Politik Uang, Pemilihan Ketua Umum PBNU Diusulkan Lewat AHWA</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:34:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1270" t="inlineStr">
+        <is>
+          <t>TribunNews.com menyajikan berita dan video terkini dari regional, nasional dan internasional dengan sudut pandang dan nilai-nilai lokal</t>
+        </is>
+      </c>
+      <c r="F1270" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1270" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/</t>
+        </is>
+      </c>
+      <c r="H1270" t="inlineStr">
+        <is>
+          <t>https://asset-2.tribunnews.com/tribunnews/foto/bank/images/logo-tribunnews1_20160901_101844.jpg</t>
+        </is>
+      </c>
+      <c r="I1270" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>Malapetaka Menghantam Amerika, Ratusan Sudah Jadi Korban</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1271" t="inlineStr">
+        <is>
+          <t>Serangan siber terus menghantam AS, dengan peretas menargetkan lembaga keuangan dan perusahaan besar. Simak!</t>
+        </is>
+      </c>
+      <c r="F1271" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1271" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807132653-37-757416/malapetaka-menghantam-amerika-ratusan-sudah-jadi-korban</t>
+        </is>
+      </c>
+      <c r="H1271" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2022/05/23/bendera-amerika-serikat-1_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1271" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>Penemuan Baru Bantah Teori Evolusi Manusia yang Sudah Lama Dipercaya</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 20:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>Novina Putri Bestari</t>
+        </is>
+      </c>
+      <c r="E1272" t="inlineStr">
+        <is>
+          <t>Penelitian terbaru membantah teori evolusi manusia yang bertahap. Temuan menunjukkan perubahan fisik manusia purba dipengaruhi oleh budaya dan teknologi.</t>
+        </is>
+      </c>
+      <c r="F1272" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1272" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807131529-37-757405/penemuan-baru-bantah-teori-evolusi-manusia-yang-sudah-lama-dipercaya</t>
+        </is>
+      </c>
+      <c r="H1272" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/02/27/ilustrasi-manusia-purba-1772188117029_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1272" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>Pembeli Switch Minta Uang Kembali Karena Nintendo Untung Gede, Ditolak</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1273" t="inlineStr">
+        <is>
+          <t>Nintendo mencatat lonjakan laba 53,5 persen berkat pengembalian tarif impor dari AS.</t>
+        </is>
+      </c>
+      <c r="F1273" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1273" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807134011-37-757434/pembeli-switch-minta-uang-kembali-karena-nintendo-untung-gede-ditolak</t>
+        </is>
+      </c>
+      <c r="H1273" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/04/05/nintendo-switch-2-ap-photorichard-drew-1743838124363_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1273" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>Amerika Buka-Bukaan Alasan Sebenarnya China Harus Diblokir Total</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>Intan Rakhmayanti</t>
+        </is>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>AS membatasi impor teknologi China untuk keamanan nasional. FCC mendorong investasi domestik dan menghindari ancaman di masa depan.</t>
+        </is>
+      </c>
+      <c r="F1274" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1274" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807145711-37-757463/amerika-buka-bukaan-alasan-sebenarnya-china-harus-diblokir-total</t>
+        </is>
+      </c>
+      <c r="H1274" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/12/02/bendera-amerikas-serikat-as-dan-china-reutersflorence-loillustrationfile_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1274" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>Ilmuwan Harvard Klaim Tahu Lokasi Tuhan, Segini Jaraknya dari Bumi</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>Mantan fisikawan Harvard, Michael Guillén, klaim mengetahui lokasi Tuhan di alam semesta. Simak lokasinya!</t>
+        </is>
+      </c>
+      <c r="F1275" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1275" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807134408-37-757422/ilmuwan-harvard-klaim-tahu-lokasi-tuhan-segini-jaraknya-dari-bumi</t>
+        </is>
+      </c>
+      <c r="H1275" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/14/roket-diluncurkan-dari-pulau-hainan-di-selatan-tiongkok-pada-hari-jumat-1072026-pukul-1215-waktu-setempat-dari-pusat-peluncura-1783997825654_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1275" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>Penampakan Bulan Ditabrak Roket 4 Ton Elon Musk Sampai Bolong-Bolong</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 17:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>Roket SpaceX menghantam Bulan, Danuri merekam perubahan medan. Temuan ini penting untuk studi dampak benda buatan manusia di permukaan Bulan.</t>
+        </is>
+      </c>
+      <c r="F1276" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1276" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807132841-37-757418/penampakan-bulan-ditabrak-roket-4-ton-elon-musk-sampai-bolong-bolong</t>
+        </is>
+      </c>
+      <c r="H1276" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/danuri-merekam-momen-saat-tingkat-atas-roket-spacex-falcon-9-menghantam-permukaan-bulan-pada-tanggal-5-agustus-pukul-1534-wakt-1786084126735_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1276" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>Demo Besar-Besaran Tolak Data Center Raksasa, Warga Sudah Muak</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 17:05:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1277" t="inlineStr">
+        <is>
+          <t>Pembangunan pusat data Google di India ditentang aktivis lingkungan dan warga sekitar. Mereka menyoroti krisis air dan lingkungan.</t>
+        </is>
+      </c>
+      <c r="F1277" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1277" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807132141-37-757412/demo-besar-besaran-tolak-data-center-raksasa-warga-sudah-muak</t>
+        </is>
+      </c>
+      <c r="H1277" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/05/22/gedung-data-center-meta-di-mansfield-as-1779441817711_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1277" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>Erajaya Food dan Nourishment dan Oriental Kopi Jalin Kemitraan Strategis</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 16:49:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>PT Era Boga Nusantara dan Oriental Coffee International membentuk joint venture PT Era Oriental Kopi untuk ekspansi restoran di Indonesia, fokus Jabodetabek.</t>
+        </is>
+      </c>
+      <c r="F1278" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1278" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807162246-37-757491/erajaya-food-nourishment-dan-oriental-kopi-jalin-kemitraan-strategis</t>
+        </is>
+      </c>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/dok-erajaya-food-nourishment-1786096066750_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1278" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>700.000 Orang Tewas, Google Peringatkan Bencana Besar Lebih Cepat</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 16:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1279" t="inlineStr">
+        <is>
+          <t>Google meluncurkan WeatherNext, AI yang memprediksi badai tropis dengan lebih cepat. Simak selengkapnya!</t>
+        </is>
+      </c>
+      <c r="F1279" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1279" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807121851-37-757398/700000-orang-tewas-google-peringatkan-bencana-besar-lebih-cepat</t>
+        </is>
+      </c>
+      <c r="H1279" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/12/03/kondisi-setelah-siklon-ditwah-melanda-kawasan-niyamgamdora-sri-lanka-selasa-2122025-reutersakila-jayawardena-1764766482101_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1279" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>Krisis Menggila, HP Mahal Mendadak Laku Keras Diborong Warga</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 16:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1280" t="inlineStr">
+        <is>
+          <t>Pasar smartphone premium global tumbuh 5% YoY pada H1 2026, dengan Apple dan Samsung tetap dominan. Simak selengkapnya!</t>
+        </is>
+      </c>
+      <c r="F1280" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1280" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807122415-37-757400/krisis-menggila-hp-mahal-mendadak-laku-keras-diborong-warga</t>
+        </is>
+      </c>
+      <c r="H1280" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/10/07/jasa-service-hp-cnbc-indonesianovina-1759823129283_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1280" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>Harga Naik, Ini Alasan Banyak Orang Ganti HP Samsung Galaxy Z Fold8</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 15:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1281" t="inlineStr">
+        <is>
+          <t>Krisis chip memori global berdampak pada harga smartphone, termasuk Galaxy Z Fold8. Namun, HP ini tetap laku keras sampai cetak rekor.</t>
+        </is>
+      </c>
+      <c r="F1281" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1281" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807115948-37-757392/harga-naik-ini-alasan-banyak-orang-ganti-hp-samsung-galaxy-z-fold8</t>
+        </is>
+      </c>
+      <c r="H1281" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/18/samsung-galaxy-z-fold8-1784366205171_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1281" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>100 Spesies Terancam Punah, Leonardi DiCaprio Langsung Turun Tangan</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 14:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1282" t="inlineStr">
+        <is>
+          <t>Leonardo DiCaprio dan Jeff Bezos luncurkan inisiatif dengan dana Rp3,5 triliun untuk menyelamatkan 100 spesies terancam punah.</t>
+        </is>
+      </c>
+      <c r="F1282" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1282" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807114627-37-757380/100-spesies-terancam-punah-leonardi-dicaprio-langsung-turun-tangan</t>
+        </is>
+      </c>
+      <c r="H1282" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/01/12/leonardo-dicaprio-berpose-di-karpet-merah-pada-acara-golden-globes-ke-83-di-beverly-hills-california-as-minggu-1112026-reuters-1768186303176_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1282" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>VinFast Indonesia dan Danamon Perkuat Ekosistem Kendaraan Listrik di RI</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 14:40:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1283" t="inlineStr">
+        <is>
+          <t>VinFast Indonesia dan Bank Danamon tandatangani kerja sama pembiayaan dealer di GIIAS 2026. Kolaborasi ini dukung ekspansi dan ekosistem kendaraan listrik.</t>
+        </is>
+      </c>
+      <c r="F1283" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1283" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807143221-37-757449/vinfast-indonesia-danamon-perkuat-ekosistem-kendaraan-listrik-di-ri</t>
+        </is>
+      </c>
+      <c r="H1283" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/vinfast-1786088440435_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1283" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>267 Titik di Kaltim 'Gelap' Tak Ada Internet, Komdigi Buka Suara</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 14:05:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1284" t="inlineStr">
+        <is>
+          <t>Meskipun konektivitas di Kalimantan Timur mencapai 95,5%, masih ada 269 titik blank spot. Simak penjelasan Wamenkomdigi!</t>
+        </is>
+      </c>
+      <c r="F1284" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1284" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807114120-37-757379/267-titik-di-kaltim-gelap-tak-ada-internet-komdigi-buka-suara</t>
+        </is>
+      </c>
+      <c r="H1284" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/05/22/wakil-menteri-komunikasi-dan-digital-nezar-patria-saat-menyampaikan-pemaparan-dalam-jogja-financial-festival-2026-di-jogja-exp-1779442550629_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1284" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>Video: Inovasi Fintech Lending Atasi Gap Kredit UMKM Sebesar Rp2.400 T</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 13:53:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1285" t="inlineStr">
+        <is>
+          <t>Inovasi Fintech Lending Atasi Gap Kredit UMKM Yang Mencapai Rp 2.400 Triliun</t>
+        </is>
+      </c>
+      <c r="F1285" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1285" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807121240-39-757394/video-inovasi-fintech-lending-atasi-gap-kredit-umkm-sebesar-rp2400-t</t>
+        </is>
+      </c>
+      <c r="H1285" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/inovasi-fintech-lending-atasi-gap-kredit-umkm-yang-mencapai-rp-2400-triliun-1786085305978_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1285" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>Pencurian Terbesar Dalam Sejarah, Uang Rp 500 Miliar Lenyap Seketika</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 13:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr">
+        <is>
+          <t>Tahun 2026 tercatat sebagai pencurian kripto terburuk dalam sejarah. Kerugian lebih dari Rp500 miliar.</t>
+        </is>
+      </c>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1286" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807113510-37-757377/pencurian-terbesar-dalam-sejarah-uang-rp-500-miliar-lenyap-seketika</t>
+        </is>
+      </c>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2023/12/03/flexing-di-medsos-sasaran-empuk-penipu-online-kuras-rekening_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1286" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>Bulan Terus Menjauhi Bumi, Manusia Mulai Rasakan Dampaknya</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>Jarak Bumi ke Bulan sekitar 384.400 km dan terus menjauh 3,8 cm per tahun. Ini berdampak pada frekuensi Gerhana Matahari Total.</t>
+        </is>
+      </c>
+      <c r="F1287" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1287" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807113304-37-757374/bulan-terus-menjauhi-bumi-manusia-mulai-rasakan-dampaknya</t>
+        </is>
+      </c>
+      <c r="H1287" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/04/08/pemandangan-bumi-yang-sebagian-tersembunyi-di-balik-bulan-yang-ditangkap-melalui-jendela-pesawat-ruang-angkasa-orion-pada-puku-1775628749897_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1287" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>Ledakan Gempa Langit Terdengar di Mana-Mana, Ilmuwan Buka Suara</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 12:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>Fenomena "gempa langit" atau skyquake terus menjadi misteri. Penelitian terbaru menunjukkan asal-muasalnya.</t>
+        </is>
+      </c>
+      <c r="F1288" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1288" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807111947-37-757370/ledakan-gempa-langit-terdengar-di-mana-mana-ilmuwan-buka-suara</t>
+        </is>
+      </c>
+      <c r="H1288" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/08/26/badai-debu-menyelimuti-langit-di-paradise-valley-arizona-as-25-agustus-2025-abc-affiliate-knxv-via-reuters-1756193111443_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1288" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>Samsung F70 Pro Baru Rilis, HP Baterai 6.000 mAh Harga Rp 4 Jutaan</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 11:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>Samsung resmi luncurkan Galaxy F70 Pro di India. Ponsel ini hadir dengan baterai 6.000 mAh, layar AMOLED 6,7 inci, kamera 50 MP.</t>
+        </is>
+      </c>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1289" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260807110648-37-757368/samsung-f70-pro-baru-rilis-hp-baterai-6000-mah-harga-rp-4-jutaan</t>
+        </is>
+      </c>
+      <c r="H1289" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/galaxy-f70-pro-5g-1786076454500_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1289" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>Energi</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>Konsumsi Listrik SPKLU Melonjak, PLN Perluas Infrastruktur Pengisian Kendaraan Listrik</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:41:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>Erdy Nasrul</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Penggunaan kendaraan listrik di Indonesia menunjukkan pertumbuhan yang semakin kuat. Hal itu tercermin dari konsumsi listrik pada Stasiun Pengisian Kendaraan Listrik Umum (SPKLU) yang mencapai 62,4 juta...</t>
+        </is>
+      </c>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1290" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjem5d451/konsumsi-listrik-spklu-melonjak-pln-perluas-infrastruktur-pengisian-kendaraan-listrik</t>
+        </is>
+      </c>
+      <c r="H1290" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/petugas-spklu-mengisi-energi-listrik-ke-sebuah_260807214053-993.jpeg</t>
+        </is>
+      </c>
+      <c r="I1290" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Jakarta Kebakaran</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:29:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Jakarta di Gambir terbakar. Sebanyak 13 unit damkar dan 65 personel dikerahkan.</t>
+        </is>
+      </c>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1291" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264699/gedung-bapenda-dki-jakarta-kebakaran</t>
+        </is>
+      </c>
+      <c r="H1291" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/HYiZgk3x63v239p53K0KX2oQJvY=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318630/original/040776900_1786116540-Kebakaran.jpg</t>
+        </is>
+      </c>
+      <c r="I1291" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>Penampakan Febrie Adriansyah Usai 7 Jam Diperiksa Kejagung</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:38:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>Febrie meninggalkan ruang pemeriksaan sekitar pukul 20.30 WIB. Ia langsung menuju mobil tahanan.</t>
+        </is>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1292" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264672/penampakan-febrie-adriansyah-usai-7-jam-diperiksa-kejagung</t>
+        </is>
+      </c>
+      <c r="H1292" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/sp4SqvNV_83npEChYsHfHfViHdc=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318625/original/014147200_1786113402-IMG_3066.jpg</t>
+        </is>
+      </c>
+      <c r="I1292" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>Kuasa Hukum: Febrie Adriansyah Kooperatif Saat Diperiksa sebagai Tersangka</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:47:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>Kuasa hukum mantan Jampidsus Febrie Adriansyah menyatakan bahwa kliennya bersikap kooperatif saat menjalani pemeriksaan sebagai tersangka.</t>
+        </is>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1293" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/07/22433161/kuasa-hukum-febrie-adriansyah-kooperatif-saat-diperiksa-sebagai-tersangka</t>
+        </is>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/TjloeZKNzN-WVra0igWLvfg3HEc=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/07/6a75f51e10fa1.jpg</t>
+        </is>
+      </c>
+      <c r="I1293" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>Dilema Warga Kuranji Padang: Antara Normalisasi Sungai dan Pilihan Berat Relokasi</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:47:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>Warga Kuranji, Padang, Sumbar dilema dengan adanya aliran sungai Batang Guo yang jebol dan ancaman banjir susulan yang menghantui.</t>
+        </is>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1294" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/07/221736278/dilema-warga-kuranji-padang-antara-normalisasi-sungai-dan-pilihan-berat</t>
+        </is>
+      </c>
+      <c r="H1294" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/tmaICnT04aLuV7IPK9dU1SnRQ_g=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/07/6a75eea4b05f1.jpeg</t>
+        </is>
+      </c>
+      <c r="I1294" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>Keluarga Ungkap Kondisi Terkahir Kesehatan Yurizal saat Posting 8 Jam Menunggu di RS : Menahan Rasa Sakit</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:47:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>Keluarga mengungkapkan kondisi kesehatan Yurizal, pasien BPJS, saat terakhirnya sebelum menghembuskan nafas terakhir.</t>
+        </is>
+      </c>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1295" t="inlineStr">
+        <is>
+          <t>https://bandung.kompas.com/read/2026/08/07/214627678/keluarga-ungkap-kondisi-terkahir-kesehatan-yurizal-saat-posting-8-jam</t>
+        </is>
+      </c>
+      <c r="H1295" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/7lnn2eO2C64CMZyw4ySmKJcGGIg=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/06/6a7476b7ed27e.jpg</t>
+        </is>
+      </c>
+      <c r="I1295" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1191"/>
+  <autoFilter ref="A1:I1295"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 16:45 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-07.xlsx
+++ b/data/berita_2026-08-07.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1295</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1361</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1295"/>
+  <dimension ref="A1:I1361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -61298,8 +61298,3110 @@
         </is>
       </c>
     </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>Indonesia akhiri perlawanan sengit Vietnam 3-2</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:38:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>Tim nasional voli putri Indonesia mengakhiri perlawanan sengit dari timnas Vietnam, 3-2 (20-25, 18-25, 25-22, 25-20, ...</t>
+        </is>
+      </c>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1296" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685180/indonesia-akhiri-perlawanan-sengit-vietnam-3-2</t>
+        </is>
+      </c>
+      <c r="H1296" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/HPG0Fg1bIAAsUKg.jpg</t>
+        </is>
+      </c>
+      <c r="I1296" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>AI Cinefest 2026 himpun 1.111 film buatan AI dari seluruh Indonesia</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:36:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>Telkomsel bersama Huawei dan MiniMax menggelar kompetisi film pendek AI Cinefest 2026 yang menghimpun 1.111 karya film ...</t>
+        </is>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1297" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685177/ai-cinefest-2026-himpun-1111-film-buatan-ai-dari-seluruh-indonesia</t>
+        </is>
+      </c>
+      <c r="H1297" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000142174.jpg</t>
+        </is>
+      </c>
+      <c r="I1297" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>RS Pusri putus kerja sama dengan Dokter Tamara buntut hina pasien BPJS</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:36:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>ANTARA - Rumah Sakit Pusri Palembang mengakhiri kerja sama dengan dokter mitra yang diduga terlibat dalam polemik ...</t>
+        </is>
+      </c>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1298" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685175/rs-pusri-putus-kerja-sama-dengan-dokter-tamara-buntut-hina-pasien-bpjs</t>
+        </is>
+      </c>
+      <c r="H1298" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-07-232436.jpg</t>
+        </is>
+      </c>
+      <c r="I1298" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>Menkum minta penanganan laporan pelanggaran KI dipercepat</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:28:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>Menteri Hukum Supratman Andi Agtas meminta jajaran Kementerian Hukum mempercepat penanganan laporan dugaan pelanggaran ...</t>
+        </is>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1299" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685171/menkum-minta-penanganan-laporan-pelanggaran-ki-dipercepat</t>
+        </is>
+      </c>
+      <c r="H1299" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000475284.jpg</t>
+        </is>
+      </c>
+      <c r="I1299" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>LPKA Klas I Kupang prioritaskan pendidikan bagi anak binaan</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:25:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>ANTARA - Lembaga Pembinaan Khusus Anak (LPKA) Klas I Kupang memprioritaskan pendidikan bagi 37 anak binaan sebagai hak ...</t>
+        </is>
+      </c>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1300" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685161/lpka-klas-i-kupang-prioritaskan-pendidikan-bagi-anak-binaan</t>
+        </is>
+      </c>
+      <c r="H1300" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-07-230421.jpg</t>
+        </is>
+      </c>
+      <c r="I1300" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>Kepala Barantin pastikan layanan karantina optimal kawal ekspor udang</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:23:42 +0700</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>Kepala Badan Karantina Indonesia (Barantin) Abdul Kadir Karding memastikan layanan karantina berjalan optimal terhadap ...</t>
+        </is>
+      </c>
+      <c r="F1301" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1301" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685169/kepala-barantin-pastikan-layanan-karantina-optimal-kawal-ekspor-udang</t>
+        </is>
+      </c>
+      <c r="H1301" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1002919266.jpg</t>
+        </is>
+      </c>
+      <c r="I1301" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>KY ungkap beda pendapat komisioner soal tiga calon hakim agung</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:18:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>Komisi Yudisial (KY) mengungkap adanya perbedaan pendapat di antara komisioner dalam penetapan kelulusan tiga calon ...</t>
+        </is>
+      </c>
+      <c r="F1302" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1302" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685165/ky-ungkap-beda-pendapat-komisioner-soal-tiga-calon-hakim-agung</t>
+        </is>
+      </c>
+      <c r="H1302" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_4555.jpeg</t>
+        </is>
+      </c>
+      <c r="I1302" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>Gerakan Langit Biru AHY di Pulau Madura berlanjut</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:18:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1303" t="inlineStr">
+        <is>
+          <t>Gerakan Langit Biru Indonesia ASRI, yakni  pendistribusian bantuan air bersih ke desa-desa terdampak kekeringan di ...</t>
+        </is>
+      </c>
+      <c r="F1303" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1303" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685164/gerakan-langit-biru-ahy-di-pulau-madura-berlanjut</t>
+        </is>
+      </c>
+      <c r="H1303" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Langit-Biru-Madura.jpg</t>
+        </is>
+      </c>
+      <c r="I1303" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>Aldila fokus adaptasi lapangan jelang laga pembuka WTA 1000 Toronto</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:14:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>Petenis ganda putri Indonesia Aldila Sutjiadi memfokuskan persiapan pada adaptasi lapangan menjelang laga pembuka ...</t>
+        </is>
+      </c>
+      <c r="F1304" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1304" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685159/aldila-fokus-adaptasi-lapangan-jelang-laga-pembuka-wta-1000-toronto</t>
+        </is>
+      </c>
+      <c r="H1304" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/09/12/Aldila.jpg</t>
+        </is>
+      </c>
+      <c r="I1304" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>Bea Cukai-Polisi gagalkan penyelundupan 10,1 kg ganja di bandara Bali</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:10:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>ANTARA - Kantor Pengawasan dan Pelayanan Bea Cukai (KPPBC) Ngurah Rai bersama Satuan Reserse Narkoba Polres Bandara I ...</t>
+        </is>
+      </c>
+      <c r="F1305" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1305" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685020/bea-cukai-polisi-gagalkan-penyelundupan-101-kg-ganja-di-bandara-bali</t>
+        </is>
+      </c>
+      <c r="H1305" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/BEA-CUKAI-POLISI-GAGALKAN-PENYELUNDUPAN-10-1-KG-GANJA-DI-BANDARA-BALI_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1305" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>PSSI akan lakukan evaluasi setelah Indonesia gagal tembus semifinal</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:09:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1306" t="inlineStr">
+        <is>
+          <t>Ketua Umum PSSI Erick Thohir mengungkapkan pihaknya akan melakukan evaluasi terhadap hasil timnas Indonesia yang gagal ...</t>
+        </is>
+      </c>
+      <c r="F1306" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1306" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685155/pssi-akan-lakukan-evaluasi-setelah-indonesia-gagal-tembus-semifinal</t>
+        </is>
+      </c>
+      <c r="H1306" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/HPILtZ8aEAI6W61.jpg</t>
+        </is>
+      </c>
+      <c r="I1306" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>INDEF sebut PFII syariah bisa jadi daya tawar pembeda</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:07:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1307" t="inlineStr">
+        <is>
+          <t>Ketua Center for Sharia Economic Development (CSED) Institute for Development of Economics and Finance (INDEF) Nur ...</t>
+        </is>
+      </c>
+      <c r="F1307" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1307" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685152/indef-sebut-pfii-syariah-bisa-jadi-daya-tawar-pembeda</t>
+        </is>
+      </c>
+      <c r="H1307" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_20260807_225436.jpg</t>
+        </is>
+      </c>
+      <c r="I1307" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>OJK: Sektor jasa keuangan Sumbar tumbuh positif pada triwulan II 2026</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:05:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1308" t="inlineStr">
+        <is>
+          <t>ANTARA - Otoritas Jasa Keuangan (OJK) mencatat kinerja sektor jasa keuangan di Sumatera Barat tetap tumbuh positif pada ...</t>
+        </is>
+      </c>
+      <c r="F1308" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1308" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685116/ojk-sektor-jasa-keuangan-sumbar-tumbuh-positif-pada-triwulan-ii-2026</t>
+        </is>
+      </c>
+      <c r="H1308" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/OJK-SEKTOR-JASA-KEUANGAN-SUMBAR-TUMBUH-POSITIF-PADA-TRIWULAN-II-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I1308" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>Kreativitas manusia jadi unsur penting dalam membuat film dengan AI</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:04:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1309" t="inlineStr">
+        <is>
+          <t>Kreativitas dari buah pikiran manusia dinilai tetap menjadi unsur penting dalam membuat film menggunakan teknologi ...</t>
+        </is>
+      </c>
+      <c r="F1309" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1309" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685148/kreativitas-manusia-jadi-unsur-penting-dalam-membuat-film-dengan-ai</t>
+        </is>
+      </c>
+      <c r="H1309" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000142158.jpg</t>
+        </is>
+      </c>
+      <c r="I1309" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>TNBTS: kebakaran di Bromo diduga sisa perapian orang di Bantengan</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:02:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1310" t="inlineStr">
+        <is>
+          <t>ANTARA - ‎Kebakaran yang melanda kawasan Gunung Bromo, Jawa Timur, pihak TNBTS menduga akibat dipicu aktivitas ...</t>
+        </is>
+      </c>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1310" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685145/tnbts-kebakaran-di-bromo-diduga-sisa-perapian-orang-di-bantengan</t>
+        </is>
+      </c>
+      <c r="H1310" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-07-225216.jpg</t>
+        </is>
+      </c>
+      <c r="I1310" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>Menghadap Wamensos, 4 bupati siap bangun Sekolah Rakyat permanen</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:00:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>Empat kepala daerah dari Agam, Buton Selatan, Kutai Kertanegara, dan Buru datang ke kantor Kemensos untuk menegaskan ...</t>
+        </is>
+      </c>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1311" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685147/menghadap-wamensos-4-bupati-siap-bangun-sekolah-rakyat-permanen</t>
+        </is>
+      </c>
+      <c r="H1311" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-20.24.12-1.jpeg</t>
+        </is>
+      </c>
+      <c r="I1311" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>Prabowo sebut pendapatan Danantara dilaporkan naik hingga 400 persen</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>ANTARA - Presiden Prabowo Subianto menyebut Badan Pengelola Investasi (BPI) Danantara mencatat peningkatan ...</t>
+        </is>
+      </c>
+      <c r="F1312" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1312" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685047/prabowo-sebut-pendapatan-danantara-dilaporkan-naik-hingga-400-persen</t>
+        </is>
+      </c>
+      <c r="H1312" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PRABOWO-SEBUT-PENDAPATAN-DANANTARA-DILAPORKAN-NAIK-HINGGA-400-PERSEN.jpg</t>
+        </is>
+      </c>
+      <c r="I1312" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>Setengah abad, Bahlil Rilis buku "10 Karya Nyata untuk Negeri"</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:59:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia meluncurkan Buku 10 Karya Nyata untuk Negeri: ...</t>
+        </is>
+      </c>
+      <c r="F1313" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1313" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685113/setengah-abad-bahlil-rilis-buku-10-karya-nyata-untuk-negeri</t>
+        </is>
+      </c>
+      <c r="H1313" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SETENGAH-ABAD-BAHLIL-RILIS-BUKU-10-KARYA-NYATA-UNTUK-NEGERI_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1313" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>BI: Sektor perumahan dan kawasan industri perkokoh investasi Banten</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:55:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr">
+        <is>
+          <t>Kantor Perwakilan Bank Indonesia (BI) Provinsi Banten mencatat bahwa realisasi investasi di wilayah tersebut didominasi ...</t>
+        </is>
+      </c>
+      <c r="F1314" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1314" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685141/bi-sektor-perumahan-dan-kawasan-industri-perkokoh-investasi-banten</t>
+        </is>
+      </c>
+      <c r="H1314" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000879852.jpg</t>
+        </is>
+      </c>
+      <c r="I1314" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>Wamen PKP usulkan Perumnas perkuat penyediaan hunian strategis</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr">
+        <is>
+          <t>ANTARA - Wakil Menteri Perumahan dan Kawasan Permukiman (PKP) Fahri Hamzah meminta Perum Perumnas menjadi off ...</t>
+        </is>
+      </c>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1315" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685016/wamen-pkp-usulkan-perumnas-perkuat-penyediaan-hunian-strategis</t>
+        </is>
+      </c>
+      <c r="H1315" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/WAMEN-PKP-USULKAN-PERUMNAS-PERKUAT-PENYEDIAAN-HUNIAN-STRATEGIS.jpg</t>
+        </is>
+      </c>
+      <c r="I1315" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>Nissan ramaikan GIIAS 2026 melalui Serena e-Power</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:52:42 +0700</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>PT Nissan Motor Distributor Indonesia (NMDI) kembali ikut meramaikan pameran otomotif Gaikindo Indonesia Internaional ...</t>
+        </is>
+      </c>
+      <c r="F1316" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1316" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5685137/nissan-ramaikan-giias-2026-melalui-serena-e-power</t>
+        </is>
+      </c>
+      <c r="H1316" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-22.17.18.jpeg</t>
+        </is>
+      </c>
+      <c r="I1316" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>Khofifah tinjau kebakaran Bromo, area terbakar meluas capai 176 hektar</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:50:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>ANTARA - ‎‎Gubernur Jawa Timur Khofifah Indar Parawansa meninjau langsung penanganan kebakaran di kawasan ...</t>
+        </is>
+      </c>
+      <c r="F1317" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1317" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685132/khofifah-tinjau-kebakaran-bromo-area-terbakar-meluas-capai-176-hektar</t>
+        </is>
+      </c>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-07-224200.jpg</t>
+        </is>
+      </c>
+      <c r="I1317" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>Direktur STB: Kelola pengeluaran kunci agar tak bergantung "paylater"</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:48:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>Managing Director perusahaan induk investasi dan penyedia layanan finansial PT Samuel Tumbuh Bersama (STB) Tae Yong ...</t>
+        </is>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1318" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685136/direktur-stb-kelola-pengeluaran-kunci-agar-tak-bergantung-paylater</t>
+        </is>
+      </c>
+      <c r="H1318" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000178486.jpg</t>
+        </is>
+      </c>
+      <c r="I1318" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>BGN: 950 dapur MBG diduga tak layak higienis dan sanitasi</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:47:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>ANTARA - Kepala Badan Gizi Nasional (BGN) Sudaryono menyebut 950 Satuan Pelayanan Pemenuhan Gizi (SPPG) atau dapur ...</t>
+        </is>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1319" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685103/bgn-950-dapur-mbg-diduga-tak-layak-higienis-dan-sanitasi</t>
+        </is>
+      </c>
+      <c r="H1319" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/BGN-950-DAPUR-MBG-DIDUGA-TAK-LAYAK-HIGIENIS-DAN-SANITASI.jpg</t>
+        </is>
+      </c>
+      <c r="I1319" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>Prabowo sebut perjalanan hidup Bahlil jadi inspirasi generasi muda</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:46:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>ANTARA - Presiden RI Prabowo Subianto mengatakan Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia dapat ...</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1320" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685029/prabowo-sebut-perjalanan-hidup-bahlil-jadi-inspirasi-generasi-muda</t>
+        </is>
+      </c>
+      <c r="H1320" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_PRABOWO-SEBUT-PERJALANAN-HIDUP-BAHLIL-JADI-INSPIRASI-GENERASI-MUDA.jpg</t>
+        </is>
+      </c>
+      <c r="I1320" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>Wamendikdasmen ajak Pemkab Bungo tingkatkan APK kurangi ATS lewat PJJ</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:45:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Pendidikan Dasar dan Menengah (Wamendikdasmen) Fajar Riza Ul Haq mengajak Pemerintah Kabupaten Bungo, ...</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1321" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685128/wamendikdasmen-ajak-pemkab-bungo-tingkatkan-apk-kurangi-ats-lewat-pjj</t>
+        </is>
+      </c>
+      <c r="H1321" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000229856.jpg</t>
+        </is>
+      </c>
+      <c r="I1321" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>Perwira polisi terlibat kecelakaan tewaskan balita di Bone ditahan</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:44:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>Polres Bone menahan seorang perwira polisi berinisial MA berpangkat Inspektur Polisi Dua (Ipda) yang terlibat ...</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1322" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685124/perwira-polisi-terlibat-kecelakaan-tewaskan-balita-di-bone-ditahan</t>
+        </is>
+      </c>
+      <c r="H1322" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/kasus-polisi-tabrak-bocah-di-bone-dok-polisi.jpeg</t>
+        </is>
+      </c>
+      <c r="I1322" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>Kemensos kebut pembangunan Sekolah Rakyat permanen lewat TP2SR</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:42:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>Kementerian Sosial (Kemensos) membentuk Tim Percepatan Pembangunan Sekolah Rakyat (TP2SR) sebagai tim ad hoc untuk ...</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1323" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685120/kemensos-kebut-pembangunan-sekolah-rakyat-permanen-lewat-tp2sr</t>
+        </is>
+      </c>
+      <c r="H1323" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-20.24.12.jpeg</t>
+        </is>
+      </c>
+      <c r="I1323" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>Kejagung: Febrio Adiono Pegawai, Bukan Jaksa</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:04:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>Febrio Adiono, staf Kejagung, terlibat dalam kasus kematian misterius Sutrimo di depan klinik. Polisi selidiki penyebab kematian dan kumpulkan saksi.</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1324" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609321/kejagung-febrio-adiono-pegawai-bukan-jaksa</t>
+        </is>
+      </c>
+      <c r="H1324" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/27/puslabfor-polri-menggelar-olah-tempat-kejadian-perkara-tkp-di-klinik-mordent-kawasan-kebayoran-baru-jakarta-selatan-1785134569014_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1324" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>100 Personel Damkar Dikerahkan Padamkan Kebakaran Hebat di Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:54:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda gedung Bapenda DKI Jakarta, memicu pengerahan 20 unit pemadam. Asap membubung tinggi, penyebab dan korban masih belum diketahui.</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1325" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609314/100-personel-damkar-dikerahkan-padamkan-kebakaran-hebat-di-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H1325" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/10/17/ilustrasi-kebakaran_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1325" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>Bahtra Banong Raih 'Legislator Aspiratif Bidang Keadilan Sosial-Agraria' detiktimur Awards 2026</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:51:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>Tim detikSulsel</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Komisi II DPR RI, Bahtra Banong, raih detiktimur Awards 2026 sebagai Legislator Aspiratif. Ia fokus pada keadilan sosial dan agraria di Indonesia.</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1326" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609313/bahtra-banong-raih-legislator-aspiratif-bidang-keadilan-sosial-agraria-detiktimur-awards-2026</t>
+        </is>
+      </c>
+      <c r="H1326" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/detiktimur-awards-bahtra-banong-1786111191099_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1326" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>Rudianto Lallo Dianugerahi detiktimur Awards 2026 'Legislator Pengawal Supremasi Hukum'</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:46:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>Syachrul Arsyad</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>Anggota DPR Rudianto Lallo menerima detiktimur Awards 2026 sebagai Legislator Pengawal Supremasi Hukum atas dedikasinya memberikan bantuan hukum ke masyarakat.</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1327" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609309/rudianto-lallo-dianugerahi-detiktimur-awards-2026-legislator-pengawal-supremasi-hukum</t>
+        </is>
+      </c>
+      <c r="H1327" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/detiktimur-awards-rudianto-lallo-1786110858616_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1327" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>Cerita Local Hero Pertamina Bangun Kemandirian Energi Desa</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:34:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>Annisa Sekar Melati</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>Alfredo dan Burhanudin, local hero Program Desa Energi Berdikari, membawa perubahan dengan akses air bersih dan energi terbarukan.</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1328" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609294/cerita-local-hero-pertamina-bangun-kemandirian-energi-desa</t>
+        </is>
+      </c>
+      <c r="H1328" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/pertamina-1786116722039.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1328" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI di Gambir Jakpus Kebakaran</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:33:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda gedung Bapenda DKI Jakarta. Personel damkar masih berupaya memadamkan api. Penyebab dan korban belum diketahui.</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1329" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609292/gedung-bapenda-dki-di-gambir-jakpus-kebakaran</t>
+        </is>
+      </c>
+      <c r="H1329" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/11/13/ilustrasi-api_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1329" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>Danantara Gandeng JBS Perkuat Investasi Sektor Protein Indonesia</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:46:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>Danantara menjalin kemitraan dengan JBS Group, investasi US$ 2,5 miliar untuk 25% kepemilikan di JV Australia dan Selandia Baru, mendukung sektor protein.</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1330" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609310/danantara-gandeng-jbs-perkuat-investasi-sektor-protein-indonesia</t>
+        </is>
+      </c>
+      <c r="H1330" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/06/30/wisma-danantara-indonesia-1751283332958_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1330" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>Marcos Tjung Garap Video Klip Warna Warni Indonesia Sehari: Luar Biasa</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:30:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>Video klip Warna Warni Indonesia garapan Marcos Tjung melibatkan delapan penyanyi top. Lagu ini merayakan keberagaman dan semangat persatuan Indonesia.</t>
+        </is>
+      </c>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1331" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/music/d-8609289/marcos-tjung-garap-video-klip-warna-warni-indonesia-sehari-luar-biasa</t>
+        </is>
+      </c>
+      <c r="H1331" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/marcos-tjung-1786116589482_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1331" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>Arafah Rianti Terus Ekspansi Usaha Warnet-Rental PS</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:02:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>Artis Arafah Rianti hadir dengan kabar baru. Ia mengekspansi usaha warnet dan rental PS-nya.</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1332" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8608180/arafah-rianti-terus-ekspansi-usaha-warnet-rental-ps</t>
+        </is>
+      </c>
+      <c r="H1332" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/arafah-rianti-1786075896543_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1332" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>Pengacara Asisten Nikita Mirzani Ungkap Pemicu Kekecewaan di Sidang PK TPPU</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:01:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>Asisten Nikita Mirzani, Mail Syahputra, ajukan PK atas kasus pemerasan dan TPPU. Kuasa hukum ungkap pemicu kekecewaan dalam sidang.</t>
+        </is>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1333" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8608870/pengacara-asisten-nikita-mirzani-ungkap-pemicu-kekecewaan-di-sidang-pk-tppu</t>
+        </is>
+      </c>
+      <c r="H1333" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/07/24/nikita-mirzani-jalani-sidang-ttpu-1753328999091_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1333" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>Momen Api Karhutla Membara di Alun-Alun Suryakencana Gede Pangrango</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:16:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>Kebakaran lahan melanda kawasan Alun-alun Suryakencana di Taman Nasional Gunung Gede Pangrango (TNGGP), Cianjur, Jawa Barat, Kamis (6/8).</t>
+        </is>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1334" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807192715-24-1389919/momen-api-karhutla-membara-di-alun-alun-suryakencana-gede-pangrango</t>
+        </is>
+      </c>
+      <c r="H1334" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/api-lahap-alun-alun-suryakencana-diduga-akibat-kemarau-1786107276515_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1334" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>Gempa Laut Jawa Malam Ini: Guncangan Terasa di Jepara, Demak, Batang</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:02:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>Gempa magnitudo 5,0 terjadi di Laut Jawa malam ini, tidak berpotensi tsunami. Guncangan dirasakan di Jepara dan Demak, hingga Batang.</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1335" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807221317-20-1389978/gempa-laut-jawa-malam-ini-guncangan-terasa-di-jepara-demak-batang</t>
+        </is>
+      </c>
+      <c r="H1335" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2018/08/17/1db060af-1933-4880-a245-a4ff9edc6a81_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1335" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>100 Personel Dikerahkan Atasi Kebakaran Gedung Dinas Teknis Abdul Muis</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:45:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda Gedung Dinas Teknis Abdul Muis di Jakarta Pusat, J umat malam. 21 unit pemadam/100 personel dikerahkan untuk memadamkan api.</t>
+        </is>
+      </c>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1336" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807223646-20-1389980/100-personel-dikerahkan-atasi-kebakaran-gedung-dinas-teknis-abdul-muis</t>
+        </is>
+      </c>
+      <c r="H1336" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/05/30/ilustrasi-kebakaran-5_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1336" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>UPDATE Kebakaran Gedung Bapenda DKI: Api Membesar di Lantai Paling Atas, Puing Berjatuhan</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:29:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>Gedung Badan Pendapatan Daerah(Bapenda) DKI Jakarta dilalap api pada Jumat(7/8/2026) malam.</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1337" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865541/update-kebakaran-gedung-bapenda-dki-api-membesar-di-lantai-paling-atas-puing-berjatuhan</t>
+        </is>
+      </c>
+      <c r="H1337" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/vCWaggZXVG9j8HCC3w7rBy8DrbY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kebakaran-di-gedung-bapenda-dki-jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I1337" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>Golkar Usul Jabatan Wakil Kepala Daerah Dihapus, Klaim Bisa Tekan Konflik dan Biaya Politik</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:23:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>Golkar mengusulkan jabatan wakil kepala daerah dihapus dari Pilkada karena dinilai memicu konflik dan membebani biaya politik.</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1338" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865540/golkar-usul-jabatan-wakil-kepala-daerah-dihapus-klaim-bisa-tekan-konflik-dan-biaya-politik</t>
+        </is>
+      </c>
+      <c r="H1338" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/n4f-DiF2fXuszFf1sIRByQSzGHY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Wakil-Ketua-Badan-Legislasi-Baleg-DPR-RI-Ahmad-Doli-Kurnia.jpg</t>
+        </is>
+      </c>
+      <c r="I1338" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>1.155 Mahasiswa Indonesia Kuliah di Thailand, Pilihan Studi di Asean Makin Beragam</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:13:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>Sebanyak 1.155 mahasiswa Indonesia tercatat menempuh pendidikan di Thailand hingga 2025, menunjukkan semakin terbukanya pilihan studi.</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1339" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865539/1155-mahasiswa-indonesia-kuliah-di-thailand-pilihan-studi-di-asean-makin-beragam</t>
+        </is>
+      </c>
+      <c r="H1339" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ncXvUod70I_NWVHp9nPvrNhuX5Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-mahasiswa-kuliah-di-luar-negeri.jpg</t>
+        </is>
+      </c>
+      <c r="I1339" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>Jadwal Semifinal Korea Masters 2026: Yuta/Maya Incar Back to Back Final, Malaysia Bidik Derbi</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:10:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>Semifinal Korea Masters 2026 menghadirkan misi berbeda dari Jepang, Malaysia, dan Korea Selatan untuk sama-sama lolos ke final.</t>
+        </is>
+      </c>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1340" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865538/jadwal-semifinal-korea-masters-2026-yutamaya-incar-back-to-back-final-malaysia-bidik-derbi</t>
+        </is>
+      </c>
+      <c r="H1340" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/kCgeNAywY4bB7c1l4koRAi22PfE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/profil-maya-taguchi-tandem-anyar-yuta-watanabe-di-sektor-ganda-campuran-jepang.jpg</t>
+        </is>
+      </c>
+      <c r="I1340" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>Lika Liku Perjalanan Joanna di Modeling dan Mimpinya Mengangkat Identitas Indonesia ke Kancah Global</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:08:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>Jejak modeling Indonesia dari pionir Non Kawilarang hingga generasi baru Joanna Adelaide yang membawa identitas lokal ke global.</t>
+        </is>
+      </c>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1341" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865537/lika-liku-perjalanan-joanna-di-modeling-dan-mimpinya-mengangkat-identitas-indonesia-ke-kancah-global</t>
+        </is>
+      </c>
+      <c r="H1341" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/u1YW2Lk8dlDoOyAzBtxIln7NMOc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/momen-menteri-dan-istri-pejabat-negara-catwalk-di-istana-berkebaya_20230806_210137.jpg</t>
+        </is>
+      </c>
+      <c r="I1341" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>Idrus Marham Nilai Kabinet Bayangan Bagian dari Dinamika Demokrasi</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:07:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>Idrus Marham menilai pembentukan Kabinet Bayangan oleh koalisi masyarakat sipil merupakan bagian dari dinamika demokrasi dan hak warga.</t>
+        </is>
+      </c>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1342" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865536/idrus-marham-nilai-kabinet-bayangan-bagian-dari-dinamika-demokrasi</t>
+        </is>
+      </c>
+      <c r="H1342" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/fEQ4y2P9_Tdpmm4P3Yndltf76PE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/wawancara-khusus-ketua-dewan-pembina-bappilu-golkar-idrus-marham_20240809_114219.jpg</t>
+        </is>
+      </c>
+      <c r="I1342" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>Pengamat Politik Unas: Publik Ingin Jangan Ada Pihak yang 'Dilindungi' dalam Kasus Eks Jampidsus</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:01:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>publik ingin kasus dugaan korupsi dan TPPU eks Jampidsus Febrie Adriansyah diusut tuntas tanpa ada pihak yang dilindungi.</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1343" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865535/pengamat-politik-unas-publik-ingin-jangan-ada-pihak-yang-dilindungi-dalam-kasus-eks-jampidsus</t>
+        </is>
+      </c>
+      <c r="H1343" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/7nYnvNOC8BdbFnfyWZMwIUfCcqI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/diskusi-bertajuk-1.jpg</t>
+        </is>
+      </c>
+      <c r="I1343" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>Kronologi Pria Bunuh Mantan Istri di Pekanbaru, Pelaku Bacok Wajah Korban Setelah Terlibat Cekcok</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:52:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>Marhalim (64) membacok wajah mantan istrinya Rosdiana (55) hingga tewas di Tuah Madani, Kota Pekanbaru, Riau, Jumat (7/8/2026) pagi.</t>
+        </is>
+      </c>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1344" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865534/kronologi-pria-bunuh-mantan-istri-di-pekanbaru-pelaku-bacok-wajah-korban-setelah-terlibat-cekcok</t>
+        </is>
+      </c>
+      <c r="H1344" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0vnfr07ygtSQr0kVzLyuJpOqNYY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ilustrasi-pembunuhan-wae-lah.jpg</t>
+        </is>
+      </c>
+      <c r="I1344" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>Wacana Pilkada Tanpa Wakil Berpotensi Jadi Pintu Masuk Pemilihan Lewat DPRD</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:51:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>Usulan Pilkada tanpa wakil dinilai bukan sekadar perubahan teknis, tetapi berpotensi mengubah arah demokrasi daerah secara bertahap.</t>
+        </is>
+      </c>
+      <c r="F1345" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1345" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865533/wacana-pilkada-tanpa-wakil-berpotensi-jadi-pintu-masuk-pemilihan-lewat-dprd</t>
+        </is>
+      </c>
+      <c r="H1345" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GZLuQllSU5AIAGFRMXJDUPrXhnQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Simulasi-Pemungutan-Suara-Pilgub-Jakarta_20241117_160050.jpg</t>
+        </is>
+      </c>
+      <c r="I1345" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>Apa Kita Benar-Benar Butuh Tidur 8 Jam?</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:47:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr">
+        <is>
+          <t>Politisi atau CEO sering mengeklaim hanya punya sedikit waktu untuk tidur, bahkan hanya sempat tidur 3 jam di malam hari. Jika mereka…</t>
+        </is>
+      </c>
+      <c r="F1346" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1346" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865532/apa-kita-benar-benar-butuh-tidur-8-jam</t>
+        </is>
+      </c>
+      <c r="H1346" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qPKMk6l8QMnnSYy7E7E28OXgKDo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/BDeutsche-Welle76146878_403.jpg.jpg</t>
+        </is>
+      </c>
+      <c r="I1346" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>Pemulihan Ekosistem Laut Bali Barat Diharapkan Dukung Pariwisata Pesisir</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:46:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1347" t="inlineStr">
+        <is>
+          <t>struktur fisik terumbu karang di laut Bali Barat yang mengalami kerusakan direhabilitasi guna mengembalikan habitat alami.</t>
+        </is>
+      </c>
+      <c r="F1347" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1347" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865531/pemulihan-ekosistem-laut-bali-barat-diharapkan-dukung-pariwisata-pesisir</t>
+        </is>
+      </c>
+      <c r="H1347" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/L1ie-WMdsyx4zIzhCDrtJEx2g_E=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/dca-bantu-ekosistem.jpg</t>
+        </is>
+      </c>
+      <c r="I1347" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>BREAKING NEWS Gedung Bapenda DKI Jakarta Terbakar, Api dan Asap Hitam Membumbung Tinggi</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:40:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1348" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta di Jalan Abdul Muis, Petojo.</t>
+        </is>
+      </c>
+      <c r="F1348" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1348" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865530/breaking-news-gedung-bapenda-dki-jakarta-terbakar-api-dan-asap-hitam-membumbung-tinggi</t>
+        </is>
+      </c>
+      <c r="H1348" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/3nU5duk4s3XXHJSRQYafr_rV9FE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kebakaran-di-gedung-bapenda-dki.jpg</t>
+        </is>
+      </c>
+      <c r="I1348" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>Krisis Kemanusiaan Palestina Makin Dalam, 300 Anak Tewas di Gaza</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:39:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1349" t="inlineStr">
+        <is>
+          <t>UNICEF mencatat 300 anak tewas di Gaza dalam 300 hari. Di Tepi Barat, serangan pemukim dan penutupan akses terus menambah krisis</t>
+        </is>
+      </c>
+      <c r="F1349" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1349" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865529/krisis-kemanusiaan-palestina-makin-dalam-300-anak-tewas-di-gaza</t>
+        </is>
+      </c>
+      <c r="H1349" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Ztk0o1a2h3t-EQaaVSlhpEUMm14=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/bocah-berusia-13-tahun-dari-Kota-Gaza-yang.jpg</t>
+        </is>
+      </c>
+      <c r="I1349" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>Klasemen Akhir Grup A Piala AFF 2026: Kegagalan ke-6 Timnas Indonesia Melaju ke Semifinal</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:38:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1350" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia gagal ke semifinal Piala AFF 2026 setelah ditahan Singapura 1-1 dan finis di peringkat ketiga Grup A dengan 7 poin.</t>
+        </is>
+      </c>
+      <c r="F1350" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1350" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865528/klasemen-akhir-grup-a-piala-aff-2026-kegagalan-ke-6-timnas-indonesia-melaju-ke-semifinal</t>
+        </is>
+      </c>
+      <c r="H1350" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1a7ILPPDpySjbwe7SeQea4Z15Rg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Timnas-Indonesia-Dicukur-Timnas-Vietnam-3-0_20260804_065849.jpg</t>
+        </is>
+      </c>
+      <c r="I1350" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>Exam Concert Jadi Pelepas Penat usai Ujian, Yovie dan Nuno Hibur Mahasiswa Budi Luhur University</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:25:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1351" t="inlineStr">
+        <is>
+          <t>After Exam Concert dengan line up Yovie &amp; Nuno digelar untuk menjaga keseimbangan akademis dan kesehatan mental mahasiswa.</t>
+        </is>
+      </c>
+      <c r="F1351" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1351" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865527/exam-concert-jadi-pelepas-penat-usai-ujian-yovie-nuno-hibur-mahasiswa-budi-luhur-university</t>
+        </is>
+      </c>
+      <c r="H1351" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1QPTDghBoKYDEzDSOlMPsaaK9b0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Yovie-Nuno-1234.jpg</t>
+        </is>
+      </c>
+      <c r="I1351" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>Klaim Kriminalisasi Febrie Adriansyah Dinilai Wajar, Pakar Hukum: Dulu Kerap Lakukan Hal Serupa</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:13:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1352" t="inlineStr">
+        <is>
+          <t>Pakar Hukum UMJ Chairul Huda menilai pernyataan Febrie Adriansyah yang mengaku dikriminalisasi merupakan hal yang wajar disampaikan.</t>
+        </is>
+      </c>
+      <c r="F1352" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1352" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865526/klaim-kriminalisasi-febrie-adriansyah-dinilai-wajar-pakar-hukum-dulu-kerap-lakukan-hal-serupa</t>
+        </is>
+      </c>
+      <c r="H1352" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Z8LfULQiAjAelAU76TuRVZDVlnY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Febrie-Adriansyah-Jalani-Pemeriksaan-Lanjutan-Kasus-TPPU_20260807_134518.jpg</t>
+        </is>
+      </c>
+      <c r="I1352" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>Mobil Terjun ke Jurang 250 Meter di India, Lima Orang Tewas Termasuk Balita</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:12:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1353" t="inlineStr">
+        <is>
+          <t>Lima orang tewas setelah mobil Bolero terjun ke jurang sedalam hampir 250 meter di Uttarakhand India.</t>
+        </is>
+      </c>
+      <c r="F1353" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1353" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865525/mobil-terjun-ke-jurang-250-meter-di-india-lima-orang-tewas-termasuk-balita</t>
+        </is>
+      </c>
+      <c r="H1353" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/fye_UtxGjhYnqU3NPrNAQhorVCE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/lakalatasindia22222.jpg</t>
+        </is>
+      </c>
+      <c r="I1353" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>Eks Penyidik KPK Nilai Kasus Dugaan Korupsi dan TPPU Eks Jampidsus Perlu Dikembangkan ke Segala Arah</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:04:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1354" t="inlineStr">
+        <is>
+          <t>Mantan Penyidik KPK Yudi Purnomo Harahap menilai kasus dugaan korupsi dan TPPU yang menjerat eks Jampidsus Febrie Adriansyah perlu dikembangkan.</t>
+        </is>
+      </c>
+      <c r="F1354" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1354" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865524/eks-penyidik-kpk-nilai-kasus-dugaan-korupsi-dan-tppu-eks-jampidsus-perlu-dikembangkan-ke-segala-arah</t>
+        </is>
+      </c>
+      <c r="H1354" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8OfEROsNAENYYSUhKhNzr11IIxM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/diskusi-mencari-aktor-di-balik.jpg</t>
+        </is>
+      </c>
+      <c r="I1354" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>Niat Bayar COD Rp93 Ribu, Wanita di Palembang Salah Transfer Rp93 Juta, Uangnya Dihabiskan Kurir</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:02:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1355" t="inlineStr">
+        <is>
+          <t>NI seharusnya Rp93 ribu, namun justru mengirim uang sebesar Rp93 juta. Nahas, uang tersebut tidak dikembalikan oleh kurir paket.</t>
+        </is>
+      </c>
+      <c r="F1355" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1355" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865523/niat-bayar-cod-rp93-ribu-wanita-di-palembang-salah-transfer-rp93-juta-uangnya-dihabiskan-kurir</t>
+        </is>
+      </c>
+      <c r="H1355" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/jUb25Pvl71aBZZHrea6vweJM08g=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/DITAHAN-Kurir-paket.jpg</t>
+        </is>
+      </c>
+      <c r="I1355" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>Hasil Akhir Timnas Indonesia vs Singapura 1-1: Wasit Kontroversi, Skuad Garuda Gagal ke Semifinal</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:58:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1356" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia gagal ke semifinal Piala AFF 2026 seusai ditahan imbang Singapura 1-1 yang diwarnai kontroversi wasit asal Oman.</t>
+        </is>
+      </c>
+      <c r="F1356" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1356" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865522/hasil-akhir-timnas-indonesia-vs-singapura-1-1-wasit-kontroversi-skuad-garuda-gagal-ke-semifinal</t>
+        </is>
+      </c>
+      <c r="H1356" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tZqFKgwVQ5eW_YBK_O5n7jSWMXA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Timnas-Indonesia-Dicukur-Timnas-Vietnam-3-0_20260804_065938.jpg</t>
+        </is>
+      </c>
+      <c r="I1356" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>Enam Jam Pemeriksaan Eks Jampidsus Febrie Adriansyah</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:25:19 +0700</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1357" t="inlineStr">
+        <is>
+          <t>Kuasa hukum menyebut Febrie Adriansyah kooperatif saat diperiksa dan akan menghadirkan saksi meringankan.</t>
+        </is>
+      </c>
+      <c r="F1357" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1357" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264718/enam-jam-pemeriksaan-eks-jampidsus-febrie-adriansyah</t>
+        </is>
+      </c>
+      <c r="H1357" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/2WEvQ2hmLFTijz9iyBipOx1Njqg=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318624/original/089072000_1786113401-IMG_3067.jpg</t>
+        </is>
+      </c>
+      <c r="I1357" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>Penampakan Febrie Adriansyah Usai Diperiksa Tim 9 Kejagung</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:11:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1358" t="inlineStr">
+        <is>
+          <t>Febrie meninggalkan ruang pemeriksaan sekitar pukul 20.30 WIB. Ia langsung menuju mobil tahanan.</t>
+        </is>
+      </c>
+      <c r="F1358" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1358" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264672/penampakan-febrie-adriansyah-usai-diperiksa-tim-9-kejagung</t>
+        </is>
+      </c>
+      <c r="H1358" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/sp4SqvNV_83npEChYsHfHfViHdc=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318625/original/014147200_1786113402-IMG_3066.jpg</t>
+        </is>
+      </c>
+      <c r="I1358" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>Warga Dengar 2 Ledakan Saat Kebakaran Gedung Bapenda Jakarta, Sempat Dikira dari SPBU</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:44:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1359" t="inlineStr">
+        <is>
+          <t>Warga sempat mendengar dua ledakan saat Gedung Bapenda kebakaran pada Jumat (7/8/2026) malam.</t>
+        </is>
+      </c>
+      <c r="F1359" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1359" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/07/23404371/warga-dengar-2-ledakan-saat-kebakaran-gedung-bapenda-jakarta-sempat</t>
+        </is>
+      </c>
+      <c r="H1359" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/Xam7pd5ZbVyKKyx4Een4EDcC8v4=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/07/6a7608c1eab96.jpg</t>
+        </is>
+      </c>
+      <c r="I1359" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>Hype</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>Film Baby Udon: Sinopsis, Daftar Pemain, dan Jadwal Tayang</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:44:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1360" t="inlineStr">
+        <is>
+          <t>Film Baby Udon, kisah nyata selebgram Fanny Kondoh dan mendiang suaminya Hajime, segera tayang. Mengangkat perjuangan IVF dan keteguhan hati Fanny.</t>
+        </is>
+      </c>
+      <c r="F1360" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1360" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/hype/read/2026/08/07/225112166/film-baby-udon-sinopsis-daftar-pemain-dan-jadwal-tayang</t>
+        </is>
+      </c>
+      <c r="H1360" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/SR2u2g8xxO6xNGB-48QQaa9Rqeo=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c8191ee571.png,0,-0,1)/data/photo/2026/01/22/6971a80934093.jpg</t>
+        </is>
+      </c>
+      <c r="I1360" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>Permintaan Maaf Rizky Ridho kepada Suporter Usai Timnas Indonesia Gagal Lolos dari Fase Grup Piala AFF</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:44:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1361" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia harus memupus mimpi untuk menyudahi dahaga gelar juara di Piala AFF.</t>
+        </is>
+      </c>
+      <c r="F1361" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1361" t="inlineStr">
+        <is>
+          <t>https://bola.kompas.com/read/2026/08/07/22212338/permintaan-maaf-rizky-ridho-kepada-suporter-usai-timnas-indonesia-gagal-lolos</t>
+        </is>
+      </c>
+      <c r="H1361" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/TEBkzl24l2b4Mn3aThNjri6hlKU=/500x334:4500x3000/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/07/27/6a678dab0ec5a.jpg</t>
+        </is>
+      </c>
+      <c r="I1361" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1295"/>
+  <autoFilter ref="A1:I1361"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 17:48 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-07.xlsx
+++ b/data/berita_2026-08-07.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1361</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1373</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1361"/>
+  <dimension ref="A1:I1373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -64400,8 +64400,572 @@
         </is>
       </c>
     </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>Api Masih Berkobar di Gedung Bapenda DKI, Asap Hitam Membubung</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:56:19 +0700</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E1362" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Jakarta di kawasan Gambir, Jakarta Pusat kebakaran. Hingga tengah malam ini api masih berkobar.</t>
+        </is>
+      </c>
+      <c r="F1362" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1362" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609350/api-masih-berkobar-di-gedung-bapenda-dki-asap-hitam-membubung</t>
+        </is>
+      </c>
+      <c r="H1362" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/kebakaran-gedung-bapenda-dki-jakarta-rolandodetikcom-1786121738496_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1362" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>Daniel Johan Raih detiktimur Awards 2026 'Legislator Benteng Nelayan dan Petani'</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:41:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>Andi Sitti Nurfaisah</t>
+        </is>
+      </c>
+      <c r="E1363" t="inlineStr">
+        <is>
+          <t>Anggota DPR Daniel Johan meraih detiktimur Awards 2026 sebagai Legislator Benteng Nelayan dan Petani atas dedikasinya dalam memperjuangkan kesejahteraan petani.</t>
+        </is>
+      </c>
+      <c r="F1363" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1363" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609342/daniel-johan-raih-detiktimur-awards-2026-legislator-benteng-nelayan-dan-petani</t>
+        </is>
+      </c>
+      <c r="H1363" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/12/22/ketua-dpp-pkb-daniel-johan-tangkapan-layar_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1363" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>Kecelakaan Maut di Lampu Merah, Mobil Polisi Bone Diklaim Rem Blong</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:45:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1364" t="inlineStr">
+        <is>
+          <t>Kecelakaan tragis di Bone, mobil Ipda MA menabrak motor dan menewaskan balita usai menerobos lampu merah. Dari pemeriksaan Satlantas disebut rem mobil blong.</t>
+        </is>
+      </c>
+      <c r="F1364" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1364" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807160623-12-1389802/kecelakaan-maut-di-lampu-merah-mobil-polisi-bone-diklaim-rem-blong</t>
+        </is>
+      </c>
+      <c r="H1364" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2019/09/14/5cf965a3-c769-46ef-a4b8-ca0c095cfd58_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1364" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Kebakaran, 100 Personel Damkar Dikerahkan</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:45:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1365" t="inlineStr">
+        <is>
+          <t>Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta mengalami kebakaran pada Jumat (7/8) malam. Dikutip dari Detik, sebanyak 100 personel Damkar dikerahkan.</t>
+        </is>
+      </c>
+      <c r="F1365" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1365" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807233808-20-1389985/gedung-bapenda-dki-kebakaran-100-personel-damkar-dikerahkan</t>
+        </is>
+      </c>
+      <c r="H1365" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/03/30/ilustrasi-ledakan-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1365" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>Ada 995 Senjata di Sekolah, DPR Curiga Jaringan Manfaatkan Pendidikan</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:40:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1366" t="inlineStr">
+        <is>
+          <t>Anggota DPR Soedeson Tandra mendesak polisi usut tuntas temuan 995 senjata dan narkoba di sekolah swasta. Ia khawatir ada jaringan kejahatan di baliknya.</t>
+        </is>
+      </c>
+      <c r="F1366" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1366" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807160119-12-1389800/ada-995-senjata-di-sekolah-dpr-curiga-jaringan-manfaatkan-pendidikan</t>
+        </is>
+      </c>
+      <c r="H1366" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/995-senjata-yang-ditemukan-di-ruang-mantan-ketua-yayasan-sekolah-jaksel-1786011308187_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1366" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>Pria Berkostum Grim Reaper Manjat Atap RS Bikin Panik Pasien</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:00:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1367" t="inlineStr">
+        <is>
+          <t>Seorang pria dari Deganwy, Wales, ditangkap dan didenda usai membuat panik pasien rumah sakit karena mengenakan kostum Grim Reaper atau malaikat maut.</t>
+        </is>
+      </c>
+      <c r="F1367" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1367" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260806193238-134-1389472/pria-berkostum-grim-reaper-manjat-atap-rs-bikin-panik-pasien</t>
+        </is>
+      </c>
+      <c r="H1367" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/germany-economy-industry-automobile-layoffs-unions-protest-1786020097027_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1367" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>Mau Dicaplok Trump, Belgia Ikut Kirim Pasukan ke Greenland</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:05:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1368" t="inlineStr">
+        <is>
+          <t>Belgia ikut mengirim pasukan mereka ke Pulau Greenland sebagai bagian dari misi Pakta Pertahanan Atlantik Utara (NATO).</t>
+        </is>
+      </c>
+      <c r="F1368" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1368" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260807200752-134-1389937/mau-dicaplok-trump-belgia-ikut-kirim-pasukan-ke-greenland</t>
+        </is>
+      </c>
+      <c r="H1368" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/01/20/trump-kirim-pesawat-militer-ke-greenland-tentara-denmark-siaga-invasi-1768879805860_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1368" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>Tak Lagi Sekadar Busana, Kebaya Kini Bisa Jadi Pesan Pelestarian Alam dan Budaya</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:59:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1369" t="inlineStr">
+        <is>
+          <t>Kebaya Adhikari hadir di IFW 2026, memadukan identitas budaya, Bundengan, dan konservasi gajah dalam narasi pelestarian.</t>
+        </is>
+      </c>
+      <c r="F1369" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1369" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865546/tak-lagi-sekadar-busana-kebaya-kini-bisa-jadi-pesan-pelestarian-alam-dan-budaya</t>
+        </is>
+      </c>
+      <c r="H1369" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/fVPdaKLg4RsCBRsIJP77MhxGv3k=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Tren-kebaya-tak-hanya-sekedar-busana.jpg</t>
+        </is>
+      </c>
+      <c r="I1369" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>Bukan Cuma Lari, Pancasakti Run 2026 Suntik Rp18 Miliar ke Ekonomi Banten</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:52:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1370" t="inlineStr">
+        <is>
+          <t>Perhelatan olahraga berbasis sport tourism makin terbukti ampuh menggerakkan roda ekonomi daerah.</t>
+        </is>
+      </c>
+      <c r="F1370" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1370" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865545/bukan-cuma-lari-pancasakti-run-2026-suntik-rp18-miliar-ke-ekonomi-banten</t>
+        </is>
+      </c>
+      <c r="H1370" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/v3Dn2RmgA5zl6T6FhI0HV_ZARMU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Mantan-Gubernur-DKI-Basuki-Tjahaja-Purnama-alias-Ahok.jpg</t>
+        </is>
+      </c>
+      <c r="I1370" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>Klarifikasi Kepala BGN soal Ucapan Makan Telur Bikin Bisulan: Memang Saya Sengaja</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:50:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1371" t="inlineStr">
+        <is>
+          <t>Kepala BGN Sudaryono ungkap alasan di balik ucapan telur bikin bisul yang menuai kritik dan sebut sengaja memancing edukasi gizi.</t>
+        </is>
+      </c>
+      <c r="F1371" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1371" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865544/klarifikasi-kepala-bgn-soal-ucapan-makan-telur-bikin-bisulan-memang-saya-sengaja</t>
+        </is>
+      </c>
+      <c r="H1371" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/fupn177hoCNSBh0082fDnbmrJfs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sudaryono-MBG-Kepala-BGN.jpg</t>
+        </is>
+      </c>
+      <c r="I1371" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Terbakar, Api Diduga Berasal dari Lantai 11</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:48:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1372" t="inlineStr">
+        <is>
+          <t>Informasi yang diterima Tribun api pertama kali muncul dari lantai 11 gedung Bapenda DKI Jakarta.</t>
+        </is>
+      </c>
+      <c r="F1372" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1372" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865543/gedung-bapenda-dki-terbakar-api-diduga-berasal-dari-lantai-11</t>
+        </is>
+      </c>
+      <c r="H1372" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RHt7QpX6GbddeeJDO8EDZujKiDY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kebakaran-gedung-bapenda-dki-jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I1372" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>Dua Dekade Dinamika BLBI, Verifikasi Data Objektif Dinilai Jadi Kunci Optimalisasi Aset</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:35:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1373" t="inlineStr">
+        <is>
+          <t>Kasus BLBI yang bergulir lebih dari dua dekade tetap menjadi sorotan karena menyangkut pemulihan aset keuangan negara.</t>
+        </is>
+      </c>
+      <c r="F1373" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1373" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865542/dua-dekade-dinamika-blbi-verifikasi-data-objektif-dinilai-jadi-kunci-optimalisasi-aset</t>
+        </is>
+      </c>
+      <c r="H1373" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1iVKAATZm8TQbSOeeRvmwqrYkvU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Menteri-Purbaya-bahas-perekonomian-RI-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I1373" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1361"/>
+  <autoFilter ref="A1:I1373"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 18:45 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-07.xlsx
+++ b/data/berita_2026-08-07.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1373</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1395</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1373"/>
+  <dimension ref="A1:I1395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -64964,8 +64964,1042 @@
         </is>
       </c>
     </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>Aceh tunggu pasokan semen dari Jawa-Sumbar rekonstruksi pascabencana</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:57:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>Redaksi Antara</t>
+        </is>
+      </c>
+      <c r="E1374" t="inlineStr">
+        <is>
+          <t>ANTARA - Meningkatnya kebutuhan material untuk pembangunan rehabilitasi dan rekonstruksi pascabencana, memicu ...</t>
+        </is>
+      </c>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1374" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685192/aceh-tunggu-pasokan-semen-dari-jawa-sumbar-rekonstruksi-pascabencana</t>
+        </is>
+      </c>
+      <c r="H1374" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-07-233819_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1374" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>Trump perketat aturan kewarganegaraan berdasarkan tempat kelahiran</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:53:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>Redaksi Antara</t>
+        </is>
+      </c>
+      <c r="E1375" t="inlineStr">
+        <is>
+          <t>Presiden AS Donald Trump, Kamis (6/8), menandatangani dua perintah eksekutif yang bertujuan untuk semakin membatasi ...</t>
+        </is>
+      </c>
+      <c r="F1375" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1375" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685204/trump-perketat-aturan-kewarganegaraan-berdasarkan-tempat-kelahiran</t>
+        </is>
+      </c>
+      <c r="H1375" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/thumbs_b_c_7585b7a40076b45ff76a5da72d4e66da.jpg</t>
+        </is>
+      </c>
+      <c r="I1375" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>Jepang tetapkan pedoman hak suara, targetkan penggunaan AI tanpa izin</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:50:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>Redaksi Antara</t>
+        </is>
+      </c>
+      <c r="E1376" t="inlineStr">
+        <is>
+          <t>Suara para selebriti dan pengisi suara Jepang harus dilindungi di bawah hak publisitas yang diperluas karena merupakan ...</t>
+        </is>
+      </c>
+      <c r="F1376" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1376" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685203/jepang-tetapkan-pedoman-hak-suara-targetkan-penggunaan-ai-tanpa-izin</t>
+        </is>
+      </c>
+      <c r="H1376" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/01/JepangBenderaAnadolu_as.jpg</t>
+        </is>
+      </c>
+      <c r="I1376" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>Ombudsman perkuat pengawasan tiga program prioritas nasional</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:49:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>Redaksi Antara</t>
+        </is>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>Ombudsman RI memperkuat pengawasan terhadap tiga program prioritas nasional, yakni Makan Bergizi Gratis (MBG), Sekolah ...</t>
+        </is>
+      </c>
+      <c r="F1377" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1377" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685199/ombudsman-perkuat-pengawasan-tiga-program-prioritas-nasional</t>
+        </is>
+      </c>
+      <c r="H1377" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000475325.jpg</t>
+        </is>
+      </c>
+      <c r="I1377" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>Tim Pengawalan Streamlining BUMN perkuat regulasi transformasi BUMN</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:48:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>Redaksi Antara</t>
+        </is>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>Tim Pengawalan Streamlining BUMN yang terdiri atas BP BUMN, Danantara, Kementerian Hukum, dan Kejaksaan RI terus ...</t>
+        </is>
+      </c>
+      <c r="F1378" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1378" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685196/tim-pengawalan-streamlining-bumn-perkuat-regulasi-transformasi-bumn</t>
+        </is>
+      </c>
+      <c r="H1378" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/WhatsApp-Image-2026-08-07-at-10.05.33.jpeg</t>
+        </is>
+      </c>
+      <c r="I1378" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>BP BUMN catat 274 BUMN telah ditata dalam rangka transformasi</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:44:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>Redaksi Antara</t>
+        </is>
+      </c>
+      <c r="E1379" t="inlineStr">
+        <is>
+          <t>Kepala Badan Pengaturan Badan Usaha Milik Negara (BP BUMN) Dony Oskaria mencatat sebanyak 274 perusahaan pelat ...</t>
+        </is>
+      </c>
+      <c r="F1379" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1379" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685188/bp-bumn-catat-274-bumn-telah-ditata-dalam-rangka-transformasi</t>
+        </is>
+      </c>
+      <c r="H1379" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/IMG_3638.jpeg</t>
+        </is>
+      </c>
+      <c r="I1379" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>Eks penyidik KPK: Kasus eks Jampidsus perlu terus diawasi publik</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:44:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>Redaksi Antara</t>
+        </is>
+      </c>
+      <c r="E1380" t="inlineStr">
+        <is>
+          <t>Mantan penyidik Komisi Pemberantasan Korupsi (KPK) Yudi Purnomo Harahap menilai penanganan kasus dugaan tindak pidana ...</t>
+        </is>
+      </c>
+      <c r="F1380" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1380" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685184/eks-penyidik-kpk-kasus-eks-jampidsus-perlu-terus-diawasi-publik</t>
+        </is>
+      </c>
+      <c r="H1380" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/08/16/IMG-20191206-WA0012_1610529146924.jpg</t>
+        </is>
+      </c>
+      <c r="I1380" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>Klasemen Grup A Piala AFF 2026: Vietnam dan Singapura ke semifinal</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 23:42:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>Redaksi Antara</t>
+        </is>
+      </c>
+      <c r="E1381" t="inlineStr">
+        <is>
+          <t>Timnas Vietnam dan Timnas Singapura melaju ke semifinal Piala AFF 2026 setelah menempati peringkat kedua teratas ...</t>
+        </is>
+      </c>
+      <c r="F1381" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1381" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685181/klasemen-grup-a-piala-aff-2026-vietnam-dan-singapura-ke-semifinal</t>
+        </is>
+      </c>
+      <c r="H1381" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/aff.jpg</t>
+        </is>
+      </c>
+      <c r="I1381" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>Freeport Pastikan Smelter Manyar Gresik Produksi Lagi Mulai September</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:30:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>PT Freeport Indonesia (PTFI) memastikan smelter Manyar di JIIPE, Gresik, Jawa Timur, mulai memproduksi katoda tembaga pada September 2026.</t>
+        </is>
+      </c>
+      <c r="F1382" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1382" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807204055-85-1389951/freeport-pastikan-smelter-manyar-gresik-produksi-lagi-mulai-september</t>
+        </is>
+      </c>
+      <c r="H1382" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/29/tony-wenas-presiden-direktur-pt-freeport-indonesia-1785306971048_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1382" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>Pertamina Perkuat SDM Local Hero, Bangun Kemandirian Energi Desa</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:01:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>Melalui Program Desa Energi Berdikari, Pertamina membina para local hero melalui edukasi, pelatihan, hingga sertifikasi kompetensi.</t>
+        </is>
+      </c>
+      <c r="F1383" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1383" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807205732-625-1389962/pertamina-perkuat-sdm-local-hero-bangun-kemandirian-energi-desa</t>
+        </is>
+      </c>
+      <c r="H1383" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/pertamina-1786111216109_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1383" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>ASDP Terapkan Standar Baru Keselamatan Nasional di 6 Pelabuhan Utama</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 20:30:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1384" t="inlineStr">
+        <is>
+          <t>PT ASDP Indonesia Ferry (Persero) resmi menerapkan program sterilisasi pelabuhan secara penuh di enam pelabuhan utama mulai Rabu (5/8).</t>
+        </is>
+      </c>
+      <c r="F1384" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1384" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807135157-92-1389713/asdp-terapkan-standar-baru-keselamatan-nasional-di-6-pelabuhan-utama</t>
+        </is>
+      </c>
+      <c r="H1384" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/asdp-resmi-terapkan-standar-baru-keselamatan-nasional-di-6-pelabuhan-utama-1786074467002_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1384" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>BGN Bakal Pasang CCTV yang Terhubung ke Kantor Pusat Buat Awasi SPPG</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 20:23:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>BGN tengah menyiapkan sistem pengawasan baru berupa CCTV terintegrasi di seluruh SPPG. CCTV tersebut akan terhubung langsung ke kantor pusat.</t>
+        </is>
+      </c>
+      <c r="F1385" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1385" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807195839-92-1389933/bgn-bakal-pasang-cctv-yang-terhubung-ke-kantor-pusat-buat-awasi-sppg</t>
+        </is>
+      </c>
+      <c r="H1385" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/05/20/pemerintah-pangkas-anggaran-mbg-1779256675949_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1385" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>Bank Mandiri Konsisten Perluas Manfaat Lewat Program Sosial Lingkungan</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 20:21:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>Implementasi tanggung jawab sosial itu diwujudkan lewat tiga pilar utama, yakni Sustainable Banking, Sustainable Operation, dan Sustainability Beyond Banking.</t>
+        </is>
+      </c>
+      <c r="F1386" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1386" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807200857-625-1389938/bank-mandiri-konsisten-perluas-manfaat-lewat-program-sosial-lingkungan</t>
+        </is>
+      </c>
+      <c r="H1386" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/09/30/bank-mandiri-1759222272580_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1386" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>Semangat Koperasi Berhembus di Festival Lembah Baliem</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 20:01:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>Festival Budaya Lembah Baliem yang mempromosikan produk unggulan seperti kopi dan budaya ini dinilai Menkop sebagai momentum membangun kekuatan ekonomi lokal.</t>
+        </is>
+      </c>
+      <c r="F1387" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1387" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807181301-97-1389932/semangat-koperasi-berhembus-di-festival-lembah-baliem</t>
+        </is>
+      </c>
+      <c r="H1387" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/kemenkop-1786107655627_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1387" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>Digitalisasi Jadi Motor Dongkrak Produktivitas Bank Mandiri</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:59:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>Bank Mandiri terus tingkatkan kapabilitas digital, memperluas layanan dan efisiensi. Aplikasi Livin' dan Kopra tumbuh pesat, mendukung inklusi ekonomi.</t>
+        </is>
+      </c>
+      <c r="F1388" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1388" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807194135-625-1389925/digitalisasi-jadi-motor-dongkrak-produktivitas-bank-mandiri</t>
+        </is>
+      </c>
+      <c r="H1388" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/06/23/livin-bank-mandiri-5_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1388" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>BGN Bakal Pasang Label Batas Konsumsi Maksimal 4 Jam di Ompreng MBG</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:47:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>BGN akan memperketat standar operasional prosedur (SOP) program MBG dengan mewajibkan makanan dikonsumsi maksimal empat jam setelah selesai dimasak.</t>
+        </is>
+      </c>
+      <c r="F1389" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1389" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807193427-92-1389921/bgn-bakal-pasang-label-batas-konsumsi-maksimal-4-jam-di-ompreng-mbg</t>
+        </is>
+      </c>
+      <c r="H1389" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/05/20/pemerintah-pangkas-anggaran-mbg-1779256686908_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1389" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>Swasembada Beras, Fondasi Pemerintah Jaga Kedaulatan Pangan Nasional</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:38:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1390" t="inlineStr">
+        <is>
+          <t>Momentum Hari Kemerdekaan RI menekankan pentingnya swasembada beras. Kementan targetkan 2025, dengan stok beras mencapai 26 juta ton untuk stabilitas pangan.</t>
+        </is>
+      </c>
+      <c r="F1390" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1390" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807193251-97-1389920/swasembada-beras-fondasi-pemerintah-jaga-kedaulatan-pangan-nasional</t>
+        </is>
+      </c>
+      <c r="H1390" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/02/17/bulog-guyur-beras-ke-pasar-induk-cipinang-8_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1390" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>Bos BGN Pecat 66 Kepala SPPG, Ada yang Terlibat Judol hingga Minta Fee</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:25:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1391" t="inlineStr">
+        <is>
+          <t>Kepala BGN Sudaryono menyebut 66 kepala SPPG dipecat karena berbagai pelanggaran, mulai dari indisipliner, judi online, hingga diduga meminta fee kepada mitra.</t>
+        </is>
+      </c>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1391" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807191247-92-1389912/bos-bgn-pecat-66-kepala-sppg-ada-yang-terlibat-judol-hingga-minta-fee</t>
+        </is>
+      </c>
+      <c r="H1391" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/05/bos-bgn-ultimatum-dapur-mbg-1785936867455_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1391" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>BGN Mulai Coret Sekolah Swasta Elite dari Daftar Penerima MBG</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:12:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1392" t="inlineStr">
+        <is>
+          <t>Sudaryono menegaskan tak akan memaksakan pemberian MBG kepada sekolah yang menyatakan tidak membutuhkan program tersebut.</t>
+        </is>
+      </c>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1392" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807190126-92-1389897/bgn-mulai-coret-sekolah-swasta-elite-dari-daftar-penerima-mbg</t>
+        </is>
+      </c>
+      <c r="H1392" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/29/bgn-tutup-833-dapur-sppg-bermasalah-1785317578338_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1392" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>Bos BGN: Guru Tak Seharusnya Urus Ompreng MBG</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:58:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>Kepala BGN Sudaryono merespons keluhan sejumlah guru yang mengaku terbebani pelaksanaan MBG, termasuk mengurus ompreng.</t>
+        </is>
+      </c>
+      <c r="F1393" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1393" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807184759-92-1389881/bos-bgn-guru-tak-seharusnya-urus-ompreng-mbg</t>
+        </is>
+      </c>
+      <c r="H1393" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/29/bgn-tutup-833-dapur-sppg-bermasalah-1785317578257_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1393" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>Bahlil Kenang Didemo 1,5 Bulan Gara-gara Larangan Ekspor Bijih Nikel</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 18:43:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1394" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1394" t="inlineStr">
+        <is>
+          <t>Bahlil membagikan kisah menghadapi gelombang demo selama 1,5 bulan terkait kebijakan larangan ekspor bijih nikel. Saat itu, ia baru 4 hari menjabat Kepala BKPM.</t>
+        </is>
+      </c>
+      <c r="F1394" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1394" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807181838-85-1389861/bahlil-kenang-didemo-15-bulan-gara-gara-larangan-ekspor-bijih-nikel</t>
+        </is>
+      </c>
+      <c r="H1394" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/peluncuran-sepuluh-buku-karya-nyata-untuk-negeri-bahlil-lahadalia-1786099773487_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1394" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>Prabowo Mau Perbaiki Buku SD-SMA, Malaysia-Kamboja Jadi Pembanding</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 19:54:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1395" t="inlineStr">
+        <is>
+          <t>Pemerintah tengah menggelar program perbaikan kualitas buku pelajaran di sekolah SD-SMA.</t>
+        </is>
+      </c>
+      <c r="F1395" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1395" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260807194220-17-757542/prabowo-mau-perbaiki-buku-sd-sma-malaysia-kamboja-jadi-pembanding</t>
+        </is>
+      </c>
+      <c r="H1395" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/menteri-sekertaris-negera-dan-sekertaris-kabinet-di-depan-buku-buku-pelajaran-sd-sma-negara-negara-tetangga-ri-jumat-782026-1786106683018_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1395" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1373"/>
+  <autoFilter ref="A1:I1395"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 19:48 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-07.xlsx
+++ b/data/berita_2026-08-07.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1395</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1401</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1395"/>
+  <dimension ref="A1:I1401"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -65998,8 +65998,290 @@
         </is>
       </c>
     </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>Presiden Ini Mendadak Dievakuasi Tengah Malam, Ada Apa?</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 22:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>tfa</t>
+        </is>
+      </c>
+      <c r="E1396" t="inlineStr">
+        <is>
+          <t>Presiden Taiwan Lai Ching-te mendadak dievakuasi menggunakan kendaraan pengangkut personel lapis baja menuju pusat komando pada Rabu malam lalu.</t>
+        </is>
+      </c>
+      <c r="F1396" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1396" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807171848-4-757520/presiden-ini-mendadak-dievakuasi-tengah-malam-ada-apa</t>
+        </is>
+      </c>
+      <c r="H1396" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/10/25/tentara-berdiri-selama-latihan-militer-di-pulau-penghu-taiwan-kamis-24-oktober-2024_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1396" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>Korut "Terpanggang", Kim Jong Un Dorong Warga Makan Daging Anjing</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>tps</t>
+        </is>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>Korea Utara menghadapi gelombang panas ekstrem, media pemerintah mendorong konsumsi sup daging anjing dan kaldu ayam.</t>
+        </is>
+      </c>
+      <c r="F1397" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1397" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807152252-4-757464/korut-terpanggang-kim-jong-un-dorong-warga-makan-daging-anjing</t>
+        </is>
+      </c>
+      <c r="H1397" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/08/10/pemimpin-korea-utara-kim-jong-un-menyapa-anak-anak-saat-berkunjung-ke-daerah-yang-terkena-banjir-di-kabupaten-uiju-provinsi-py_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1397" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>Stres Belajar, Kronologi Siswa 14 Tahun Tembak Sekolah dan Bunuh Guru</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>Seorang siswa 14 tahun melakukan penembakan di Sekolah Debsirin Nonthaburi, Thailand, menewaskan delapan orang.</t>
+        </is>
+      </c>
+      <c r="F1398" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1398" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807171445-4-757518/stres-belajar-kronologi-siswa-14-tahun-tembak-sekolah-bunuh-guru</t>
+        </is>
+      </c>
+      <c r="H1398" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/petugas-penyelamat-berdiri-di-dekat-ambulans-di-sekolah-debsirin-nonthaburilokasi-terjadinya-insiden-penembakandi-distrik-bang-1786084015199_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1398" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>"Neraka Luber-Luber" di Eropa, Sungai Menghilang-Suhu Panas Mendidih</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>Eropa menghadapi gelombang panas ekstrem dengan suhu melebihi 40°C. Kebakaran hutan melanda, dan negara-negara mengambil langkah</t>
+        </is>
+      </c>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1399" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807081855-4-757300/neraka-luber-luber-di-eropa-sungai-menghilang-suhu-panas-mendidih</t>
+        </is>
+      </c>
+      <c r="H1399" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/tampilan-dari-drone-memperlihatkan-gosong-pasir-yang-muncul-di-permukaan-sungai-vistula-dekat-jozefowdi-pinggiran-warsawa-pola-1785897303805_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1399" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>Pertamina Bangun Kemandirian Energi Desa Lewat Local Hero</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:17:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1400" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1400" t="inlineStr">
+        <is>
+          <t>PPertamina mengubah kehidupan masyarakat dengan menyediakan akses air bersih dan energi terbarukan, meningkatkan kemandirian dan kesejahteraan desa.</t>
+        </is>
+      </c>
+      <c r="F1400" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1400" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807211326-4-757548/pertamina-bangun-kemandirian-energi-desa-lewat-local-hero</t>
+        </is>
+      </c>
+      <c r="H1400" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/pertamina-1786112206041_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1400" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>Danantara dan JBS Group Kerja Sama Kembangkan Ekosistem Protein</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>Fri, 07 Aug 2026 21:11:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>Danantara Indonesia menjalin kemitraan strategis dengan JBS Group senilai USD 2,5 miliar untuk pengelolaan operasi di Australia dan Selandia Baru.</t>
+        </is>
+      </c>
+      <c r="F1401" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1401" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807210838-4-757547/danantara-jbs-group-kerja-sama-kembangkan-ekosistem-protein</t>
+        </is>
+      </c>
+      <c r="H1401" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/03/05/kantor-danantara-pusat-di-jakarta-indonesia-28-februari-2025-1741144820212_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1401" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1395"/>
+  <autoFilter ref="A1:I1401"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>